<commit_message>
Cambio modelo en SPA y actualizo pred
</commit_message>
<xml_diff>
--- a/data/historial_predicciones.xlsx
+++ b/data/historial_predicciones.xlsx
@@ -62253,43 +62253,43 @@
         <v>0.05958670893507123</v>
       </c>
       <c r="N620" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O620" t="n">
-        <v>0.7184902928921869</v>
+        <v>0.4380788505077362</v>
       </c>
       <c r="P620" t="n">
-        <v>0.2034047392590317</v>
+        <v>0.487432450056076</v>
       </c>
       <c r="Q620" t="n">
-        <v>0.07810496784878133</v>
+        <v>0.07448867708444595</v>
       </c>
       <c r="R620" t="n">
         <v>1</v>
       </c>
       <c r="S620" t="n">
-        <v>0.1533620309386161</v>
+        <v>0.2098547449200575</v>
       </c>
       <c r="T620" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U620" t="n">
-        <v>0.1533620309386161</v>
+        <v>0.2098547449200575</v>
       </c>
       <c r="V620" t="n">
-        <v>0.7184902928921869</v>
+        <v>0.487432450056076</v>
       </c>
       <c r="W620" t="n">
-        <v>1.67</v>
+        <v>3.4</v>
       </c>
       <c r="X620" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.5</t>
+          <t>dif_prob_mod_bm &gt; -0.25</t>
         </is>
       </c>
       <c r="Y620" t="inlineStr"/>
       <c r="Z620" t="n">
-        <v>12.57358012561327</v>
+        <v>8.530067875981331</v>
       </c>
       <c r="AA620" t="inlineStr">
         <is>
@@ -62355,40 +62355,40 @@
         <v>0</v>
       </c>
       <c r="O621" t="n">
-        <v>0.06510227056649795</v>
+        <v>0.3059642314910889</v>
       </c>
       <c r="P621" t="n">
-        <v>0.5041676322345764</v>
+        <v>0.4625942409038544</v>
       </c>
       <c r="Q621" t="n">
-        <v>0.4307300971989256</v>
+        <v>0.2314416021108627</v>
       </c>
       <c r="R621" t="n">
         <v>1</v>
       </c>
       <c r="S621" t="n">
-        <v>0.1884853511755133</v>
+        <v>0.1469119598447913</v>
       </c>
       <c r="T621" t="n">
         <v>0</v>
       </c>
       <c r="U621" t="n">
-        <v>0.1884853511755133</v>
+        <v>0.1469119598447913</v>
       </c>
       <c r="V621" t="n">
-        <v>0.5041676322345764</v>
+        <v>0.4625942409038544</v>
       </c>
       <c r="W621" t="n">
         <v>3</v>
       </c>
       <c r="X621" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.5</t>
+          <t>dif_prob_mod_bm &gt; -0.25</t>
         </is>
       </c>
       <c r="Y621" t="inlineStr"/>
       <c r="Z621" t="n">
-        <v>8.822933564105087</v>
+        <v>8.095399215817451</v>
       </c>
       <c r="AA621" t="inlineStr">
         <is>
@@ -62456,40 +62456,40 @@
         <v>1</v>
       </c>
       <c r="O622" t="n">
-        <v>0.7619521193300006</v>
+        <v>0.8815600275993347</v>
       </c>
       <c r="P622" t="n">
-        <v>0.1918999227194019</v>
+        <v>0.09728441387414932</v>
       </c>
       <c r="Q622" t="n">
-        <v>0.04614795795059752</v>
+        <v>0.02115556225180626</v>
       </c>
       <c r="R622" t="n">
         <v>1</v>
       </c>
       <c r="S622" t="n">
-        <v>0.08122601148162889</v>
+        <v>0.200833919750963</v>
       </c>
       <c r="T622" t="n">
         <v>1</v>
       </c>
       <c r="U622" t="n">
-        <v>0.08122601148162889</v>
+        <v>0.200833919750963</v>
       </c>
       <c r="V622" t="n">
-        <v>0.7619521193300006</v>
+        <v>0.8815600275993347</v>
       </c>
       <c r="W622" t="n">
         <v>1.38</v>
       </c>
       <c r="X622" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.5</t>
+          <t>dif_prob_mod_bm &gt; -0.25</t>
         </is>
       </c>
       <c r="Y622" t="inlineStr"/>
       <c r="Z622" t="n">
-        <v>13.33416208827501</v>
+        <v>15.42730048298836</v>
       </c>
       <c r="AA622" t="inlineStr">
         <is>
@@ -62555,40 +62555,40 @@
         <v>1</v>
       </c>
       <c r="O623" t="n">
-        <v>0.4651637178206616</v>
+        <v>0.4232662916183472</v>
       </c>
       <c r="P623" t="n">
-        <v>0.3021492415741182</v>
+        <v>0.1972329318523407</v>
       </c>
       <c r="Q623" t="n">
-        <v>0.2326870406052202</v>
+        <v>0.3795007765293121</v>
       </c>
       <c r="R623" t="n">
         <v>1</v>
       </c>
       <c r="S623" t="n">
-        <v>-0.1104213549181113</v>
+        <v>-0.1523187811204257</v>
       </c>
       <c r="T623" t="n">
         <v>1</v>
       </c>
       <c r="U623" t="n">
-        <v>-0.1104213549181113</v>
+        <v>-0.1523187811204257</v>
       </c>
       <c r="V623" t="n">
-        <v>0.4651637178206616</v>
+        <v>0.4232662916183472</v>
       </c>
       <c r="W623" t="n">
         <v>1.65</v>
       </c>
       <c r="X623" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.5</t>
+          <t>dif_prob_mod_bm &gt; -0.25</t>
         </is>
       </c>
       <c r="Y623" t="inlineStr"/>
       <c r="Z623" t="n">
-        <v>0.4108702175937888</v>
+        <v>2.076002764106175</v>
       </c>
       <c r="AA623" t="inlineStr">
         <is>
@@ -62653,43 +62653,43 @@
         <v>0.06277630415561442</v>
       </c>
       <c r="N624" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O624" t="n">
-        <v>0.1317361903191667</v>
+        <v>0.2766321897506714</v>
       </c>
       <c r="P624" t="n">
-        <v>0.3171854353409633</v>
+        <v>0.4907961785793304</v>
       </c>
       <c r="Q624" t="n">
-        <v>0.5510783743398699</v>
+        <v>0.2325715571641922</v>
       </c>
       <c r="R624" t="n">
         <v>1</v>
       </c>
       <c r="S624" t="n">
-        <v>0.1891815357375405</v>
+        <v>0.1663369439703454</v>
       </c>
       <c r="T624" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="U624" t="n">
-        <v>0.1891815357375405</v>
+        <v>0.1663369439703454</v>
       </c>
       <c r="V624" t="n">
-        <v>0.5510783743398699</v>
+        <v>0.4907961785793304</v>
       </c>
       <c r="W624" t="n">
-        <v>2.6</v>
+        <v>2.9</v>
       </c>
       <c r="X624" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.5</t>
+          <t>dif_prob_mod_bm &gt; -0.25</t>
         </is>
       </c>
       <c r="Y624" t="inlineStr"/>
       <c r="Z624" t="n">
-        <v>9.643871550947724</v>
+        <v>8.588933125138283</v>
       </c>
       <c r="AA624" t="inlineStr">
         <is>
@@ -62755,40 +62755,40 @@
         <v>2</v>
       </c>
       <c r="O625" t="n">
-        <v>0.03682417779639348</v>
+        <v>0.04302779212594032</v>
       </c>
       <c r="P625" t="n">
-        <v>0.07686330039214101</v>
+        <v>0.08403868973255157</v>
       </c>
       <c r="Q625" t="n">
-        <v>0.8863125218114655</v>
+        <v>0.8729335069656372</v>
       </c>
       <c r="R625" t="n">
         <v>1</v>
       </c>
       <c r="S625" t="n">
-        <v>0.3380096497488022</v>
+        <v>0.3246306349029739</v>
       </c>
       <c r="T625" t="n">
         <v>2</v>
       </c>
       <c r="U625" t="n">
-        <v>0.3380096497488022</v>
+        <v>0.3246306349029739</v>
       </c>
       <c r="V625" t="n">
-        <v>0.8863125218114655</v>
+        <v>0.8729335069656372</v>
       </c>
       <c r="W625" t="n">
         <v>1.73</v>
       </c>
       <c r="X625" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.5</t>
+          <t>dif_prob_mod_bm &gt; -0.25</t>
         </is>
       </c>
       <c r="Y625" t="inlineStr"/>
       <c r="Z625" t="n">
-        <v>15.51046913170065</v>
+        <v>15.27633637189865</v>
       </c>
       <c r="AA625" t="inlineStr">
         <is>
@@ -62854,40 +62854,40 @@
         <v>2</v>
       </c>
       <c r="O626" t="n">
-        <v>0.08865098957765606</v>
+        <v>0.2263692766427994</v>
       </c>
       <c r="P626" t="n">
-        <v>0.3173732192583593</v>
+        <v>0.2608787417411804</v>
       </c>
       <c r="Q626" t="n">
-        <v>0.5939757911639847</v>
+        <v>0.5127519965171814</v>
       </c>
       <c r="R626" t="n">
         <v>1</v>
       </c>
       <c r="S626" t="n">
-        <v>0.2110537065934923</v>
+        <v>0.129829911946689</v>
       </c>
       <c r="T626" t="n">
         <v>2</v>
       </c>
       <c r="U626" t="n">
-        <v>0.2110537065934923</v>
+        <v>0.129829911946689</v>
       </c>
       <c r="V626" t="n">
-        <v>0.5939757911639847</v>
+        <v>0.5127519965171814</v>
       </c>
       <c r="W626" t="n">
         <v>2.45</v>
       </c>
       <c r="X626" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.5</t>
+          <t>dif_prob_mod_bm &gt; -0.25</t>
         </is>
       </c>
       <c r="Y626" t="inlineStr"/>
       <c r="Z626" t="n">
-        <v>10.39457634536973</v>
+        <v>8.973159939050674</v>
       </c>
       <c r="AA626" t="inlineStr">
         <is>
@@ -62953,40 +62953,40 @@
         <v>0</v>
       </c>
       <c r="O627" t="n">
-        <v>0.3090568887998504</v>
+        <v>0.2207784503698349</v>
       </c>
       <c r="P627" t="n">
-        <v>0.4106878150893326</v>
+        <v>0.5502509474754333</v>
       </c>
       <c r="Q627" t="n">
-        <v>0.280255296110817</v>
+        <v>0.2289706021547318</v>
       </c>
       <c r="R627" t="n">
         <v>1</v>
       </c>
       <c r="S627" t="n">
-        <v>0.09688364173459746</v>
+        <v>0.2364467741206983</v>
       </c>
       <c r="T627" t="n">
         <v>0</v>
       </c>
       <c r="U627" t="n">
-        <v>0.09688364173459746</v>
+        <v>0.2364467741206983</v>
       </c>
       <c r="V627" t="n">
-        <v>0.4106878150893326</v>
+        <v>0.5502509474754333</v>
       </c>
       <c r="W627" t="n">
         <v>3</v>
       </c>
       <c r="X627" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.5</t>
+          <t>dif_prob_mod_bm &gt; -0.25</t>
         </is>
       </c>
       <c r="Y627" t="inlineStr"/>
       <c r="Z627" t="n">
-        <v>7.187036764063319</v>
+        <v>9.629391580820084</v>
       </c>
       <c r="AA627" t="inlineStr">
         <is>
@@ -63054,40 +63054,40 @@
         <v>2</v>
       </c>
       <c r="O628" t="n">
-        <v>0.004314461375559076</v>
+        <v>0.07501446455717087</v>
       </c>
       <c r="P628" t="n">
-        <v>0.01836210622104234</v>
+        <v>0.0668170303106308</v>
       </c>
       <c r="Q628" t="n">
-        <v>0.9773234324033986</v>
+        <v>0.8581684827804565</v>
       </c>
       <c r="R628" t="n">
         <v>1</v>
       </c>
       <c r="S628" t="n">
-        <v>0.3234573192741822</v>
+        <v>0.2043023696512402</v>
       </c>
       <c r="T628" t="n">
         <v>2</v>
       </c>
       <c r="U628" t="n">
-        <v>0.3234573192741822</v>
+        <v>0.2043023696512402</v>
       </c>
       <c r="V628" t="n">
-        <v>0.9773234324033986</v>
+        <v>0.8581684827804565</v>
       </c>
       <c r="W628" t="n">
         <v>1.45</v>
       </c>
       <c r="X628" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.5</t>
+          <t>dif_prob_mod_bm &gt; -0.25</t>
         </is>
       </c>
       <c r="Y628" t="inlineStr"/>
       <c r="Z628" t="n">
-        <v>17.10316006705948</v>
+        <v>15.01794844865799</v>
       </c>
       <c r="AA628" t="inlineStr">
         <is>
@@ -63150,43 +63150,43 @@
         <v>0.06565656565656575</v>
       </c>
       <c r="N629" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O629" t="n">
-        <v>0.4424752725230887</v>
+        <v>0.3437532186508179</v>
       </c>
       <c r="P629" t="n">
-        <v>0.2448774174274614</v>
+        <v>0.1945755779743195</v>
       </c>
       <c r="Q629" t="n">
-        <v>0.31264731004945</v>
+        <v>0.4616712033748627</v>
       </c>
       <c r="R629" t="n">
         <v>1</v>
       </c>
       <c r="S629" t="n">
-        <v>0.01593498816289918</v>
+        <v>0.201007696265858</v>
       </c>
       <c r="T629" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U629" t="n">
-        <v>0.01593498816289918</v>
+        <v>0.201007696265858</v>
       </c>
       <c r="V629" t="n">
-        <v>0.4424752725230887</v>
+        <v>0.4616712033748627</v>
       </c>
       <c r="W629" t="n">
-        <v>2.2</v>
+        <v>3.6</v>
       </c>
       <c r="X629" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.5</t>
+          <t>dif_prob_mod_bm &gt; -0.25</t>
         </is>
       </c>
       <c r="Y629" t="inlineStr"/>
       <c r="Z629" t="n">
-        <v>7.743317269154052</v>
+        <v>8.079246059060097</v>
       </c>
       <c r="AA629" t="inlineStr">
         <is>
@@ -63252,40 +63252,40 @@
         <v>1</v>
       </c>
       <c r="O630" t="n">
-        <v>0.5694948776563049</v>
+        <v>0.5841125249862671</v>
       </c>
       <c r="P630" t="n">
-        <v>0.2014548824272862</v>
+        <v>0.2444181740283966</v>
       </c>
       <c r="Q630" t="n">
-        <v>0.2290502399164089</v>
+        <v>0.1714693456888199</v>
       </c>
       <c r="R630" t="n">
         <v>1</v>
       </c>
       <c r="S630" t="n">
-        <v>0.07528075624943209</v>
+        <v>0.08989840357939427</v>
       </c>
       <c r="T630" t="n">
         <v>1</v>
       </c>
       <c r="U630" t="n">
-        <v>0.07528075624943209</v>
+        <v>0.08989840357939427</v>
       </c>
       <c r="V630" t="n">
-        <v>0.5694948776563049</v>
+        <v>0.5841125249862671</v>
       </c>
       <c r="W630" t="n">
         <v>1.9</v>
       </c>
       <c r="X630" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.5</t>
+          <t>dif_prob_mod_bm &gt; -0.25</t>
         </is>
       </c>
       <c r="Y630" t="inlineStr"/>
       <c r="Z630" t="n">
-        <v>9.966160358985336</v>
+        <v>10.22196918725967</v>
       </c>
       <c r="AA630" t="inlineStr">
         <is>
@@ -63351,40 +63351,40 @@
         <v>1</v>
       </c>
       <c r="O631" t="n">
-        <v>0.951221279460578</v>
+        <v>0.6555708050727844</v>
       </c>
       <c r="P631" t="n">
-        <v>0.04302405013321797</v>
+        <v>0.2326910942792892</v>
       </c>
       <c r="Q631" t="n">
-        <v>0.005754670406204023</v>
+        <v>0.1117381155490875</v>
       </c>
       <c r="R631" t="n">
         <v>1</v>
       </c>
       <c r="S631" t="n">
-        <v>0.2029959165393015</v>
+        <v>-0.09265455784849208</v>
       </c>
       <c r="T631" t="n">
         <v>1</v>
       </c>
       <c r="U631" t="n">
-        <v>0.2029959165393015</v>
+        <v>-0.09265455784849208</v>
       </c>
       <c r="V631" t="n">
-        <v>0.951221279460578</v>
+        <v>0.6555708050727844</v>
       </c>
       <c r="W631" t="n">
         <v>1.27</v>
       </c>
       <c r="X631" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.5</t>
+          <t>dif_prob_mod_bm &gt; -0.25</t>
         </is>
       </c>
       <c r="Y631" t="inlineStr"/>
       <c r="Z631" t="n">
-        <v>16.64637239056011</v>
+        <v>8.229579564076504</v>
       </c>
       <c r="AA631" t="inlineStr">
         <is>
@@ -63450,40 +63450,40 @@
         <v>1</v>
       </c>
       <c r="O632" t="n">
-        <v>0.4721386647460002</v>
+        <v>0.5136918425559998</v>
       </c>
       <c r="P632" t="n">
-        <v>0.2222211274056271</v>
+        <v>0.2290997058153152</v>
       </c>
       <c r="Q632" t="n">
-        <v>0.3056402078483726</v>
+        <v>0.2572084963321686</v>
       </c>
       <c r="R632" t="n">
         <v>1</v>
       </c>
       <c r="S632" t="n">
-        <v>-0.03843755698995899</v>
+        <v>0.003115620820040577</v>
       </c>
       <c r="T632" t="n">
         <v>1</v>
       </c>
       <c r="U632" t="n">
-        <v>-0.03843755698995899</v>
+        <v>0.003115620820040577</v>
       </c>
       <c r="V632" t="n">
-        <v>0.4721386647460002</v>
+        <v>0.5136918425559998</v>
       </c>
       <c r="W632" t="n">
         <v>1.83</v>
       </c>
       <c r="X632" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.5</t>
+          <t>dif_prob_mod_bm &gt; -0.25</t>
         </is>
       </c>
       <c r="Y632" t="inlineStr"/>
       <c r="Z632" t="n">
-        <v>5.571797643757874</v>
+        <v>8.989607244729996</v>
       </c>
       <c r="AA632" t="inlineStr">
         <is>
@@ -63549,40 +63549,40 @@
         <v>0</v>
       </c>
       <c r="O633" t="n">
-        <v>0.278567760480365</v>
+        <v>0.2504731118679047</v>
       </c>
       <c r="P633" t="n">
-        <v>0.4390872220153065</v>
+        <v>0.4024161696434021</v>
       </c>
       <c r="Q633" t="n">
-        <v>0.2823450175043283</v>
+        <v>0.3471106588840485</v>
       </c>
       <c r="R633" t="n">
         <v>1</v>
       </c>
       <c r="S633" t="n">
-        <v>0.1537198874676441</v>
+        <v>0.1170488350957397</v>
       </c>
       <c r="T633" t="n">
         <v>0</v>
       </c>
       <c r="U633" t="n">
-        <v>0.1537198874676441</v>
+        <v>0.1170488350957397</v>
       </c>
       <c r="V633" t="n">
-        <v>0.4390872220153065</v>
+        <v>0.4024161696434021</v>
       </c>
       <c r="W633" t="n">
         <v>3.3</v>
       </c>
       <c r="X633" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.5</t>
+          <t>dif_prob_mod_bm &gt; -0.25</t>
         </is>
       </c>
       <c r="Y633" t="inlineStr"/>
       <c r="Z633" t="n">
-        <v>7.684026385267864</v>
+        <v>7.042282968759537</v>
       </c>
       <c r="AA633" t="inlineStr">
         <is>
@@ -63650,40 +63650,40 @@
         <v>2</v>
       </c>
       <c r="O634" t="n">
-        <v>0.01731246134187259</v>
+        <v>0.2667881846427917</v>
       </c>
       <c r="P634" t="n">
-        <v>0.2238994226737401</v>
+        <v>0.06890491396188736</v>
       </c>
       <c r="Q634" t="n">
-        <v>0.7587881159843872</v>
+        <v>0.6643068790435791</v>
       </c>
       <c r="R634" t="n">
         <v>1</v>
       </c>
       <c r="S634" t="n">
-        <v>0.2225105134607279</v>
+        <v>0.1280292765199198</v>
       </c>
       <c r="T634" t="n">
         <v>2</v>
       </c>
       <c r="U634" t="n">
-        <v>0.2225105134607279</v>
+        <v>0.1280292765199198</v>
       </c>
       <c r="V634" t="n">
-        <v>0.7587881159843872</v>
+        <v>0.6643068790435791</v>
       </c>
       <c r="W634" t="n">
         <v>1.75</v>
       </c>
       <c r="X634" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.5</t>
+          <t>dif_prob_mod_bm &gt; -0.25</t>
         </is>
       </c>
       <c r="Y634" t="inlineStr"/>
       <c r="Z634" t="n">
-        <v>13.27879202972678</v>
+        <v>11.62537038326263</v>
       </c>
       <c r="AA634" t="inlineStr">
         <is>
@@ -63746,43 +63746,43 @@
         <v>0.06633877564817636</v>
       </c>
       <c r="N635" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O635" t="n">
-        <v>0.4026825348140227</v>
+        <v>0.1618411689996719</v>
       </c>
       <c r="P635" t="n">
-        <v>0.4010809930803445</v>
+        <v>0.6041640639305115</v>
       </c>
       <c r="Q635" t="n">
-        <v>0.1962364721056327</v>
+        <v>0.233994796872139</v>
       </c>
       <c r="R635" t="n">
         <v>1</v>
       </c>
       <c r="S635" t="n">
-        <v>-0.1393916120532008</v>
+        <v>0.343667321130429</v>
       </c>
       <c r="T635" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U635" t="n">
-        <v>-0.1393916120532008</v>
+        <v>0.343667321130429</v>
       </c>
       <c r="V635" t="n">
-        <v>0.4026825348140227</v>
+        <v>0.6041640639305115</v>
       </c>
       <c r="W635" t="n">
-        <v>1.73</v>
+        <v>3.6</v>
       </c>
       <c r="X635" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.5</t>
+          <t>dif_prob_mod_bm &gt; -0.25</t>
         </is>
       </c>
       <c r="Y635" t="inlineStr"/>
       <c r="Z635" t="n">
-        <v>0</v>
+        <v>10.57287111878395</v>
       </c>
       <c r="AA635" t="inlineStr">
         <is>
@@ -63848,40 +63848,40 @@
         <v>1</v>
       </c>
       <c r="O636" t="n">
-        <v>0.7745913844514704</v>
+        <v>0.6979084014892578</v>
       </c>
       <c r="P636" t="n">
-        <v>0.2172895827385753</v>
+        <v>0.2521724700927734</v>
       </c>
       <c r="Q636" t="n">
-        <v>0.008119032809954187</v>
+        <v>0.04991911724209785</v>
       </c>
       <c r="R636" t="n">
         <v>1</v>
       </c>
       <c r="S636" t="n">
-        <v>0.1037505973316135</v>
+        <v>0.02706761436940097</v>
       </c>
       <c r="T636" t="n">
         <v>1</v>
       </c>
       <c r="U636" t="n">
-        <v>0.1037505973316135</v>
+        <v>0.02706761436940097</v>
       </c>
       <c r="V636" t="n">
-        <v>0.7745913844514704</v>
+        <v>0.6979084014892578</v>
       </c>
       <c r="W636" t="n">
         <v>1.4</v>
       </c>
       <c r="X636" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.5</t>
+          <t>dif_prob_mod_bm &gt; -0.25</t>
         </is>
       </c>
       <c r="Y636" t="inlineStr"/>
       <c r="Z636" t="n">
-        <v>13.55534922790073</v>
+        <v>12.21339702606201</v>
       </c>
       <c r="AA636" t="inlineStr">
         <is>
@@ -63947,40 +63947,40 @@
         <v>2</v>
       </c>
       <c r="O637" t="n">
-        <v>0.26709617836359</v>
+        <v>0.2134273052215576</v>
       </c>
       <c r="P637" t="n">
-        <v>0.2749479399344654</v>
+        <v>0.1886194497346878</v>
       </c>
       <c r="Q637" t="n">
-        <v>0.4579558817019445</v>
+        <v>0.597953200340271</v>
       </c>
       <c r="R637" t="n">
         <v>1</v>
       </c>
       <c r="S637" t="n">
-        <v>0.1151458281378737</v>
+        <v>0.2551431467762001</v>
       </c>
       <c r="T637" t="n">
         <v>2</v>
       </c>
       <c r="U637" t="n">
-        <v>0.1151458281378737</v>
+        <v>0.2551431467762001</v>
       </c>
       <c r="V637" t="n">
-        <v>0.4579558817019445</v>
+        <v>0.597953200340271</v>
       </c>
       <c r="W637" t="n">
         <v>2.75</v>
       </c>
       <c r="X637" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.5</t>
+          <t>dif_prob_mod_bm &gt; -0.25</t>
         </is>
       </c>
       <c r="Y637" t="inlineStr"/>
       <c r="Z637" t="n">
-        <v>8.014227929784029</v>
+        <v>10.46418100595474</v>
       </c>
       <c r="AA637" t="inlineStr">
         <is>
@@ -64046,40 +64046,40 @@
         <v>0</v>
       </c>
       <c r="O638" t="n">
-        <v>0.3015195750249093</v>
+        <v>0.3529403209686279</v>
       </c>
       <c r="P638" t="n">
-        <v>0.4061404499255671</v>
+        <v>0.4221764802932739</v>
       </c>
       <c r="Q638" t="n">
-        <v>0.2923399750495236</v>
+        <v>0.2248831689357758</v>
       </c>
       <c r="R638" t="n">
         <v>1</v>
       </c>
       <c r="S638" t="n">
-        <v>0.1388192198403503</v>
+        <v>0.1548552502080572</v>
       </c>
       <c r="T638" t="n">
         <v>0</v>
       </c>
       <c r="U638" t="n">
-        <v>0.1388192198403503</v>
+        <v>0.1548552502080572</v>
       </c>
       <c r="V638" t="n">
-        <v>0.4061404499255671</v>
+        <v>0.4221764802932739</v>
       </c>
       <c r="W638" t="n">
         <v>3.5</v>
       </c>
       <c r="X638" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.5</t>
+          <t>dif_prob_mod_bm &gt; -0.25</t>
         </is>
       </c>
       <c r="Y638" t="inlineStr"/>
       <c r="Z638" t="n">
-        <v>7.107457873697424</v>
+        <v>7.388088405132294</v>
       </c>
       <c r="AA638" t="inlineStr">
         <is>
@@ -64147,40 +64147,40 @@
         <v>1</v>
       </c>
       <c r="O639" t="n">
-        <v>0.5894690908832416</v>
+        <v>0.4925592541694641</v>
       </c>
       <c r="P639" t="n">
-        <v>0.2590308906176526</v>
+        <v>0.3403346836566925</v>
       </c>
       <c r="Q639" t="n">
-        <v>0.1515000184991058</v>
+        <v>0.1671060621738434</v>
       </c>
       <c r="R639" t="n">
         <v>1</v>
       </c>
       <c r="S639" t="n">
-        <v>0.2038330592338198</v>
+        <v>0.1069232225200423</v>
       </c>
       <c r="T639" t="n">
         <v>1</v>
       </c>
       <c r="U639" t="n">
-        <v>0.2038330592338198</v>
+        <v>0.1069232225200423</v>
       </c>
       <c r="V639" t="n">
-        <v>0.5894690908832416</v>
+        <v>0.4925592541694641</v>
       </c>
       <c r="W639" t="n">
         <v>2.45</v>
       </c>
       <c r="X639" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.5</t>
+          <t>dif_prob_mod_bm &gt; -0.25</t>
         </is>
       </c>
       <c r="Y639" t="inlineStr"/>
       <c r="Z639" t="n">
-        <v>10.31570909045673</v>
+        <v>8.619786947965622</v>
       </c>
       <c r="AA639" t="inlineStr">
         <is>
@@ -64234,13 +64234,13 @@
         <v>2</v>
       </c>
       <c r="O640" t="n">
-        <v>0.04759327094221052</v>
+        <v>0.2457361966371536</v>
       </c>
       <c r="P640" t="n">
-        <v>0.1400388062730517</v>
+        <v>0.2980333566665649</v>
       </c>
       <c r="Q640" t="n">
-        <v>0.8123679227847378</v>
+        <v>0.4562304019927979</v>
       </c>
       <c r="R640" t="n">
         <v>1</v>
@@ -64251,12 +64251,12 @@
       </c>
       <c r="U640" t="inlineStr"/>
       <c r="V640" t="n">
-        <v>0.1876320772152622</v>
+        <v>0.5437695980072021</v>
       </c>
       <c r="W640" t="inlineStr"/>
       <c r="X640" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &lt; -0.5</t>
+          <t>dif_prob_mod_bm &lt; -0.25</t>
         </is>
       </c>
       <c r="Y640" t="inlineStr"/>
@@ -64311,13 +64311,13 @@
         <v>2</v>
       </c>
       <c r="O641" t="n">
-        <v>0.03427928789846806</v>
+        <v>0.04795290529727936</v>
       </c>
       <c r="P641" t="n">
-        <v>0.07558148975112403</v>
+        <v>0.05862414836883545</v>
       </c>
       <c r="Q641" t="n">
-        <v>0.890139222350408</v>
+        <v>0.8934229612350464</v>
       </c>
       <c r="R641" t="n">
         <v>1</v>
@@ -64328,12 +64328,12 @@
       </c>
       <c r="U641" t="inlineStr"/>
       <c r="V641" t="n">
-        <v>0.109860777649592</v>
+        <v>0.1065770387649536</v>
       </c>
       <c r="W641" t="inlineStr"/>
       <c r="X641" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &lt; -0.5</t>
+          <t>dif_prob_mod_bm &lt; -0.25</t>
         </is>
       </c>
       <c r="Y641" t="inlineStr"/>

</xml_diff>

<commit_message>
Actualizo predicciones de GER tras cambio de modelo
</commit_message>
<xml_diff>
--- a/data/historial_predicciones.xlsx
+++ b/data/historial_predicciones.xlsx
@@ -61474,197 +61474,195 @@
     <row r="613">
       <c r="A613" s="1" t="inlineStr">
         <is>
-          <t>EuQnZBVQ</t>
+          <t>WENRFI84</t>
         </is>
       </c>
       <c r="B613" s="2" t="n">
-        <v>45618.6875</v>
+        <v>45619.45833333334</v>
       </c>
       <c r="C613" t="inlineStr">
         <is>
-          <t>bayern munich</t>
+          <t>verona</t>
         </is>
       </c>
       <c r="D613" t="inlineStr">
         <is>
-          <t>augsburg</t>
+          <t>inter</t>
         </is>
       </c>
       <c r="E613" t="n">
-        <v>59</v>
+        <v>77</v>
       </c>
       <c r="F613" t="n">
-        <v>591</v>
+        <v>771</v>
       </c>
       <c r="G613" t="n">
-        <v>1.13</v>
+        <v>7</v>
       </c>
       <c r="H613" t="n">
-        <v>10</v>
+        <v>5.25</v>
       </c>
       <c r="I613" t="n">
-        <v>15</v>
+        <v>1.38</v>
       </c>
       <c r="J613" t="n">
-        <v>0.8415147265077139</v>
+        <v>0.1350293542074364</v>
       </c>
       <c r="K613" t="n">
-        <v>0.09509116409537166</v>
+        <v>0.1800391389432485</v>
       </c>
       <c r="L613" t="n">
-        <v>0.06339410939691444</v>
+        <v>0.6849315068493151</v>
       </c>
       <c r="M613" t="n">
-        <v>0.05162241887905616</v>
+        <v>0.05797101449275366</v>
       </c>
       <c r="N613" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O613" t="n">
-        <v>0.6659861207008362</v>
+        <v>0.07605352458246978</v>
       </c>
       <c r="P613" t="n">
-        <v>0.1339152902364731</v>
+        <v>0.2423606517662135</v>
       </c>
       <c r="Q613" t="n">
-        <v>0.2000985443592072</v>
+        <v>0.6815858236513167</v>
       </c>
       <c r="R613" t="n">
         <v>1</v>
       </c>
       <c r="S613" t="n">
-        <v>-0.1755286058068777</v>
+        <v>-0.003345683197998439</v>
       </c>
       <c r="T613" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U613" t="n">
-        <v>-0.1755286058068777</v>
+        <v>-0.003345683197998439</v>
       </c>
       <c r="V613" t="n">
-        <v>0.6659861207008362</v>
+        <v>0.6815858236513167</v>
       </c>
       <c r="W613" t="n">
-        <v>1.13</v>
+        <v>1.38</v>
       </c>
       <c r="X613" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.25</t>
+          <t>dif_prob_mod_bm &gt; -0.5</t>
         </is>
       </c>
       <c r="Y613" t="inlineStr"/>
       <c r="Z613" t="n">
-        <v>0</v>
+        <v>11.69355409003815</v>
       </c>
       <c r="AA613" t="inlineStr">
         <is>
-          <t>germany</t>
+          <t>italy</t>
         </is>
       </c>
       <c r="AB613" t="inlineStr">
         <is>
-          <t>bundesliga</t>
-        </is>
-      </c>
-      <c r="AC613" t="n">
-        <v>1</v>
-      </c>
+          <t>serie a</t>
+        </is>
+      </c>
+      <c r="AC613" t="inlineStr"/>
       <c r="AD613" t="inlineStr"/>
       <c r="AE613" t="inlineStr"/>
     </row>
     <row r="614">
       <c r="A614" s="1" t="inlineStr">
         <is>
-          <t>2qNaDU87</t>
+          <t>z7KrCz8T</t>
         </is>
       </c>
       <c r="B614" s="2" t="n">
-        <v>45619.47916666666</v>
+        <v>45619.58333333334</v>
       </c>
       <c r="C614" t="inlineStr">
         <is>
-          <t>bayer leverkusen</t>
+          <t>ac milan</t>
         </is>
       </c>
       <c r="D614" t="inlineStr">
         <is>
-          <t>heidenheim</t>
+          <t>juventus</t>
         </is>
       </c>
       <c r="E614" t="n">
-        <v>59</v>
+        <v>77</v>
       </c>
       <c r="F614" t="n">
-        <v>591</v>
+        <v>771</v>
       </c>
       <c r="G614" t="n">
-        <v>1.2</v>
+        <v>2.15</v>
       </c>
       <c r="H614" t="n">
-        <v>6.5</v>
+        <v>3.3</v>
       </c>
       <c r="I614" t="n">
-        <v>15</v>
+        <v>3.5</v>
       </c>
       <c r="J614" t="n">
-        <v>0.7907542579075426</v>
+        <v>0.4413450515857852</v>
       </c>
       <c r="K614" t="n">
-        <v>0.145985401459854</v>
+        <v>0.2875429881543752</v>
       </c>
       <c r="L614" t="n">
-        <v>0.0632603406326034</v>
+        <v>0.2711119602598395</v>
       </c>
       <c r="M614" t="n">
-        <v>0.05384615384615388</v>
+        <v>0.05386086781435617</v>
       </c>
       <c r="N614" t="n">
         <v>1</v>
       </c>
       <c r="O614" t="n">
-        <v>0.8486636281013489</v>
+        <v>0.35669835414836</v>
       </c>
       <c r="P614" t="n">
-        <v>0.1071945801377296</v>
+        <v>0.3483631099687277</v>
       </c>
       <c r="Q614" t="n">
-        <v>0.04414178058505058</v>
+        <v>0.2949385358829122</v>
       </c>
       <c r="R614" t="n">
         <v>1</v>
       </c>
       <c r="S614" t="n">
-        <v>0.05790937019380626</v>
+        <v>-0.0846466974374252</v>
       </c>
       <c r="T614" t="n">
         <v>1</v>
       </c>
       <c r="U614" t="n">
-        <v>0.05790937019380626</v>
+        <v>-0.0846466974374252</v>
       </c>
       <c r="V614" t="n">
-        <v>0.8486636281013489</v>
+        <v>0.35669835414836</v>
       </c>
       <c r="W614" t="n">
-        <v>1.2</v>
+        <v>2.15</v>
       </c>
       <c r="X614" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.25</t>
+          <t>dif_prob_mod_bm &gt; -0.5</t>
         </is>
       </c>
       <c r="Y614" t="inlineStr"/>
       <c r="Z614" t="n">
-        <v>5.940645396709442</v>
+        <v>0.3169523769765367</v>
       </c>
       <c r="AA614" t="inlineStr">
         <is>
-          <t>germany</t>
+          <t>italy</t>
         </is>
       </c>
       <c r="AB614" t="inlineStr">
         <is>
-          <t>bundesliga</t>
+          <t>serie a</t>
         </is>
       </c>
       <c r="AC614" t="inlineStr"/>
@@ -61674,96 +61672,96 @@
     <row r="615">
       <c r="A615" s="1" t="inlineStr">
         <is>
-          <t>pOGITkgl</t>
+          <t>Qyq1UHNc</t>
         </is>
       </c>
       <c r="B615" s="2" t="n">
-        <v>45619.47916666666</v>
+        <v>45619.69791666666</v>
       </c>
       <c r="C615" t="inlineStr">
         <is>
-          <t>dortmund</t>
+          <t>parma</t>
         </is>
       </c>
       <c r="D615" t="inlineStr">
         <is>
-          <t>freiburg</t>
+          <t>atalanta</t>
         </is>
       </c>
       <c r="E615" t="n">
-        <v>59</v>
+        <v>77</v>
       </c>
       <c r="F615" t="n">
-        <v>591</v>
+        <v>771</v>
       </c>
       <c r="G615" t="n">
-        <v>1.67</v>
+        <v>5</v>
       </c>
       <c r="H615" t="n">
         <v>4.2</v>
       </c>
       <c r="I615" t="n">
-        <v>4.75</v>
+        <v>1.62</v>
       </c>
       <c r="J615" t="n">
-        <v>0.5716905706876048</v>
+        <v>0.1895053475935829</v>
       </c>
       <c r="K615" t="n">
-        <v>0.2273150602495952</v>
+        <v>0.2256016042780749</v>
       </c>
       <c r="L615" t="n">
-        <v>0.2009943690628</v>
+        <v>0.5848930481283423</v>
       </c>
       <c r="M615" t="n">
-        <v>0.04742394909429271</v>
+        <v>0.0553791887125219</v>
       </c>
       <c r="N615" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O615" t="n">
-        <v>0.7468887567520142</v>
+        <v>0.1777861207576573</v>
       </c>
       <c r="P615" t="n">
-        <v>0.1249512881040573</v>
+        <v>0.2673919524648737</v>
       </c>
       <c r="Q615" t="n">
-        <v>0.1281599253416061</v>
+        <v>0.554821926777469</v>
       </c>
       <c r="R615" t="n">
         <v>1</v>
       </c>
       <c r="S615" t="n">
-        <v>0.1751981860644094</v>
+        <v>-0.03007112135087331</v>
       </c>
       <c r="T615" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U615" t="n">
-        <v>0.1751981860644094</v>
+        <v>-0.03007112135087331</v>
       </c>
       <c r="V615" t="n">
-        <v>0.7468887567520142</v>
+        <v>0.554821926777469</v>
       </c>
       <c r="W615" t="n">
-        <v>1.67</v>
+        <v>1.62</v>
       </c>
       <c r="X615" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.25</t>
+          <t>dif_prob_mod_bm &gt; -0.5</t>
         </is>
       </c>
       <c r="Y615" t="inlineStr"/>
       <c r="Z615" t="n">
-        <v>5.228221297264099</v>
+        <v>7.604405224044576</v>
       </c>
       <c r="AA615" t="inlineStr">
         <is>
-          <t>germany</t>
+          <t>italy</t>
         </is>
       </c>
       <c r="AB615" t="inlineStr">
         <is>
-          <t>bundesliga</t>
+          <t>serie a</t>
         </is>
       </c>
       <c r="AC615" t="inlineStr"/>
@@ -61773,96 +61771,96 @@
     <row r="616">
       <c r="A616" s="1" t="inlineStr">
         <is>
-          <t>E38ZP7hD</t>
+          <t>b1PJHvvh</t>
         </is>
       </c>
       <c r="B616" s="2" t="n">
-        <v>45619.47916666666</v>
+        <v>45620.35416666666</v>
       </c>
       <c r="C616" t="inlineStr">
         <is>
-          <t>hoffenheim</t>
+          <t>genoa</t>
         </is>
       </c>
       <c r="D616" t="inlineStr">
         <is>
-          <t>rb leipzig</t>
+          <t>cagliari</t>
         </is>
       </c>
       <c r="E616" t="n">
-        <v>59</v>
+        <v>77</v>
       </c>
       <c r="F616" t="n">
-        <v>591</v>
+        <v>771</v>
       </c>
       <c r="G616" t="n">
-        <v>3.4</v>
+        <v>2.6</v>
       </c>
       <c r="H616" t="n">
-        <v>3.6</v>
+        <v>3.1</v>
       </c>
       <c r="I616" t="n">
-        <v>2.1</v>
+        <v>2.9</v>
       </c>
       <c r="J616" t="n">
-        <v>0.2806236080178174</v>
+        <v>0.3655957706384709</v>
       </c>
       <c r="K616" t="n">
-        <v>0.2650334075723831</v>
+        <v>0.3066287108580724</v>
       </c>
       <c r="L616" t="n">
-        <v>0.4543429844097996</v>
+        <v>0.3277755185034567</v>
       </c>
       <c r="M616" t="n">
-        <v>0.04808590102707733</v>
+        <v>0.05202361598357141</v>
       </c>
       <c r="N616" t="n">
         <v>0</v>
       </c>
       <c r="O616" t="n">
-        <v>0.1142816692590714</v>
+        <v>0.2535054733691977</v>
       </c>
       <c r="P616" t="n">
-        <v>0.4521372020244598</v>
+        <v>0.3798675715489841</v>
       </c>
       <c r="Q616" t="n">
-        <v>0.4335811138153076</v>
+        <v>0.3666269550818181</v>
       </c>
       <c r="R616" t="n">
         <v>1</v>
       </c>
       <c r="S616" t="n">
-        <v>0.1871037944520767</v>
+        <v>0.07323886069091168</v>
       </c>
       <c r="T616" t="n">
         <v>0</v>
       </c>
       <c r="U616" t="n">
-        <v>0.1871037944520767</v>
+        <v>0.07323886069091168</v>
       </c>
       <c r="V616" t="n">
-        <v>0.4521372020244598</v>
+        <v>0.3798675715489841</v>
       </c>
       <c r="W616" t="n">
-        <v>3.6</v>
+        <v>3.1</v>
       </c>
       <c r="X616" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.25</t>
+          <t>dif_prob_mod_bm &gt; -0.5</t>
         </is>
       </c>
       <c r="Y616" t="inlineStr"/>
       <c r="Z616" t="n">
-        <v>3.164960414171219</v>
+        <v>6.647682502107221</v>
       </c>
       <c r="AA616" t="inlineStr">
         <is>
-          <t>germany</t>
+          <t>italy</t>
         </is>
       </c>
       <c r="AB616" t="inlineStr">
         <is>
-          <t>bundesliga</t>
+          <t>serie a</t>
         </is>
       </c>
       <c r="AC616" t="inlineStr"/>
@@ -61872,195 +61870,197 @@
     <row r="617">
       <c r="A617" s="1" t="inlineStr">
         <is>
-          <t>fwAoyY0E</t>
+          <t>Ewi1acON</t>
         </is>
       </c>
       <c r="B617" s="2" t="n">
-        <v>45619.47916666666</v>
+        <v>45620.45833333334</v>
       </c>
       <c r="C617" t="inlineStr">
         <is>
-          <t>stuttgart</t>
+          <t>como</t>
         </is>
       </c>
       <c r="D617" t="inlineStr">
         <is>
-          <t>bochum</t>
+          <t>fiorentina</t>
         </is>
       </c>
       <c r="E617" t="n">
-        <v>59</v>
+        <v>77</v>
       </c>
       <c r="F617" t="n">
-        <v>591</v>
+        <v>771</v>
       </c>
       <c r="G617" t="n">
-        <v>1.29</v>
+        <v>3.2</v>
       </c>
       <c r="H617" t="n">
-        <v>6</v>
+        <v>3.1</v>
       </c>
       <c r="I617" t="n">
-        <v>9.5</v>
+        <v>2.38</v>
       </c>
       <c r="J617" t="n">
-        <v>0.7403078121955972</v>
+        <v>0.2961387171871237</v>
       </c>
       <c r="K617" t="n">
-        <v>0.1591661796220534</v>
+        <v>0.3056915790318696</v>
       </c>
       <c r="L617" t="n">
-        <v>0.1005260081823495</v>
+        <v>0.3981697037810067</v>
       </c>
       <c r="M617" t="n">
-        <v>0.04712362301101569</v>
+        <v>0.05524871238818108</v>
       </c>
       <c r="N617" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O617" t="n">
-        <v>0.3674966990947723</v>
+        <v>0.04644974435671278</v>
       </c>
       <c r="P617" t="n">
-        <v>0.3553413152694702</v>
+        <v>0.1673757544185006</v>
       </c>
       <c r="Q617" t="n">
-        <v>0.2771620154380798</v>
+        <v>0.7861745012247867</v>
       </c>
       <c r="R617" t="n">
         <v>1</v>
       </c>
       <c r="S617" t="n">
-        <v>-0.3728111131008248</v>
+        <v>0.38800479744378</v>
       </c>
       <c r="T617" t="n">
-        <v>-1</v>
+        <v>2</v>
       </c>
       <c r="U617" t="n">
-        <v>0.3728111131008248</v>
+        <v>0.38800479744378</v>
       </c>
       <c r="V617" t="n">
-        <v>0.6325033009052277</v>
+        <v>0.7861745012247867</v>
       </c>
       <c r="W617" t="n">
-        <v>3.67741935483871</v>
+        <v>2.38</v>
       </c>
       <c r="X617" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &lt; -0.25</t>
+          <t>dif_prob_mod_bm &gt; -0.5</t>
         </is>
       </c>
       <c r="Y617" t="inlineStr"/>
       <c r="Z617" t="n">
-        <v>4.427523106336594</v>
+        <v>13.75805377143377</v>
       </c>
       <c r="AA617" t="inlineStr">
         <is>
-          <t>germany</t>
+          <t>italy</t>
         </is>
       </c>
       <c r="AB617" t="inlineStr">
         <is>
-          <t>bundesliga</t>
-        </is>
-      </c>
-      <c r="AC617" t="inlineStr"/>
+          <t>serie a</t>
+        </is>
+      </c>
+      <c r="AC617" t="n">
+        <v>1</v>
+      </c>
       <c r="AD617" t="inlineStr"/>
       <c r="AE617" t="inlineStr"/>
     </row>
     <row r="618">
       <c r="A618" s="1" t="inlineStr">
         <is>
-          <t>SrjMmBpK</t>
+          <t>M3xASehA</t>
         </is>
       </c>
       <c r="B618" s="2" t="n">
-        <v>45619.47916666666</v>
+        <v>45620.45833333334</v>
       </c>
       <c r="C618" t="inlineStr">
         <is>
-          <t>wolfsburg</t>
+          <t>torino</t>
         </is>
       </c>
       <c r="D618" t="inlineStr">
         <is>
-          <t>union berlin</t>
+          <t>monza</t>
         </is>
       </c>
       <c r="E618" t="n">
-        <v>59</v>
+        <v>77</v>
       </c>
       <c r="F618" t="n">
-        <v>591</v>
+        <v>771</v>
       </c>
       <c r="G618" t="n">
-        <v>2.25</v>
+        <v>2.05</v>
       </c>
       <c r="H618" t="n">
-        <v>3.3</v>
+        <v>3.2</v>
       </c>
       <c r="I618" t="n">
-        <v>3.3</v>
+        <v>4.1</v>
       </c>
       <c r="J618" t="n">
-        <v>0.4230769230769231</v>
+        <v>0.4671532846715329</v>
       </c>
       <c r="K618" t="n">
-        <v>0.2884615384615385</v>
+        <v>0.2992700729927008</v>
       </c>
       <c r="L618" t="n">
-        <v>0.2884615384615385</v>
+        <v>0.2335766423357664</v>
       </c>
       <c r="M618" t="n">
-        <v>0.05050505050505039</v>
+        <v>0.04420731707317072</v>
       </c>
       <c r="N618" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O618" t="n">
-        <v>0.2910822629928589</v>
+        <v>0.2445397211952143</v>
       </c>
       <c r="P618" t="n">
-        <v>0.188929095864296</v>
+        <v>0.4735163323756597</v>
       </c>
       <c r="Q618" t="n">
-        <v>0.5199886560440063</v>
+        <v>0.2819439464291261</v>
       </c>
       <c r="R618" t="n">
         <v>1</v>
       </c>
       <c r="S618" t="n">
-        <v>0.2315271175824679</v>
+        <v>0.174246259382959</v>
       </c>
       <c r="T618" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="U618" t="n">
-        <v>0.2315271175824679</v>
+        <v>0.174246259382959</v>
       </c>
       <c r="V618" t="n">
-        <v>0.5199886560440063</v>
+        <v>0.4735163323756597</v>
       </c>
       <c r="W618" t="n">
-        <v>3.3</v>
+        <v>3.2</v>
       </c>
       <c r="X618" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.25</t>
+          <t>dif_prob_mod_bm &gt; -0.5</t>
         </is>
       </c>
       <c r="Y618" t="inlineStr"/>
       <c r="Z618" t="n">
-        <v>3.639920592308044</v>
+        <v>8.286535816574045</v>
       </c>
       <c r="AA618" t="inlineStr">
         <is>
-          <t>germany</t>
+          <t>italy</t>
         </is>
       </c>
       <c r="AB618" t="inlineStr">
         <is>
-          <t>bundesliga</t>
+          <t>serie a</t>
         </is>
       </c>
       <c r="AC618" t="inlineStr"/>
@@ -62070,96 +62070,96 @@
     <row r="619">
       <c r="A619" s="1" t="inlineStr">
         <is>
-          <t>6w5RRTN0</t>
+          <t>KvdF6EVj</t>
         </is>
       </c>
       <c r="B619" s="2" t="n">
-        <v>45619.60416666666</v>
+        <v>45620.58333333334</v>
       </c>
       <c r="C619" t="inlineStr">
         <is>
-          <t>eintracht frankfurt</t>
+          <t>napoli</t>
         </is>
       </c>
       <c r="D619" t="inlineStr">
         <is>
-          <t>werder bremen</t>
+          <t>as roma</t>
         </is>
       </c>
       <c r="E619" t="n">
-        <v>59</v>
+        <v>77</v>
       </c>
       <c r="F619" t="n">
-        <v>591</v>
+        <v>771</v>
       </c>
       <c r="G619" t="n">
         <v>1.73</v>
       </c>
       <c r="H619" t="n">
-        <v>4.1</v>
+        <v>3.6</v>
       </c>
       <c r="I619" t="n">
-        <v>4.33</v>
+        <v>5</v>
       </c>
       <c r="J619" t="n">
-        <v>0.5490012957333573</v>
+        <v>0.5474785570898474</v>
       </c>
       <c r="K619" t="n">
-        <v>0.2316517662484654</v>
+        <v>0.2630938621570655</v>
       </c>
       <c r="L619" t="n">
-        <v>0.2193469380181774</v>
+        <v>0.1894275807530872</v>
       </c>
       <c r="M619" t="n">
-        <v>0.05288400332240517</v>
+        <v>0.05581245985870265</v>
       </c>
       <c r="N619" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O619" t="n">
-        <v>0.231614962220192</v>
+        <v>0.423275112177328</v>
       </c>
       <c r="P619" t="n">
-        <v>0.5006377100944519</v>
+        <v>0.3892870005141383</v>
       </c>
       <c r="Q619" t="n">
-        <v>0.2677473425865173</v>
+        <v>0.1874378873085338</v>
       </c>
       <c r="R619" t="n">
         <v>1</v>
       </c>
       <c r="S619" t="n">
-        <v>0.2689859438459865</v>
+        <v>-0.1242034449125194</v>
       </c>
       <c r="T619" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U619" t="n">
-        <v>0.2689859438459865</v>
+        <v>-0.1242034449125194</v>
       </c>
       <c r="V619" t="n">
-        <v>0.5006377100944519</v>
+        <v>0.423275112177328</v>
       </c>
       <c r="W619" t="n">
-        <v>4.1</v>
+        <v>1.73</v>
       </c>
       <c r="X619" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.25</t>
+          <t>dif_prob_mod_bm &gt; -0.5</t>
         </is>
       </c>
       <c r="Y619" t="inlineStr"/>
       <c r="Z619" t="n">
-        <v>3.504463970661163</v>
+        <v>0</v>
       </c>
       <c r="AA619" t="inlineStr">
         <is>
-          <t>germany</t>
+          <t>italy</t>
         </is>
       </c>
       <c r="AB619" t="inlineStr">
         <is>
-          <t>bundesliga</t>
+          <t>serie a</t>
         </is>
       </c>
       <c r="AC619" t="inlineStr"/>
@@ -62169,96 +62169,96 @@
     <row r="620">
       <c r="A620" s="1" t="inlineStr">
         <is>
-          <t>KtV0tTxf</t>
+          <t>StHzEdwH</t>
         </is>
       </c>
       <c r="B620" s="2" t="n">
-        <v>45620.47916666666</v>
+        <v>45620.69791666666</v>
       </c>
       <c r="C620" t="inlineStr">
         <is>
-          <t>holstein kiel</t>
+          <t>lazio</t>
         </is>
       </c>
       <c r="D620" t="inlineStr">
         <is>
-          <t>mainz</t>
+          <t>bologna</t>
         </is>
       </c>
       <c r="E620" t="n">
-        <v>59</v>
+        <v>77</v>
       </c>
       <c r="F620" t="n">
-        <v>591</v>
+        <v>771</v>
       </c>
       <c r="G620" t="n">
-        <v>3.1</v>
+        <v>1.9</v>
       </c>
       <c r="H620" t="n">
-        <v>3.4</v>
+        <v>3.5</v>
       </c>
       <c r="I620" t="n">
-        <v>2.3</v>
+        <v>4.2</v>
       </c>
       <c r="J620" t="n">
-        <v>0.3067869752844252</v>
+        <v>0.5011933174224343</v>
       </c>
       <c r="K620" t="n">
-        <v>0.2797175362887406</v>
+        <v>0.2720763723150358</v>
       </c>
       <c r="L620" t="n">
-        <v>0.413495488426834</v>
+        <v>0.2267303102625298</v>
       </c>
       <c r="M620" t="n">
-        <v>0.05148090091576618</v>
+        <v>0.05012531328320802</v>
       </c>
       <c r="N620" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O620" t="n">
-        <v>0.0898820087313652</v>
+        <v>0.3619515607914891</v>
       </c>
       <c r="P620" t="n">
-        <v>0.2830811440944672</v>
+        <v>0.3888795289225333</v>
       </c>
       <c r="Q620" t="n">
-        <v>0.6270368695259094</v>
+        <v>0.2491689102859776</v>
       </c>
       <c r="R620" t="n">
         <v>1</v>
       </c>
       <c r="S620" t="n">
-        <v>0.2135413810990754</v>
+        <v>0.1168031566074975</v>
       </c>
       <c r="T620" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="U620" t="n">
-        <v>0.2135413810990754</v>
+        <v>0.1168031566074975</v>
       </c>
       <c r="V620" t="n">
-        <v>0.6270368695259094</v>
+        <v>0.3888795289225333</v>
       </c>
       <c r="W620" t="n">
-        <v>2.3</v>
+        <v>3.5</v>
       </c>
       <c r="X620" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.25</t>
+          <t>dif_prob_mod_bm &gt; -0.5</t>
         </is>
       </c>
       <c r="Y620" t="inlineStr"/>
       <c r="Z620" t="n">
-        <v>4.389258086681366</v>
+        <v>6.805391756144333</v>
       </c>
       <c r="AA620" t="inlineStr">
         <is>
-          <t>germany</t>
+          <t>italy</t>
         </is>
       </c>
       <c r="AB620" t="inlineStr">
         <is>
-          <t>bundesliga</t>
+          <t>serie a</t>
         </is>
       </c>
       <c r="AC620" t="inlineStr"/>
@@ -62268,96 +62268,96 @@
     <row r="621">
       <c r="A621" s="1" t="inlineStr">
         <is>
-          <t>OEyhrk8s</t>
+          <t>pMsXgyno</t>
         </is>
       </c>
       <c r="B621" s="2" t="n">
-        <v>45620.5625</v>
+        <v>45621.60416666666</v>
       </c>
       <c r="C621" t="inlineStr">
         <is>
-          <t>b  monchengladbach</t>
+          <t>empoli</t>
         </is>
       </c>
       <c r="D621" t="inlineStr">
         <is>
-          <t>st  pauli</t>
+          <t>udinese</t>
         </is>
       </c>
       <c r="E621" t="n">
-        <v>59</v>
+        <v>77</v>
       </c>
       <c r="F621" t="n">
-        <v>591</v>
+        <v>771</v>
       </c>
       <c r="G621" t="n">
-        <v>1.8</v>
+        <v>2.8</v>
       </c>
       <c r="H621" t="n">
-        <v>3.8</v>
+        <v>2.9</v>
       </c>
       <c r="I621" t="n">
-        <v>4.2</v>
+        <v>2.8</v>
       </c>
       <c r="J621" t="n">
-        <v>0.5256916996047432</v>
+        <v>0.3372093023255813</v>
       </c>
       <c r="K621" t="n">
-        <v>0.2490118577075099</v>
+        <v>0.3255813953488372</v>
       </c>
       <c r="L621" t="n">
-        <v>0.225296442687747</v>
+        <v>0.3372093023255813</v>
       </c>
       <c r="M621" t="n">
-        <v>0.05680868838763575</v>
+        <v>0.05911330049261099</v>
       </c>
       <c r="N621" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O621" t="n">
-        <v>0.3624015152454376</v>
+        <v>0.4336302148290543</v>
       </c>
       <c r="P621" t="n">
-        <v>0.4057324230670929</v>
+        <v>0.3649604099178962</v>
       </c>
       <c r="Q621" t="n">
-        <v>0.2318660914897919</v>
+        <v>0.2014093752530495</v>
       </c>
       <c r="R621" t="n">
         <v>1</v>
       </c>
       <c r="S621" t="n">
-        <v>0.156720565359583</v>
+        <v>0.09642091250347301</v>
       </c>
       <c r="T621" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U621" t="n">
-        <v>0.156720565359583</v>
+        <v>0.09642091250347301</v>
       </c>
       <c r="V621" t="n">
-        <v>0.4057324230670929</v>
+        <v>0.4336302148290543</v>
       </c>
       <c r="W621" t="n">
-        <v>3.8</v>
+        <v>2.8</v>
       </c>
       <c r="X621" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.25</t>
+          <t>dif_prob_mod_bm &gt; -0.5</t>
         </is>
       </c>
       <c r="Y621" t="inlineStr"/>
       <c r="Z621" t="n">
-        <v>2.84012696146965</v>
+        <v>7.588528759508451</v>
       </c>
       <c r="AA621" t="inlineStr">
         <is>
-          <t>germany</t>
+          <t>italy</t>
         </is>
       </c>
       <c r="AB621" t="inlineStr">
         <is>
-          <t>bundesliga</t>
+          <t>serie a</t>
         </is>
       </c>
       <c r="AC621" t="inlineStr"/>
@@ -62367,20 +62367,20 @@
     <row r="622">
       <c r="A622" s="1" t="inlineStr">
         <is>
-          <t>WENRFI84</t>
+          <t>hjasAmxq</t>
         </is>
       </c>
       <c r="B622" s="2" t="n">
-        <v>45619.45833333334</v>
+        <v>45621.69791666666</v>
       </c>
       <c r="C622" t="inlineStr">
         <is>
-          <t>verona</t>
+          <t>venezia</t>
         </is>
       </c>
       <c r="D622" t="inlineStr">
         <is>
-          <t>inter</t>
+          <t>lecce</t>
         </is>
       </c>
       <c r="E622" t="n">
@@ -62390,55 +62390,55 @@
         <v>771</v>
       </c>
       <c r="G622" t="n">
-        <v>7</v>
+        <v>2.3</v>
       </c>
       <c r="H622" t="n">
-        <v>5.25</v>
+        <v>3.25</v>
       </c>
       <c r="I622" t="n">
-        <v>1.38</v>
+        <v>3.2</v>
       </c>
       <c r="J622" t="n">
-        <v>0.1350293542074364</v>
+        <v>0.4121260154547257</v>
       </c>
       <c r="K622" t="n">
-        <v>0.1800391389432485</v>
+        <v>0.2916584109371904</v>
       </c>
       <c r="L622" t="n">
-        <v>0.6849315068493151</v>
+        <v>0.296215573608084</v>
       </c>
       <c r="M622" t="n">
-        <v>0.05797101449275366</v>
+        <v>0.05497491638795982</v>
       </c>
       <c r="N622" t="n">
         <v>2</v>
       </c>
       <c r="O622" t="n">
-        <v>0.07605352458246978</v>
+        <v>0.1856164616886396</v>
       </c>
       <c r="P622" t="n">
-        <v>0.2423606517662135</v>
+        <v>0.3424946146248241</v>
       </c>
       <c r="Q622" t="n">
-        <v>0.6815858236513167</v>
+        <v>0.4718889236865362</v>
       </c>
       <c r="R622" t="n">
         <v>1</v>
       </c>
       <c r="S622" t="n">
-        <v>-0.003345683197998439</v>
+        <v>0.1756733500784522</v>
       </c>
       <c r="T622" t="n">
         <v>2</v>
       </c>
       <c r="U622" t="n">
-        <v>-0.003345683197998439</v>
+        <v>0.1756733500784522</v>
       </c>
       <c r="V622" t="n">
-        <v>0.6815858236513167</v>
+        <v>0.4718889236865362</v>
       </c>
       <c r="W622" t="n">
-        <v>1.38</v>
+        <v>3.2</v>
       </c>
       <c r="X622" t="inlineStr">
         <is>
@@ -62447,7 +62447,7 @@
       </c>
       <c r="Y622" t="inlineStr"/>
       <c r="Z622" t="n">
-        <v>11.69355409003815</v>
+        <v>8.258056164514384</v>
       </c>
       <c r="AA622" t="inlineStr">
         <is>
@@ -62466,96 +62466,96 @@
     <row r="623">
       <c r="A623" s="1" t="inlineStr">
         <is>
-          <t>z7KrCz8T</t>
+          <t>SCX7iT7M</t>
         </is>
       </c>
       <c r="B623" s="2" t="n">
-        <v>45619.58333333334</v>
+        <v>45618.70833333334</v>
       </c>
       <c r="C623" t="inlineStr">
         <is>
-          <t>ac milan</t>
+          <t>getafe</t>
         </is>
       </c>
       <c r="D623" t="inlineStr">
         <is>
-          <t>juventus</t>
+          <t>valladolid</t>
         </is>
       </c>
       <c r="E623" t="n">
-        <v>77</v>
+        <v>148</v>
       </c>
       <c r="F623" t="n">
-        <v>771</v>
+        <v>1481</v>
       </c>
       <c r="G623" t="n">
-        <v>2.15</v>
+        <v>1.73</v>
       </c>
       <c r="H623" t="n">
         <v>3.3</v>
       </c>
       <c r="I623" t="n">
-        <v>3.5</v>
+        <v>5.75</v>
       </c>
       <c r="J623" t="n">
-        <v>0.4413450515857852</v>
+        <v>0.5479115833850685</v>
       </c>
       <c r="K623" t="n">
-        <v>0.2875429881543752</v>
+        <v>0.2872384967442935</v>
       </c>
       <c r="L623" t="n">
-        <v>0.2711119602598395</v>
+        <v>0.164849919870638</v>
       </c>
       <c r="M623" t="n">
-        <v>0.05386086781435617</v>
+        <v>0.05497802858948875</v>
       </c>
       <c r="N623" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O623" t="n">
-        <v>0.35669835414836</v>
+        <v>0.2291478365659714</v>
       </c>
       <c r="P623" t="n">
-        <v>0.3483631099687277</v>
+        <v>0.6676607728004456</v>
       </c>
       <c r="Q623" t="n">
-        <v>0.2949385358829122</v>
+        <v>0.1031913980841637</v>
       </c>
       <c r="R623" t="n">
         <v>1</v>
       </c>
       <c r="S623" t="n">
-        <v>-0.0846466974374252</v>
+        <v>0.380422276056152</v>
       </c>
       <c r="T623" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U623" t="n">
-        <v>-0.0846466974374252</v>
+        <v>0.380422276056152</v>
       </c>
       <c r="V623" t="n">
-        <v>0.35669835414836</v>
+        <v>0.6676607728004456</v>
       </c>
       <c r="W623" t="n">
-        <v>2.15</v>
+        <v>3.3</v>
       </c>
       <c r="X623" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.5</t>
+          <t>dif_prob_mod_bm &gt; -0.25</t>
         </is>
       </c>
       <c r="Y623" t="inlineStr"/>
       <c r="Z623" t="n">
-        <v>0.3169523769765367</v>
+        <v>11.6840635240078</v>
       </c>
       <c r="AA623" t="inlineStr">
         <is>
-          <t>italy</t>
+          <t>spain</t>
         </is>
       </c>
       <c r="AB623" t="inlineStr">
         <is>
-          <t>serie a</t>
+          <t>laliga</t>
         </is>
       </c>
       <c r="AC623" t="inlineStr"/>
@@ -62565,195 +62565,197 @@
     <row r="624">
       <c r="A624" s="1" t="inlineStr">
         <is>
-          <t>Qyq1UHNc</t>
+          <t>C2KEmK6l</t>
         </is>
       </c>
       <c r="B624" s="2" t="n">
-        <v>45619.69791666666</v>
+        <v>45619.41666666666</v>
       </c>
       <c r="C624" t="inlineStr">
         <is>
-          <t>parma</t>
+          <t>valencia</t>
         </is>
       </c>
       <c r="D624" t="inlineStr">
         <is>
-          <t>atalanta</t>
+          <t>betis</t>
         </is>
       </c>
       <c r="E624" t="n">
-        <v>77</v>
+        <v>148</v>
       </c>
       <c r="F624" t="n">
-        <v>771</v>
+        <v>1481</v>
       </c>
       <c r="G624" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H624" t="n">
-        <v>4.2</v>
+        <v>3</v>
       </c>
       <c r="I624" t="n">
-        <v>1.62</v>
+        <v>2.6</v>
       </c>
       <c r="J624" t="n">
-        <v>0.1895053475935829</v>
+        <v>0.3170731707317074</v>
       </c>
       <c r="K624" t="n">
-        <v>0.2256016042780749</v>
+        <v>0.3170731707317074</v>
       </c>
       <c r="L624" t="n">
-        <v>0.5848930481283423</v>
+        <v>0.3658536585365854</v>
       </c>
       <c r="M624" t="n">
-        <v>0.0553791887125219</v>
+        <v>0.0512820512820511</v>
       </c>
       <c r="N624" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O624" t="n">
-        <v>0.1777861207576573</v>
+        <v>0.3059642314910889</v>
       </c>
       <c r="P624" t="n">
-        <v>0.2673919524648737</v>
+        <v>0.4625942409038544</v>
       </c>
       <c r="Q624" t="n">
-        <v>0.554821926777469</v>
+        <v>0.2314416021108627</v>
       </c>
       <c r="R624" t="n">
         <v>1</v>
       </c>
       <c r="S624" t="n">
-        <v>-0.03007112135087331</v>
+        <v>0.145521070172147</v>
       </c>
       <c r="T624" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="U624" t="n">
-        <v>-0.03007112135087331</v>
+        <v>0.145521070172147</v>
       </c>
       <c r="V624" t="n">
-        <v>0.554821926777469</v>
+        <v>0.4625942409038544</v>
       </c>
       <c r="W624" t="n">
-        <v>1.62</v>
+        <v>3</v>
       </c>
       <c r="X624" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.5</t>
+          <t>dif_prob_mod_bm &gt; -0.25</t>
         </is>
       </c>
       <c r="Y624" t="inlineStr"/>
       <c r="Z624" t="n">
-        <v>7.604405224044576</v>
+        <v>8.095399215817451</v>
       </c>
       <c r="AA624" t="inlineStr">
         <is>
-          <t>italy</t>
+          <t>spain</t>
         </is>
       </c>
       <c r="AB624" t="inlineStr">
         <is>
-          <t>serie a</t>
-        </is>
-      </c>
-      <c r="AC624" t="inlineStr"/>
+          <t>laliga</t>
+        </is>
+      </c>
+      <c r="AC624" t="n">
+        <v>1</v>
+      </c>
       <c r="AD624" t="inlineStr"/>
       <c r="AE624" t="inlineStr"/>
     </row>
     <row r="625">
       <c r="A625" s="1" t="inlineStr">
         <is>
-          <t>b1PJHvvh</t>
+          <t>vVwOqx6D</t>
         </is>
       </c>
       <c r="B625" s="2" t="n">
-        <v>45620.35416666666</v>
+        <v>45619.51041666666</v>
       </c>
       <c r="C625" t="inlineStr">
         <is>
-          <t>genoa</t>
+          <t>atl  madrid</t>
         </is>
       </c>
       <c r="D625" t="inlineStr">
         <is>
-          <t>cagliari</t>
+          <t>alaves</t>
         </is>
       </c>
       <c r="E625" t="n">
-        <v>77</v>
+        <v>148</v>
       </c>
       <c r="F625" t="n">
-        <v>771</v>
+        <v>1481</v>
       </c>
       <c r="G625" t="n">
-        <v>2.6</v>
+        <v>1.36</v>
       </c>
       <c r="H625" t="n">
-        <v>3.1</v>
+        <v>4.75</v>
       </c>
       <c r="I625" t="n">
-        <v>2.9</v>
+        <v>9</v>
       </c>
       <c r="J625" t="n">
-        <v>0.3655957706384709</v>
+        <v>0.6956875508543532</v>
       </c>
       <c r="K625" t="n">
-        <v>0.3066287108580724</v>
+        <v>0.199186330349878</v>
       </c>
       <c r="L625" t="n">
-        <v>0.3277755185034567</v>
+        <v>0.1051261187957689</v>
       </c>
       <c r="M625" t="n">
-        <v>0.05202361598357141</v>
+        <v>0.05693154454764349</v>
       </c>
       <c r="N625" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O625" t="n">
-        <v>0.2535054733691977</v>
+        <v>0.8715217709541321</v>
       </c>
       <c r="P625" t="n">
-        <v>0.3798675715489841</v>
+        <v>0.09871138632297516</v>
       </c>
       <c r="Q625" t="n">
-        <v>0.3666269550818181</v>
+        <v>0.02976679056882858</v>
       </c>
       <c r="R625" t="n">
         <v>1</v>
       </c>
       <c r="S625" t="n">
-        <v>0.07323886069091168</v>
+        <v>0.1758342200997789</v>
       </c>
       <c r="T625" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U625" t="n">
-        <v>0.07323886069091168</v>
+        <v>0.1758342200997789</v>
       </c>
       <c r="V625" t="n">
-        <v>0.3798675715489841</v>
+        <v>0.8715217709541321</v>
       </c>
       <c r="W625" t="n">
-        <v>3.1</v>
+        <v>1.36</v>
       </c>
       <c r="X625" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.5</t>
+          <t>dif_prob_mod_bm &gt; -0.25</t>
         </is>
       </c>
       <c r="Y625" t="inlineStr"/>
       <c r="Z625" t="n">
-        <v>6.647682502107221</v>
+        <v>15.25163099169731</v>
       </c>
       <c r="AA625" t="inlineStr">
         <is>
-          <t>italy</t>
+          <t>spain</t>
         </is>
       </c>
       <c r="AB625" t="inlineStr">
         <is>
-          <t>serie a</t>
+          <t>laliga</t>
         </is>
       </c>
       <c r="AC625" t="inlineStr"/>
@@ -62763,96 +62765,96 @@
     <row r="626">
       <c r="A626" s="1" t="inlineStr">
         <is>
-          <t>Ewi1acON</t>
+          <t>buKPeYL5</t>
         </is>
       </c>
       <c r="B626" s="2" t="n">
-        <v>45620.45833333334</v>
+        <v>45619.60416666666</v>
       </c>
       <c r="C626" t="inlineStr">
         <is>
-          <t>como</t>
+          <t>girona</t>
         </is>
       </c>
       <c r="D626" t="inlineStr">
         <is>
-          <t>fiorentina</t>
+          <t>espanyol</t>
         </is>
       </c>
       <c r="E626" t="n">
-        <v>77</v>
+        <v>148</v>
       </c>
       <c r="F626" t="n">
-        <v>771</v>
+        <v>1481</v>
       </c>
       <c r="G626" t="n">
-        <v>3.2</v>
+        <v>1.67</v>
       </c>
       <c r="H626" t="n">
-        <v>3.1</v>
+        <v>3.8</v>
       </c>
       <c r="I626" t="n">
-        <v>2.38</v>
+        <v>5.25</v>
       </c>
       <c r="J626" t="n">
-        <v>0.2961387171871237</v>
+        <v>0.5689677299756157</v>
       </c>
       <c r="K626" t="n">
-        <v>0.3056915790318696</v>
+        <v>0.2500463444892837</v>
       </c>
       <c r="L626" t="n">
-        <v>0.3981697037810067</v>
+        <v>0.1809859255351006</v>
       </c>
       <c r="M626" t="n">
-        <v>0.05524871238818108</v>
+        <v>0.0524364804226134</v>
       </c>
       <c r="N626" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O626" t="n">
-        <v>0.04644974435671278</v>
+        <v>0.6232661008834839</v>
       </c>
       <c r="P626" t="n">
-        <v>0.1673757544185006</v>
+        <v>0.1015298962593079</v>
       </c>
       <c r="Q626" t="n">
-        <v>0.7861745012247867</v>
+        <v>0.2752040326595306</v>
       </c>
       <c r="R626" t="n">
         <v>1</v>
       </c>
       <c r="S626" t="n">
-        <v>0.38800479744378</v>
+        <v>0.05429837090786815</v>
       </c>
       <c r="T626" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U626" t="n">
-        <v>0.38800479744378</v>
+        <v>0.05429837090786815</v>
       </c>
       <c r="V626" t="n">
-        <v>0.7861745012247867</v>
+        <v>0.6232661008834839</v>
       </c>
       <c r="W626" t="n">
-        <v>2.38</v>
+        <v>1.67</v>
       </c>
       <c r="X626" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.5</t>
+          <t>dif_prob_mod_bm &gt; -0.25</t>
         </is>
       </c>
       <c r="Y626" t="inlineStr"/>
       <c r="Z626" t="n">
-        <v>13.75805377143377</v>
+        <v>10.90715676546097</v>
       </c>
       <c r="AA626" t="inlineStr">
         <is>
-          <t>italy</t>
+          <t>spain</t>
         </is>
       </c>
       <c r="AB626" t="inlineStr">
         <is>
-          <t>serie a</t>
+          <t>laliga</t>
         </is>
       </c>
       <c r="AC626" t="n">
@@ -62864,96 +62866,96 @@
     <row r="627">
       <c r="A627" s="1" t="inlineStr">
         <is>
-          <t>M3xASehA</t>
+          <t>IsCnpo0d</t>
         </is>
       </c>
       <c r="B627" s="2" t="n">
-        <v>45620.45833333334</v>
+        <v>45619.60416666666</v>
       </c>
       <c r="C627" t="inlineStr">
         <is>
-          <t>torino</t>
+          <t>las palmas</t>
         </is>
       </c>
       <c r="D627" t="inlineStr">
         <is>
-          <t>monza</t>
+          <t>mallorca</t>
         </is>
       </c>
       <c r="E627" t="n">
-        <v>77</v>
+        <v>148</v>
       </c>
       <c r="F627" t="n">
-        <v>771</v>
+        <v>1481</v>
       </c>
       <c r="G627" t="n">
-        <v>2.05</v>
+        <v>3</v>
       </c>
       <c r="H627" t="n">
-        <v>3.2</v>
+        <v>3</v>
       </c>
       <c r="I627" t="n">
-        <v>4.1</v>
+        <v>2.55</v>
       </c>
       <c r="J627" t="n">
-        <v>0.4671532846715329</v>
+        <v>0.3148148148148148</v>
       </c>
       <c r="K627" t="n">
-        <v>0.2992700729927008</v>
+        <v>0.3148148148148148</v>
       </c>
       <c r="L627" t="n">
-        <v>0.2335766423357664</v>
+        <v>0.3703703703703704</v>
       </c>
       <c r="M627" t="n">
-        <v>0.04420731707317072</v>
+        <v>0.05882352941176472</v>
       </c>
       <c r="N627" t="n">
         <v>0</v>
       </c>
       <c r="O627" t="n">
-        <v>0.2445397211952143</v>
+        <v>0.2897258102893829</v>
       </c>
       <c r="P627" t="n">
-        <v>0.4735163323756597</v>
+        <v>0.4301001131534576</v>
       </c>
       <c r="Q627" t="n">
-        <v>0.2819439464291261</v>
+        <v>0.2801741063594818</v>
       </c>
       <c r="R627" t="n">
         <v>1</v>
       </c>
       <c r="S627" t="n">
-        <v>0.174246259382959</v>
+        <v>0.1152852983386429</v>
       </c>
       <c r="T627" t="n">
         <v>0</v>
       </c>
       <c r="U627" t="n">
-        <v>0.174246259382959</v>
+        <v>0.1152852983386429</v>
       </c>
       <c r="V627" t="n">
-        <v>0.4735163323756597</v>
+        <v>0.4301001131534576</v>
       </c>
       <c r="W627" t="n">
-        <v>3.2</v>
+        <v>3</v>
       </c>
       <c r="X627" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.5</t>
+          <t>dif_prob_mod_bm &gt; -0.25</t>
         </is>
       </c>
       <c r="Y627" t="inlineStr"/>
       <c r="Z627" t="n">
-        <v>8.286535816574045</v>
+        <v>7.526751980185509</v>
       </c>
       <c r="AA627" t="inlineStr">
         <is>
-          <t>italy</t>
+          <t>spain</t>
         </is>
       </c>
       <c r="AB627" t="inlineStr">
         <is>
-          <t>serie a</t>
+          <t>laliga</t>
         </is>
       </c>
       <c r="AC627" t="inlineStr"/>
@@ -62963,96 +62965,96 @@
     <row r="628">
       <c r="A628" s="1" t="inlineStr">
         <is>
-          <t>KvdF6EVj</t>
+          <t>tGcs6SMF</t>
         </is>
       </c>
       <c r="B628" s="2" t="n">
-        <v>45620.58333333334</v>
+        <v>45619.70833333334</v>
       </c>
       <c r="C628" t="inlineStr">
         <is>
-          <t>napoli</t>
+          <t>celta vigo</t>
         </is>
       </c>
       <c r="D628" t="inlineStr">
         <is>
-          <t>as roma</t>
+          <t>barcelona</t>
         </is>
       </c>
       <c r="E628" t="n">
-        <v>77</v>
+        <v>148</v>
       </c>
       <c r="F628" t="n">
-        <v>771</v>
+        <v>1481</v>
       </c>
       <c r="G628" t="n">
-        <v>1.73</v>
+        <v>4.5</v>
       </c>
       <c r="H628" t="n">
-        <v>3.6</v>
+        <v>4.33</v>
       </c>
       <c r="I628" t="n">
-        <v>5</v>
+        <v>1.67</v>
       </c>
       <c r="J628" t="n">
-        <v>0.5474785570898474</v>
+        <v>0.2112435767474606</v>
       </c>
       <c r="K628" t="n">
-        <v>0.2630938621570655</v>
+        <v>0.2195372044719568</v>
       </c>
       <c r="L628" t="n">
-        <v>0.1894275807530872</v>
+        <v>0.5692192187805826</v>
       </c>
       <c r="M628" t="n">
-        <v>0.05581245985870265</v>
+        <v>0.05197149964889314</v>
       </c>
       <c r="N628" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O628" t="n">
-        <v>0.423275112177328</v>
+        <v>0.04584328830242157</v>
       </c>
       <c r="P628" t="n">
-        <v>0.3892870005141383</v>
+        <v>0.1309177875518799</v>
       </c>
       <c r="Q628" t="n">
-        <v>0.1874378873085338</v>
+        <v>0.8232389092445374</v>
       </c>
       <c r="R628" t="n">
         <v>1</v>
       </c>
       <c r="S628" t="n">
-        <v>-0.1242034449125194</v>
+        <v>0.2540196904639548</v>
       </c>
       <c r="T628" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U628" t="n">
-        <v>-0.1242034449125194</v>
+        <v>0.2540196904639548</v>
       </c>
       <c r="V628" t="n">
-        <v>0.423275112177328</v>
+        <v>0.8232389092445374</v>
       </c>
       <c r="W628" t="n">
-        <v>1.73</v>
+        <v>1.67</v>
       </c>
       <c r="X628" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.5</t>
+          <t>dif_prob_mod_bm &gt; -0.25</t>
         </is>
       </c>
       <c r="Y628" t="inlineStr"/>
       <c r="Z628" t="n">
-        <v>0</v>
+        <v>14.4066809117794</v>
       </c>
       <c r="AA628" t="inlineStr">
         <is>
-          <t>italy</t>
+          <t>spain</t>
         </is>
       </c>
       <c r="AB628" t="inlineStr">
         <is>
-          <t>serie a</t>
+          <t>laliga</t>
         </is>
       </c>
       <c r="AC628" t="inlineStr"/>
@@ -63062,96 +63064,96 @@
     <row r="629">
       <c r="A629" s="1" t="inlineStr">
         <is>
-          <t>StHzEdwH</t>
+          <t>dSNwn7Vq</t>
         </is>
       </c>
       <c r="B629" s="2" t="n">
-        <v>45620.69791666666</v>
+        <v>45620.41666666666</v>
       </c>
       <c r="C629" t="inlineStr">
         <is>
-          <t>lazio</t>
+          <t>osasuna</t>
         </is>
       </c>
       <c r="D629" t="inlineStr">
         <is>
-          <t>bologna</t>
+          <t>villarreal</t>
         </is>
       </c>
       <c r="E629" t="n">
-        <v>77</v>
+        <v>148</v>
       </c>
       <c r="F629" t="n">
-        <v>771</v>
+        <v>1481</v>
       </c>
       <c r="G629" t="n">
-        <v>1.9</v>
+        <v>2.7</v>
       </c>
       <c r="H629" t="n">
-        <v>3.5</v>
+        <v>3.3</v>
       </c>
       <c r="I629" t="n">
-        <v>4.2</v>
+        <v>2.63</v>
       </c>
       <c r="J629" t="n">
-        <v>0.5011933174224343</v>
+        <v>0.3515188335358444</v>
       </c>
       <c r="K629" t="n">
-        <v>0.2720763723150358</v>
+        <v>0.287606318347509</v>
       </c>
       <c r="L629" t="n">
-        <v>0.2267303102625298</v>
+        <v>0.3608748481166464</v>
       </c>
       <c r="M629" t="n">
-        <v>0.05012531328320802</v>
+        <v>0.05362881028280286</v>
       </c>
       <c r="N629" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O629" t="n">
-        <v>0.3619515607914891</v>
+        <v>0.2457459270954132</v>
       </c>
       <c r="P629" t="n">
-        <v>0.3888795289225333</v>
+        <v>0.3619625866413116</v>
       </c>
       <c r="Q629" t="n">
-        <v>0.2491689102859776</v>
+        <v>0.3922915160655975</v>
       </c>
       <c r="R629" t="n">
         <v>1</v>
       </c>
       <c r="S629" t="n">
-        <v>0.1168031566074975</v>
+        <v>0.03141666794895115</v>
       </c>
       <c r="T629" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="U629" t="n">
-        <v>0.1168031566074975</v>
+        <v>0.03141666794895115</v>
       </c>
       <c r="V629" t="n">
-        <v>0.3888795289225333</v>
+        <v>0.3922915160655975</v>
       </c>
       <c r="W629" t="n">
-        <v>3.5</v>
+        <v>2.63</v>
       </c>
       <c r="X629" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.5</t>
+          <t>dif_prob_mod_bm &gt; -0.25</t>
         </is>
       </c>
       <c r="Y629" t="inlineStr"/>
       <c r="Z629" t="n">
-        <v>6.805391756144333</v>
+        <v>6.865101531147957</v>
       </c>
       <c r="AA629" t="inlineStr">
         <is>
-          <t>italy</t>
+          <t>spain</t>
         </is>
       </c>
       <c r="AB629" t="inlineStr">
         <is>
-          <t>serie a</t>
+          <t>laliga</t>
         </is>
       </c>
       <c r="AC629" t="inlineStr"/>
@@ -63161,195 +63163,197 @@
     <row r="630">
       <c r="A630" s="1" t="inlineStr">
         <is>
-          <t>pMsXgyno</t>
+          <t>W4zGoby1</t>
         </is>
       </c>
       <c r="B630" s="2" t="n">
-        <v>45621.60416666666</v>
+        <v>45620.51041666666</v>
       </c>
       <c r="C630" t="inlineStr">
         <is>
-          <t>empoli</t>
+          <t>sevilla</t>
         </is>
       </c>
       <c r="D630" t="inlineStr">
         <is>
-          <t>udinese</t>
+          <t>rayo vallecano</t>
         </is>
       </c>
       <c r="E630" t="n">
-        <v>77</v>
+        <v>148</v>
       </c>
       <c r="F630" t="n">
-        <v>771</v>
+        <v>1481</v>
       </c>
       <c r="G630" t="n">
-        <v>2.8</v>
+        <v>2.3</v>
       </c>
       <c r="H630" t="n">
-        <v>2.9</v>
+        <v>3.2</v>
       </c>
       <c r="I630" t="n">
-        <v>2.8</v>
+        <v>3.3</v>
       </c>
       <c r="J630" t="n">
-        <v>0.3372093023255813</v>
+        <v>0.4139553116424932</v>
       </c>
       <c r="K630" t="n">
-        <v>0.3255813953488372</v>
+        <v>0.2975303802430419</v>
       </c>
       <c r="L630" t="n">
-        <v>0.3372093023255813</v>
+        <v>0.2885143081144649</v>
       </c>
       <c r="M630" t="n">
-        <v>0.05911330049261099</v>
+        <v>0.05031291172595531</v>
       </c>
       <c r="N630" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O630" t="n">
-        <v>0.4336302148290543</v>
+        <v>0.2018209844827652</v>
       </c>
       <c r="P630" t="n">
-        <v>0.3649604099178962</v>
+        <v>0.5636378526687622</v>
       </c>
       <c r="Q630" t="n">
-        <v>0.2014093752530495</v>
+        <v>0.2345411628484726</v>
       </c>
       <c r="R630" t="n">
         <v>1</v>
       </c>
       <c r="S630" t="n">
-        <v>0.09642091250347301</v>
+        <v>0.2661074724257203</v>
       </c>
       <c r="T630" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U630" t="n">
-        <v>0.09642091250347301</v>
+        <v>0.2661074724257203</v>
       </c>
       <c r="V630" t="n">
-        <v>0.4336302148290543</v>
+        <v>0.5636378526687622</v>
       </c>
       <c r="W630" t="n">
-        <v>2.8</v>
+        <v>3.2</v>
       </c>
       <c r="X630" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.5</t>
+          <t>dif_prob_mod_bm &gt; -0.25</t>
         </is>
       </c>
       <c r="Y630" t="inlineStr"/>
       <c r="Z630" t="n">
-        <v>7.588528759508451</v>
+        <v>9.863662421703339</v>
       </c>
       <c r="AA630" t="inlineStr">
         <is>
-          <t>italy</t>
+          <t>spain</t>
         </is>
       </c>
       <c r="AB630" t="inlineStr">
         <is>
-          <t>serie a</t>
-        </is>
-      </c>
-      <c r="AC630" t="inlineStr"/>
+          <t>laliga</t>
+        </is>
+      </c>
+      <c r="AC630" t="n">
+        <v>1</v>
+      </c>
       <c r="AD630" t="inlineStr"/>
       <c r="AE630" t="inlineStr"/>
     </row>
     <row r="631">
       <c r="A631" s="1" t="inlineStr">
         <is>
-          <t>hjasAmxq</t>
+          <t>pl4Y7lh3</t>
         </is>
       </c>
       <c r="B631" s="2" t="n">
-        <v>45621.69791666666</v>
+        <v>45620.60416666666</v>
       </c>
       <c r="C631" t="inlineStr">
         <is>
-          <t>venezia</t>
+          <t>leganes</t>
         </is>
       </c>
       <c r="D631" t="inlineStr">
         <is>
-          <t>lecce</t>
+          <t>real madrid</t>
         </is>
       </c>
       <c r="E631" t="n">
-        <v>77</v>
+        <v>148</v>
       </c>
       <c r="F631" t="n">
-        <v>771</v>
+        <v>1481</v>
       </c>
       <c r="G631" t="n">
-        <v>2.3</v>
+        <v>7</v>
       </c>
       <c r="H631" t="n">
-        <v>3.25</v>
+        <v>4.5</v>
       </c>
       <c r="I631" t="n">
-        <v>3.2</v>
+        <v>1.45</v>
       </c>
       <c r="J631" t="n">
-        <v>0.4121260154547257</v>
+        <v>0.1354436948624805</v>
       </c>
       <c r="K631" t="n">
-        <v>0.2916584109371904</v>
+        <v>0.210690192008303</v>
       </c>
       <c r="L631" t="n">
-        <v>0.296215573608084</v>
+        <v>0.6538661131292164</v>
       </c>
       <c r="M631" t="n">
-        <v>0.05497491638795982</v>
+        <v>0.05473453749315826</v>
       </c>
       <c r="N631" t="n">
         <v>2</v>
       </c>
       <c r="O631" t="n">
-        <v>0.1856164616886396</v>
+        <v>0.0941070169210434</v>
       </c>
       <c r="P631" t="n">
-        <v>0.3424946146248241</v>
+        <v>0.09887459129095078</v>
       </c>
       <c r="Q631" t="n">
-        <v>0.4718889236865362</v>
+        <v>0.8070184588432312</v>
       </c>
       <c r="R631" t="n">
         <v>1</v>
       </c>
       <c r="S631" t="n">
-        <v>0.1756733500784522</v>
+        <v>0.1531523457140148</v>
       </c>
       <c r="T631" t="n">
         <v>2</v>
       </c>
       <c r="U631" t="n">
-        <v>0.1756733500784522</v>
+        <v>0.1531523457140148</v>
       </c>
       <c r="V631" t="n">
-        <v>0.4718889236865362</v>
+        <v>0.8070184588432312</v>
       </c>
       <c r="W631" t="n">
-        <v>3.2</v>
+        <v>1.45</v>
       </c>
       <c r="X631" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.5</t>
+          <t>dif_prob_mod_bm &gt; -0.25</t>
         </is>
       </c>
       <c r="Y631" t="inlineStr"/>
       <c r="Z631" t="n">
-        <v>8.258056164514384</v>
+        <v>14.12282302975655</v>
       </c>
       <c r="AA631" t="inlineStr">
         <is>
-          <t>italy</t>
+          <t>spain</t>
         </is>
       </c>
       <c r="AB631" t="inlineStr">
         <is>
-          <t>serie a</t>
+          <t>laliga</t>
         </is>
       </c>
       <c r="AC631" t="inlineStr"/>
@@ -63359,20 +63363,20 @@
     <row r="632">
       <c r="A632" s="1" t="inlineStr">
         <is>
-          <t>SCX7iT7M</t>
+          <t>WpvagkwA</t>
         </is>
       </c>
       <c r="B632" s="2" t="n">
-        <v>45618.70833333334</v>
+        <v>45620.70833333334</v>
       </c>
       <c r="C632" t="inlineStr">
         <is>
-          <t>getafe</t>
+          <t>ath bilbao</t>
         </is>
       </c>
       <c r="D632" t="inlineStr">
         <is>
-          <t>valladolid</t>
+          <t>real sociedad</t>
         </is>
       </c>
       <c r="E632" t="n">
@@ -63382,55 +63386,55 @@
         <v>1481</v>
       </c>
       <c r="G632" t="n">
-        <v>1.73</v>
+        <v>2.2</v>
       </c>
       <c r="H632" t="n">
-        <v>3.3</v>
+        <v>3</v>
       </c>
       <c r="I632" t="n">
-        <v>5.75</v>
+        <v>3.75</v>
       </c>
       <c r="J632" t="n">
-        <v>0.5479115833850685</v>
+        <v>0.4310344827586207</v>
       </c>
       <c r="K632" t="n">
-        <v>0.2872384967442935</v>
+        <v>0.3160919540229885</v>
       </c>
       <c r="L632" t="n">
-        <v>0.164849919870638</v>
+        <v>0.2528735632183908</v>
       </c>
       <c r="M632" t="n">
-        <v>0.05497802858948875</v>
+        <v>0.05454545454545445</v>
       </c>
       <c r="N632" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O632" t="n">
-        <v>0.2291478365659714</v>
+        <v>0.3089075982570648</v>
       </c>
       <c r="P632" t="n">
-        <v>0.6676607728004456</v>
+        <v>0.2107562869787216</v>
       </c>
       <c r="Q632" t="n">
-        <v>0.1031913980841637</v>
+        <v>0.4803360998630524</v>
       </c>
       <c r="R632" t="n">
         <v>1</v>
       </c>
       <c r="S632" t="n">
-        <v>0.380422276056152</v>
+        <v>0.2274625366446615</v>
       </c>
       <c r="T632" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="U632" t="n">
-        <v>0.380422276056152</v>
+        <v>0.2274625366446615</v>
       </c>
       <c r="V632" t="n">
-        <v>0.6676607728004456</v>
+        <v>0.4803360998630524</v>
       </c>
       <c r="W632" t="n">
-        <v>3.3</v>
+        <v>3.75</v>
       </c>
       <c r="X632" t="inlineStr">
         <is>
@@ -63439,7 +63443,7 @@
       </c>
       <c r="Y632" t="inlineStr"/>
       <c r="Z632" t="n">
-        <v>11.6840635240078</v>
+        <v>8.405881747603416</v>
       </c>
       <c r="AA632" t="inlineStr">
         <is>
@@ -63458,96 +63462,96 @@
     <row r="633">
       <c r="A633" s="1" t="inlineStr">
         <is>
-          <t>C2KEmK6l</t>
+          <t>EuQnZBVQ</t>
         </is>
       </c>
       <c r="B633" s="2" t="n">
-        <v>45619.41666666666</v>
+        <v>45618.6875</v>
       </c>
       <c r="C633" t="inlineStr">
         <is>
-          <t>valencia</t>
+          <t>bayern munich</t>
         </is>
       </c>
       <c r="D633" t="inlineStr">
         <is>
-          <t>betis</t>
+          <t>augsburg</t>
         </is>
       </c>
       <c r="E633" t="n">
-        <v>148</v>
+        <v>59</v>
       </c>
       <c r="F633" t="n">
-        <v>1481</v>
+        <v>591</v>
       </c>
       <c r="G633" t="n">
-        <v>3</v>
+        <v>1.13</v>
       </c>
       <c r="H633" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="I633" t="n">
-        <v>2.6</v>
+        <v>15</v>
       </c>
       <c r="J633" t="n">
-        <v>0.3170731707317074</v>
+        <v>0.8415147265077139</v>
       </c>
       <c r="K633" t="n">
-        <v>0.3170731707317074</v>
+        <v>0.09509116409537166</v>
       </c>
       <c r="L633" t="n">
-        <v>0.3658536585365854</v>
+        <v>0.06339410939691444</v>
       </c>
       <c r="M633" t="n">
-        <v>0.0512820512820511</v>
+        <v>0.05162241887905616</v>
       </c>
       <c r="N633" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O633" t="n">
-        <v>0.3059642314910889</v>
+        <v>0.816745400428772</v>
       </c>
       <c r="P633" t="n">
-        <v>0.4625942409038544</v>
+        <v>0.1343889534473419</v>
       </c>
       <c r="Q633" t="n">
-        <v>0.2314416021108627</v>
+        <v>0.04886569455265999</v>
       </c>
       <c r="R633" t="n">
         <v>1</v>
       </c>
       <c r="S633" t="n">
-        <v>0.145521070172147</v>
+        <v>-0.02476932607894189</v>
       </c>
       <c r="T633" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U633" t="n">
-        <v>0.145521070172147</v>
+        <v>-0.02476932607894189</v>
       </c>
       <c r="V633" t="n">
-        <v>0.4625942409038544</v>
+        <v>0.816745400428772</v>
       </c>
       <c r="W633" t="n">
-        <v>3</v>
+        <v>1.13</v>
       </c>
       <c r="X633" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.25</t>
+          <t>dif_prob_mod_bm &gt; -0.35</t>
         </is>
       </c>
       <c r="Y633" t="inlineStr"/>
       <c r="Z633" t="n">
-        <v>8.095399215817451</v>
+        <v>3.588340480565022</v>
       </c>
       <c r="AA633" t="inlineStr">
         <is>
-          <t>spain</t>
+          <t>germany</t>
         </is>
       </c>
       <c r="AB633" t="inlineStr">
         <is>
-          <t>laliga</t>
+          <t>bundesliga</t>
         </is>
       </c>
       <c r="AC633" t="n">
@@ -63559,96 +63563,96 @@
     <row r="634">
       <c r="A634" s="1" t="inlineStr">
         <is>
-          <t>vVwOqx6D</t>
+          <t>2qNaDU87</t>
         </is>
       </c>
       <c r="B634" s="2" t="n">
-        <v>45619.51041666666</v>
+        <v>45619.47916666666</v>
       </c>
       <c r="C634" t="inlineStr">
         <is>
-          <t>atl  madrid</t>
+          <t>bayer leverkusen</t>
         </is>
       </c>
       <c r="D634" t="inlineStr">
         <is>
-          <t>alaves</t>
+          <t>heidenheim</t>
         </is>
       </c>
       <c r="E634" t="n">
-        <v>148</v>
+        <v>59</v>
       </c>
       <c r="F634" t="n">
-        <v>1481</v>
+        <v>591</v>
       </c>
       <c r="G634" t="n">
-        <v>1.36</v>
+        <v>1.2</v>
       </c>
       <c r="H634" t="n">
-        <v>4.75</v>
+        <v>6.5</v>
       </c>
       <c r="I634" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="J634" t="n">
-        <v>0.6956875508543532</v>
+        <v>0.7907542579075426</v>
       </c>
       <c r="K634" t="n">
-        <v>0.199186330349878</v>
+        <v>0.145985401459854</v>
       </c>
       <c r="L634" t="n">
-        <v>0.1051261187957689</v>
+        <v>0.0632603406326034</v>
       </c>
       <c r="M634" t="n">
-        <v>0.05693154454764349</v>
+        <v>0.05384615384615388</v>
       </c>
       <c r="N634" t="n">
         <v>1</v>
       </c>
       <c r="O634" t="n">
-        <v>0.8715217709541321</v>
+        <v>0.58930504322052</v>
       </c>
       <c r="P634" t="n">
-        <v>0.09871138632297516</v>
+        <v>0.3469331860542297</v>
       </c>
       <c r="Q634" t="n">
-        <v>0.02976679056882858</v>
+        <v>0.06376180797815323</v>
       </c>
       <c r="R634" t="n">
         <v>1</v>
       </c>
       <c r="S634" t="n">
-        <v>0.1758342200997789</v>
+        <v>-0.2014492146870226</v>
       </c>
       <c r="T634" t="n">
         <v>1</v>
       </c>
       <c r="U634" t="n">
-        <v>0.1758342200997789</v>
+        <v>-0.2014492146870226</v>
       </c>
       <c r="V634" t="n">
-        <v>0.8715217709541321</v>
+        <v>0.58930504322052</v>
       </c>
       <c r="W634" t="n">
-        <v>1.36</v>
+        <v>1.2</v>
       </c>
       <c r="X634" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.25</t>
+          <t>dif_prob_mod_bm &gt; -0.35</t>
         </is>
       </c>
       <c r="Y634" t="inlineStr"/>
       <c r="Z634" t="n">
-        <v>15.25163099169731</v>
+        <v>0</v>
       </c>
       <c r="AA634" t="inlineStr">
         <is>
-          <t>spain</t>
+          <t>germany</t>
         </is>
       </c>
       <c r="AB634" t="inlineStr">
         <is>
-          <t>laliga</t>
+          <t>bundesliga</t>
         </is>
       </c>
       <c r="AC634" t="inlineStr"/>
@@ -63658,197 +63662,195 @@
     <row r="635">
       <c r="A635" s="1" t="inlineStr">
         <is>
-          <t>buKPeYL5</t>
+          <t>pOGITkgl</t>
         </is>
       </c>
       <c r="B635" s="2" t="n">
-        <v>45619.60416666666</v>
+        <v>45619.47916666666</v>
       </c>
       <c r="C635" t="inlineStr">
         <is>
-          <t>girona</t>
+          <t>dortmund</t>
         </is>
       </c>
       <c r="D635" t="inlineStr">
         <is>
-          <t>espanyol</t>
+          <t>freiburg</t>
         </is>
       </c>
       <c r="E635" t="n">
-        <v>148</v>
+        <v>59</v>
       </c>
       <c r="F635" t="n">
-        <v>1481</v>
+        <v>591</v>
       </c>
       <c r="G635" t="n">
         <v>1.67</v>
       </c>
       <c r="H635" t="n">
-        <v>3.8</v>
+        <v>4.2</v>
       </c>
       <c r="I635" t="n">
-        <v>5.25</v>
+        <v>4.75</v>
       </c>
       <c r="J635" t="n">
-        <v>0.5689677299756157</v>
+        <v>0.5716905706876048</v>
       </c>
       <c r="K635" t="n">
-        <v>0.2500463444892837</v>
+        <v>0.2273150602495952</v>
       </c>
       <c r="L635" t="n">
-        <v>0.1809859255351006</v>
+        <v>0.2009943690628</v>
       </c>
       <c r="M635" t="n">
-        <v>0.0524364804226134</v>
+        <v>0.04742394909429271</v>
       </c>
       <c r="N635" t="n">
         <v>1</v>
       </c>
       <c r="O635" t="n">
-        <v>0.6232661008834839</v>
+        <v>0.5137215852737427</v>
       </c>
       <c r="P635" t="n">
-        <v>0.1015298962593079</v>
+        <v>0.2179991900920868</v>
       </c>
       <c r="Q635" t="n">
-        <v>0.2752040326595306</v>
+        <v>0.2682792246341705</v>
       </c>
       <c r="R635" t="n">
         <v>1</v>
       </c>
       <c r="S635" t="n">
-        <v>0.05429837090786815</v>
+        <v>-0.05796898541386208</v>
       </c>
       <c r="T635" t="n">
         <v>1</v>
       </c>
       <c r="U635" t="n">
-        <v>0.05429837090786815</v>
+        <v>-0.05796898541386208</v>
       </c>
       <c r="V635" t="n">
-        <v>0.6232661008834839</v>
+        <v>0.5137215852737427</v>
       </c>
       <c r="W635" t="n">
         <v>1.67</v>
       </c>
       <c r="X635" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.25</t>
+          <t>dif_prob_mod_bm &gt; -0.35</t>
         </is>
       </c>
       <c r="Y635" t="inlineStr"/>
       <c r="Z635" t="n">
-        <v>10.90715676546097</v>
+        <v>1.409228218091472</v>
       </c>
       <c r="AA635" t="inlineStr">
         <is>
-          <t>spain</t>
+          <t>germany</t>
         </is>
       </c>
       <c r="AB635" t="inlineStr">
         <is>
-          <t>laliga</t>
-        </is>
-      </c>
-      <c r="AC635" t="n">
-        <v>1</v>
-      </c>
+          <t>bundesliga</t>
+        </is>
+      </c>
+      <c r="AC635" t="inlineStr"/>
       <c r="AD635" t="inlineStr"/>
       <c r="AE635" t="inlineStr"/>
     </row>
     <row r="636">
       <c r="A636" s="1" t="inlineStr">
         <is>
-          <t>IsCnpo0d</t>
+          <t>E38ZP7hD</t>
         </is>
       </c>
       <c r="B636" s="2" t="n">
-        <v>45619.60416666666</v>
+        <v>45619.47916666666</v>
       </c>
       <c r="C636" t="inlineStr">
         <is>
-          <t>las palmas</t>
+          <t>hoffenheim</t>
         </is>
       </c>
       <c r="D636" t="inlineStr">
         <is>
-          <t>mallorca</t>
+          <t>rb leipzig</t>
         </is>
       </c>
       <c r="E636" t="n">
-        <v>148</v>
+        <v>59</v>
       </c>
       <c r="F636" t="n">
-        <v>1481</v>
+        <v>591</v>
       </c>
       <c r="G636" t="n">
-        <v>3</v>
+        <v>3.4</v>
       </c>
       <c r="H636" t="n">
-        <v>3</v>
+        <v>3.6</v>
       </c>
       <c r="I636" t="n">
-        <v>2.55</v>
+        <v>2.1</v>
       </c>
       <c r="J636" t="n">
-        <v>0.3148148148148148</v>
+        <v>0.2806236080178174</v>
       </c>
       <c r="K636" t="n">
-        <v>0.3148148148148148</v>
+        <v>0.2650334075723831</v>
       </c>
       <c r="L636" t="n">
-        <v>0.3703703703703704</v>
+        <v>0.4543429844097996</v>
       </c>
       <c r="M636" t="n">
-        <v>0.05882352941176472</v>
+        <v>0.04808590102707733</v>
       </c>
       <c r="N636" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O636" t="n">
-        <v>0.2897258102893829</v>
+        <v>0.4148953557014465</v>
       </c>
       <c r="P636" t="n">
-        <v>0.4301001131534576</v>
+        <v>0.288111537694931</v>
       </c>
       <c r="Q636" t="n">
-        <v>0.2801741063594818</v>
+        <v>0.2969931662082672</v>
       </c>
       <c r="R636" t="n">
         <v>1</v>
       </c>
       <c r="S636" t="n">
-        <v>0.1152852983386429</v>
+        <v>0.1342717476836291</v>
       </c>
       <c r="T636" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U636" t="n">
-        <v>0.1152852983386429</v>
+        <v>0.1342717476836291</v>
       </c>
       <c r="V636" t="n">
-        <v>0.4301001131534576</v>
+        <v>0.4148953557014465</v>
       </c>
       <c r="W636" t="n">
-        <v>3</v>
+        <v>3.4</v>
       </c>
       <c r="X636" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.25</t>
+          <t>dif_prob_mod_bm &gt; -0.35</t>
         </is>
       </c>
       <c r="Y636" t="inlineStr"/>
       <c r="Z636" t="n">
-        <v>7.526751980185509</v>
+        <v>4.759911732179814</v>
       </c>
       <c r="AA636" t="inlineStr">
         <is>
-          <t>spain</t>
+          <t>germany</t>
         </is>
       </c>
       <c r="AB636" t="inlineStr">
         <is>
-          <t>laliga</t>
+          <t>bundesliga</t>
         </is>
       </c>
       <c r="AC636" t="inlineStr"/>
@@ -63858,96 +63860,96 @@
     <row r="637">
       <c r="A637" s="1" t="inlineStr">
         <is>
-          <t>tGcs6SMF</t>
+          <t>fwAoyY0E</t>
         </is>
       </c>
       <c r="B637" s="2" t="n">
-        <v>45619.70833333334</v>
+        <v>45619.47916666666</v>
       </c>
       <c r="C637" t="inlineStr">
         <is>
-          <t>celta vigo</t>
+          <t>stuttgart</t>
         </is>
       </c>
       <c r="D637" t="inlineStr">
         <is>
-          <t>barcelona</t>
+          <t>bochum</t>
         </is>
       </c>
       <c r="E637" t="n">
-        <v>148</v>
+        <v>59</v>
       </c>
       <c r="F637" t="n">
-        <v>1481</v>
+        <v>591</v>
       </c>
       <c r="G637" t="n">
-        <v>4.5</v>
+        <v>1.29</v>
       </c>
       <c r="H637" t="n">
-        <v>4.33</v>
+        <v>6</v>
       </c>
       <c r="I637" t="n">
-        <v>1.67</v>
+        <v>9.5</v>
       </c>
       <c r="J637" t="n">
-        <v>0.2112435767474606</v>
+        <v>0.7403078121955972</v>
       </c>
       <c r="K637" t="n">
-        <v>0.2195372044719568</v>
+        <v>0.1591661796220534</v>
       </c>
       <c r="L637" t="n">
-        <v>0.5692192187805826</v>
+        <v>0.1005260081823495</v>
       </c>
       <c r="M637" t="n">
-        <v>0.05197149964889314</v>
+        <v>0.04712362301101569</v>
       </c>
       <c r="N637" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O637" t="n">
-        <v>0.04584328830242157</v>
+        <v>0.4565851092338562</v>
       </c>
       <c r="P637" t="n">
-        <v>0.1309177875518799</v>
+        <v>0.3439750373363495</v>
       </c>
       <c r="Q637" t="n">
-        <v>0.8232389092445374</v>
+        <v>0.1994399130344391</v>
       </c>
       <c r="R637" t="n">
         <v>1</v>
       </c>
       <c r="S637" t="n">
-        <v>0.2540196904639548</v>
+        <v>-0.283722702961741</v>
       </c>
       <c r="T637" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U637" t="n">
-        <v>0.2540196904639548</v>
+        <v>-0.283722702961741</v>
       </c>
       <c r="V637" t="n">
-        <v>0.8232389092445374</v>
+        <v>0.4565851092338562</v>
       </c>
       <c r="W637" t="n">
-        <v>1.67</v>
+        <v>1.29</v>
       </c>
       <c r="X637" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.25</t>
+          <t>dif_prob_mod_bm &gt; -0.35</t>
         </is>
       </c>
       <c r="Y637" t="inlineStr"/>
       <c r="Z637" t="n">
-        <v>14.4066809117794</v>
+        <v>0</v>
       </c>
       <c r="AA637" t="inlineStr">
         <is>
-          <t>spain</t>
+          <t>germany</t>
         </is>
       </c>
       <c r="AB637" t="inlineStr">
         <is>
-          <t>laliga</t>
+          <t>bundesliga</t>
         </is>
       </c>
       <c r="AC637" t="inlineStr"/>
@@ -63957,96 +63959,96 @@
     <row r="638">
       <c r="A638" s="1" t="inlineStr">
         <is>
-          <t>dSNwn7Vq</t>
+          <t>SrjMmBpK</t>
         </is>
       </c>
       <c r="B638" s="2" t="n">
-        <v>45620.41666666666</v>
+        <v>45619.47916666666</v>
       </c>
       <c r="C638" t="inlineStr">
         <is>
-          <t>osasuna</t>
+          <t>wolfsburg</t>
         </is>
       </c>
       <c r="D638" t="inlineStr">
         <is>
-          <t>villarreal</t>
+          <t>union berlin</t>
         </is>
       </c>
       <c r="E638" t="n">
-        <v>148</v>
+        <v>59</v>
       </c>
       <c r="F638" t="n">
-        <v>1481</v>
+        <v>591</v>
       </c>
       <c r="G638" t="n">
-        <v>2.7</v>
+        <v>2.25</v>
       </c>
       <c r="H638" t="n">
         <v>3.3</v>
       </c>
       <c r="I638" t="n">
-        <v>2.63</v>
+        <v>3.3</v>
       </c>
       <c r="J638" t="n">
-        <v>0.3515188335358444</v>
+        <v>0.4230769230769231</v>
       </c>
       <c r="K638" t="n">
-        <v>0.287606318347509</v>
+        <v>0.2884615384615385</v>
       </c>
       <c r="L638" t="n">
-        <v>0.3608748481166464</v>
+        <v>0.2884615384615385</v>
       </c>
       <c r="M638" t="n">
-        <v>0.05362881028280286</v>
+        <v>0.05050505050505039</v>
       </c>
       <c r="N638" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O638" t="n">
-        <v>0.2457459270954132</v>
+        <v>0.1679377406835556</v>
       </c>
       <c r="P638" t="n">
-        <v>0.3619625866413116</v>
+        <v>0.5087574124336243</v>
       </c>
       <c r="Q638" t="n">
-        <v>0.3922915160655975</v>
+        <v>0.3233048617839813</v>
       </c>
       <c r="R638" t="n">
         <v>1</v>
       </c>
       <c r="S638" t="n">
-        <v>0.03141666794895115</v>
+        <v>0.2202958739720858</v>
       </c>
       <c r="T638" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="U638" t="n">
-        <v>0.03141666794895115</v>
+        <v>0.2202958739720858</v>
       </c>
       <c r="V638" t="n">
-        <v>0.3922915160655975</v>
+        <v>0.5087574124336243</v>
       </c>
       <c r="W638" t="n">
-        <v>2.63</v>
+        <v>3.3</v>
       </c>
       <c r="X638" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.25</t>
+          <t>dif_prob_mod_bm &gt; -0.35</t>
         </is>
       </c>
       <c r="Y638" t="inlineStr"/>
       <c r="Z638" t="n">
-        <v>6.865101531147957</v>
+        <v>6.949704541609837</v>
       </c>
       <c r="AA638" t="inlineStr">
         <is>
-          <t>spain</t>
+          <t>germany</t>
         </is>
       </c>
       <c r="AB638" t="inlineStr">
         <is>
-          <t>laliga</t>
+          <t>bundesliga</t>
         </is>
       </c>
       <c r="AC638" t="inlineStr"/>
@@ -64056,197 +64058,195 @@
     <row r="639">
       <c r="A639" s="1" t="inlineStr">
         <is>
-          <t>W4zGoby1</t>
+          <t>6w5RRTN0</t>
         </is>
       </c>
       <c r="B639" s="2" t="n">
-        <v>45620.51041666666</v>
+        <v>45619.60416666666</v>
       </c>
       <c r="C639" t="inlineStr">
         <is>
-          <t>sevilla</t>
+          <t>eintracht frankfurt</t>
         </is>
       </c>
       <c r="D639" t="inlineStr">
         <is>
-          <t>rayo vallecano</t>
+          <t>werder bremen</t>
         </is>
       </c>
       <c r="E639" t="n">
-        <v>148</v>
+        <v>59</v>
       </c>
       <c r="F639" t="n">
-        <v>1481</v>
+        <v>591</v>
       </c>
       <c r="G639" t="n">
-        <v>2.3</v>
+        <v>1.73</v>
       </c>
       <c r="H639" t="n">
-        <v>3.2</v>
+        <v>4.1</v>
       </c>
       <c r="I639" t="n">
-        <v>3.3</v>
+        <v>4.33</v>
       </c>
       <c r="J639" t="n">
-        <v>0.4139553116424932</v>
+        <v>0.5490012957333573</v>
       </c>
       <c r="K639" t="n">
-        <v>0.2975303802430419</v>
+        <v>0.2316517662484654</v>
       </c>
       <c r="L639" t="n">
-        <v>0.2885143081144649</v>
+        <v>0.2193469380181774</v>
       </c>
       <c r="M639" t="n">
-        <v>0.05031291172595531</v>
+        <v>0.05288400332240517</v>
       </c>
       <c r="N639" t="n">
         <v>0</v>
       </c>
       <c r="O639" t="n">
-        <v>0.2018209844827652</v>
+        <v>0.2694219946861267</v>
       </c>
       <c r="P639" t="n">
-        <v>0.5636378526687622</v>
+        <v>0.3896504938602448</v>
       </c>
       <c r="Q639" t="n">
-        <v>0.2345411628484726</v>
+        <v>0.3409274816513062</v>
       </c>
       <c r="R639" t="n">
         <v>1</v>
       </c>
       <c r="S639" t="n">
-        <v>0.2661074724257203</v>
+        <v>0.1579987276117794</v>
       </c>
       <c r="T639" t="n">
         <v>0</v>
       </c>
       <c r="U639" t="n">
-        <v>0.2661074724257203</v>
+        <v>0.1579987276117794</v>
       </c>
       <c r="V639" t="n">
-        <v>0.5636378526687622</v>
+        <v>0.3896504938602448</v>
       </c>
       <c r="W639" t="n">
-        <v>3.2</v>
+        <v>4.1</v>
       </c>
       <c r="X639" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.25</t>
+          <t>dif_prob_mod_bm &gt; -0.35</t>
         </is>
       </c>
       <c r="Y639" t="inlineStr"/>
       <c r="Z639" t="n">
-        <v>9.863662421703339</v>
+        <v>5.108227021536811</v>
       </c>
       <c r="AA639" t="inlineStr">
         <is>
-          <t>spain</t>
+          <t>germany</t>
         </is>
       </c>
       <c r="AB639" t="inlineStr">
         <is>
-          <t>laliga</t>
-        </is>
-      </c>
-      <c r="AC639" t="n">
-        <v>1</v>
-      </c>
+          <t>bundesliga</t>
+        </is>
+      </c>
+      <c r="AC639" t="inlineStr"/>
       <c r="AD639" t="inlineStr"/>
       <c r="AE639" t="inlineStr"/>
     </row>
     <row r="640">
       <c r="A640" s="1" t="inlineStr">
         <is>
-          <t>pl4Y7lh3</t>
+          <t>KtV0tTxf</t>
         </is>
       </c>
       <c r="B640" s="2" t="n">
-        <v>45620.60416666666</v>
+        <v>45620.47916666666</v>
       </c>
       <c r="C640" t="inlineStr">
         <is>
-          <t>leganes</t>
+          <t>holstein kiel</t>
         </is>
       </c>
       <c r="D640" t="inlineStr">
         <is>
-          <t>real madrid</t>
+          <t>mainz</t>
         </is>
       </c>
       <c r="E640" t="n">
-        <v>148</v>
+        <v>59</v>
       </c>
       <c r="F640" t="n">
-        <v>1481</v>
+        <v>591</v>
       </c>
       <c r="G640" t="n">
-        <v>7</v>
+        <v>3.1</v>
       </c>
       <c r="H640" t="n">
-        <v>4.5</v>
+        <v>3.4</v>
       </c>
       <c r="I640" t="n">
-        <v>1.45</v>
+        <v>2.3</v>
       </c>
       <c r="J640" t="n">
-        <v>0.1354436948624805</v>
+        <v>0.3067869752844252</v>
       </c>
       <c r="K640" t="n">
-        <v>0.210690192008303</v>
+        <v>0.2797175362887406</v>
       </c>
       <c r="L640" t="n">
-        <v>0.6538661131292164</v>
+        <v>0.413495488426834</v>
       </c>
       <c r="M640" t="n">
-        <v>0.05473453749315826</v>
+        <v>0.05148090091576618</v>
       </c>
       <c r="N640" t="n">
         <v>2</v>
       </c>
       <c r="O640" t="n">
-        <v>0.0941070169210434</v>
+        <v>0.2973787784576416</v>
       </c>
       <c r="P640" t="n">
-        <v>0.09887459129095078</v>
+        <v>0.2567306756973267</v>
       </c>
       <c r="Q640" t="n">
-        <v>0.8070184588432312</v>
+        <v>0.4458905756473541</v>
       </c>
       <c r="R640" t="n">
         <v>1</v>
       </c>
       <c r="S640" t="n">
-        <v>0.1531523457140148</v>
+        <v>0.03239508722052009</v>
       </c>
       <c r="T640" t="n">
         <v>2</v>
       </c>
       <c r="U640" t="n">
-        <v>0.1531523457140148</v>
+        <v>0.03239508722052009</v>
       </c>
       <c r="V640" t="n">
-        <v>0.8070184588432312</v>
+        <v>0.4458905756473541</v>
       </c>
       <c r="W640" t="n">
-        <v>1.45</v>
+        <v>2.3</v>
       </c>
       <c r="X640" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.25</t>
+          <t>dif_prob_mod_bm &gt; -0.35</t>
         </is>
       </c>
       <c r="Y640" t="inlineStr"/>
       <c r="Z640" t="n">
-        <v>14.12282302975655</v>
+        <v>2.877354622647172</v>
       </c>
       <c r="AA640" t="inlineStr">
         <is>
-          <t>spain</t>
+          <t>germany</t>
         </is>
       </c>
       <c r="AB640" t="inlineStr">
         <is>
-          <t>laliga</t>
+          <t>bundesliga</t>
         </is>
       </c>
       <c r="AC640" t="inlineStr"/>
@@ -64256,96 +64256,96 @@
     <row r="641">
       <c r="A641" s="1" t="inlineStr">
         <is>
-          <t>WpvagkwA</t>
+          <t>OEyhrk8s</t>
         </is>
       </c>
       <c r="B641" s="2" t="n">
-        <v>45620.70833333334</v>
+        <v>45620.5625</v>
       </c>
       <c r="C641" t="inlineStr">
         <is>
-          <t>ath bilbao</t>
+          <t>b  monchengladbach</t>
         </is>
       </c>
       <c r="D641" t="inlineStr">
         <is>
-          <t>real sociedad</t>
+          <t>st  pauli</t>
         </is>
       </c>
       <c r="E641" t="n">
-        <v>148</v>
+        <v>59</v>
       </c>
       <c r="F641" t="n">
-        <v>1481</v>
+        <v>591</v>
       </c>
       <c r="G641" t="n">
-        <v>2.2</v>
+        <v>1.8</v>
       </c>
       <c r="H641" t="n">
-        <v>3</v>
+        <v>3.8</v>
       </c>
       <c r="I641" t="n">
-        <v>3.75</v>
+        <v>4.2</v>
       </c>
       <c r="J641" t="n">
-        <v>0.4310344827586207</v>
+        <v>0.5256916996047432</v>
       </c>
       <c r="K641" t="n">
-        <v>0.3160919540229885</v>
+        <v>0.2490118577075099</v>
       </c>
       <c r="L641" t="n">
-        <v>0.2528735632183908</v>
+        <v>0.225296442687747</v>
       </c>
       <c r="M641" t="n">
-        <v>0.05454545454545445</v>
+        <v>0.05680868838763575</v>
       </c>
       <c r="N641" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O641" t="n">
-        <v>0.3089075982570648</v>
+        <v>0.4326812624931335</v>
       </c>
       <c r="P641" t="n">
-        <v>0.2107562869787216</v>
+        <v>0.3608728647232056</v>
       </c>
       <c r="Q641" t="n">
-        <v>0.4803360998630524</v>
+        <v>0.2064459025859833</v>
       </c>
       <c r="R641" t="n">
         <v>1</v>
       </c>
       <c r="S641" t="n">
-        <v>0.2274625366446615</v>
+        <v>-0.09301043711160961</v>
       </c>
       <c r="T641" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U641" t="n">
-        <v>0.2274625366446615</v>
+        <v>-0.09301043711160961</v>
       </c>
       <c r="V641" t="n">
-        <v>0.4803360998630524</v>
+        <v>0.4326812624931335</v>
       </c>
       <c r="W641" t="n">
-        <v>3.75</v>
+        <v>1.8</v>
       </c>
       <c r="X641" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.25</t>
+          <t>dif_prob_mod_bm &gt; -0.35</t>
         </is>
       </c>
       <c r="Y641" t="inlineStr"/>
       <c r="Z641" t="n">
-        <v>8.405881747603416</v>
+        <v>0.3031975702334755</v>
       </c>
       <c r="AA641" t="inlineStr">
         <is>
-          <t>spain</t>
+          <t>germany</t>
         </is>
       </c>
       <c r="AB641" t="inlineStr">
         <is>
-          <t>laliga</t>
+          <t>bundesliga</t>
         </is>
       </c>
       <c r="AC641" t="inlineStr"/>

</xml_diff>

<commit_message>
DATA. Actualizo predicciones de SPA tras cambio de modelo
</commit_message>
<xml_diff>
--- a/data/historial_predicciones.xlsx
+++ b/data/historial_predicciones.xlsx
@@ -68206,55 +68206,55 @@
         <v>1481</v>
       </c>
       <c r="G680" t="n">
-        <v>2.1</v>
+        <v>2</v>
       </c>
       <c r="H680" t="n">
         <v>3</v>
       </c>
       <c r="I680" t="n">
-        <v>4.2</v>
+        <v>4.5</v>
       </c>
       <c r="J680" t="n">
-        <v>0.4545454545454545</v>
+        <v>0.4736842105263159</v>
       </c>
       <c r="K680" t="n">
-        <v>0.3181818181818181</v>
+        <v>0.3157894736842106</v>
       </c>
       <c r="L680" t="n">
-        <v>0.2272727272727272</v>
+        <v>0.2105263157894737</v>
       </c>
       <c r="M680" t="n">
-        <v>0.04761904761904767</v>
+        <v>0.05555555555555536</v>
       </c>
       <c r="N680" t="n">
         <v>1</v>
       </c>
       <c r="O680" t="n">
-        <v>0.6691015928987419</v>
+        <v>0.3431180417537689</v>
       </c>
       <c r="P680" t="n">
-        <v>0.06142903498792147</v>
+        <v>0.3292394876480103</v>
       </c>
       <c r="Q680" t="n">
-        <v>0.2694693721133367</v>
+        <v>0.3276424705982208</v>
       </c>
       <c r="R680" t="n">
         <v>1</v>
       </c>
       <c r="S680" t="n">
-        <v>0.2145561383532875</v>
+        <v>-0.130566168772547</v>
       </c>
       <c r="T680" t="n">
         <v>1</v>
       </c>
       <c r="U680" t="n">
-        <v>0.2145561383532875</v>
+        <v>-0.130566168772547</v>
       </c>
       <c r="V680" t="n">
-        <v>0.6691015928987419</v>
+        <v>0.3431180417537689</v>
       </c>
       <c r="W680" t="n">
-        <v>2.1</v>
+        <v>2</v>
       </c>
       <c r="X680" t="inlineStr">
         <is>
@@ -68263,7 +68263,7 @@
       </c>
       <c r="Y680" t="inlineStr"/>
       <c r="Z680" t="n">
-        <v>7.02556672543679</v>
+        <v>3.602739438414574</v>
       </c>
       <c r="AA680" t="inlineStr">
         <is>
@@ -68329,28 +68329,28 @@
         <v>1</v>
       </c>
       <c r="O681" t="n">
-        <v>0.8036545960024415</v>
+        <v>0.3493945300579071</v>
       </c>
       <c r="P681" t="n">
-        <v>0.1338717363532121</v>
+        <v>0.3345171511173248</v>
       </c>
       <c r="Q681" t="n">
-        <v>0.06247366764434627</v>
+        <v>0.3160882890224457</v>
       </c>
       <c r="R681" t="n">
         <v>1</v>
       </c>
       <c r="S681" t="n">
-        <v>-0.01091176719832521</v>
+        <v>-0.4651718331428596</v>
       </c>
       <c r="T681" t="n">
         <v>1</v>
       </c>
       <c r="U681" t="n">
-        <v>-0.01091176719832521</v>
+        <v>-0.4651718331428596</v>
       </c>
       <c r="V681" t="n">
-        <v>0.8036545960024415</v>
+        <v>0.3493945300579071</v>
       </c>
       <c r="W681" t="n">
         <v>1.17</v>
@@ -68362,7 +68362,7 @@
       </c>
       <c r="Y681" t="inlineStr"/>
       <c r="Z681" t="n">
-        <v>7.980079035695977</v>
+        <v>3.668642565608025</v>
       </c>
       <c r="AA681" t="inlineStr">
         <is>
@@ -68425,34 +68425,34 @@
         <v>0.04967320261437913</v>
       </c>
       <c r="N682" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O682" t="n">
-        <v>0.6382183917849941</v>
+        <v>0.3312021791934967</v>
       </c>
       <c r="P682" t="n">
-        <v>0.1427516307438271</v>
+        <v>0.3346035182476044</v>
       </c>
       <c r="Q682" t="n">
-        <v>0.2190299774711789</v>
+        <v>0.3341943621635437</v>
       </c>
       <c r="R682" t="n">
         <v>1</v>
       </c>
       <c r="S682" t="n">
-        <v>0.1089531364923415</v>
+        <v>0.05440426544561183</v>
       </c>
       <c r="T682" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U682" t="n">
-        <v>0.1089531364923415</v>
+        <v>0.05440426544561183</v>
       </c>
       <c r="V682" t="n">
-        <v>0.6382183917849941</v>
+        <v>0.3346035182476044</v>
       </c>
       <c r="W682" t="n">
-        <v>1.8</v>
+        <v>3.4</v>
       </c>
       <c r="X682" t="inlineStr">
         <is>
@@ -68461,7 +68461,7 @@
       </c>
       <c r="Y682" t="inlineStr"/>
       <c r="Z682" t="n">
-        <v>6.701293113742437</v>
+        <v>3.513336941599846</v>
       </c>
       <c r="AA682" t="inlineStr">
         <is>
@@ -68527,28 +68527,28 @@
         <v>0</v>
       </c>
       <c r="O683" t="n">
-        <v>0.324682485536592</v>
+        <v>0.3099367618560791</v>
       </c>
       <c r="P683" t="n">
-        <v>0.4042483378758187</v>
+        <v>0.3478402495384216</v>
       </c>
       <c r="Q683" t="n">
-        <v>0.2710691765875894</v>
+        <v>0.3422229588031769</v>
       </c>
       <c r="R683" t="n">
         <v>1</v>
       </c>
       <c r="S683" t="n">
-        <v>0.1245873209266661</v>
+        <v>0.06817923258926911</v>
       </c>
       <c r="T683" t="n">
         <v>0</v>
       </c>
       <c r="U683" t="n">
-        <v>0.1245873209266661</v>
+        <v>0.06817923258926911</v>
       </c>
       <c r="V683" t="n">
-        <v>0.4042483378758187</v>
+        <v>0.3478402495384216</v>
       </c>
       <c r="W683" t="n">
         <v>3.4</v>
@@ -68560,7 +68560,7 @@
       </c>
       <c r="Y683" t="inlineStr"/>
       <c r="Z683" t="n">
-        <v>3.183455660772072</v>
+        <v>2.73924196511507</v>
       </c>
       <c r="AA683" t="inlineStr">
         <is>
@@ -68604,55 +68604,55 @@
         <v>1481</v>
       </c>
       <c r="G684" t="n">
-        <v>5.75</v>
+        <v>6</v>
       </c>
       <c r="H684" t="n">
-        <v>4.1</v>
+        <v>4.2</v>
       </c>
       <c r="I684" t="n">
-        <v>1.57</v>
+        <v>1.53</v>
       </c>
       <c r="J684" t="n">
-        <v>0.1648842838663405</v>
+        <v>0.1574768416409351</v>
       </c>
       <c r="K684" t="n">
-        <v>0.2312401542027946</v>
+        <v>0.2249669166299073</v>
       </c>
       <c r="L684" t="n">
-        <v>0.6038755619308649</v>
+        <v>0.6175562417291575</v>
       </c>
       <c r="M684" t="n">
-        <v>0.05475815766188674</v>
+        <v>0.05835667600373484</v>
       </c>
       <c r="N684" t="n">
         <v>2</v>
       </c>
       <c r="O684" t="n">
-        <v>0.1009777218165367</v>
+        <v>0.3339175879955292</v>
       </c>
       <c r="P684" t="n">
-        <v>0.2313452870418226</v>
+        <v>0.3184289336204529</v>
       </c>
       <c r="Q684" t="n">
-        <v>0.6676769911416407</v>
+        <v>0.3476535081863403</v>
       </c>
       <c r="R684" t="n">
         <v>1</v>
       </c>
       <c r="S684" t="n">
-        <v>0.06380142921077581</v>
+        <v>-0.2699027335428171</v>
       </c>
       <c r="T684" t="n">
         <v>2</v>
       </c>
       <c r="U684" t="n">
-        <v>0.06380142921077581</v>
+        <v>-0.2699027335428171</v>
       </c>
       <c r="V684" t="n">
-        <v>0.6676769911416407</v>
+        <v>0.3476535081863403</v>
       </c>
       <c r="W684" t="n">
-        <v>1.57</v>
+        <v>1.53</v>
       </c>
       <c r="X684" t="inlineStr">
         <is>
@@ -68661,7 +68661,7 @@
       </c>
       <c r="Y684" t="inlineStr"/>
       <c r="Z684" t="n">
-        <v>7.010608406987227</v>
+        <v>3.650361835956573</v>
       </c>
       <c r="AA684" t="inlineStr">
         <is>
@@ -68727,28 +68727,28 @@
         <v>1</v>
       </c>
       <c r="O685" t="n">
-        <v>0.507582859485448</v>
+        <v>0.3452942371368408</v>
       </c>
       <c r="P685" t="n">
-        <v>0.2727172214745165</v>
+        <v>0.342877984046936</v>
       </c>
       <c r="Q685" t="n">
-        <v>0.2196999190400354</v>
+        <v>0.3118277788162231</v>
       </c>
       <c r="R685" t="n">
         <v>1</v>
       </c>
       <c r="S685" t="n">
-        <v>-0.01046894569507006</v>
+        <v>-0.1727575680436773</v>
       </c>
       <c r="T685" t="n">
         <v>1</v>
       </c>
       <c r="U685" t="n">
-        <v>-0.01046894569507006</v>
+        <v>-0.1727575680436773</v>
       </c>
       <c r="V685" t="n">
-        <v>0.507582859485448</v>
+        <v>0.3452942371368408</v>
       </c>
       <c r="W685" t="n">
         <v>1.83</v>
@@ -68760,7 +68760,7 @@
       </c>
       <c r="Y685" t="inlineStr"/>
       <c r="Z685" t="n">
-        <v>4.889924305404262</v>
+        <v>3.625589489936829</v>
       </c>
       <c r="AA685" t="inlineStr">
         <is>
@@ -68805,49 +68805,49 @@
         <v>1.36</v>
       </c>
       <c r="H686" t="n">
-        <v>5</v>
+        <v>4.5</v>
       </c>
       <c r="I686" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="J686" t="n">
-        <v>0.6934812760055478</v>
+        <v>0.6953028430160691</v>
       </c>
       <c r="K686" t="n">
-        <v>0.188626907073509</v>
+        <v>0.2101359703337453</v>
       </c>
       <c r="L686" t="n">
-        <v>0.1178918169209431</v>
+        <v>0.09456118665018541</v>
       </c>
       <c r="M686" t="n">
-        <v>0.06029411764705883</v>
+        <v>0.05751633986928106</v>
       </c>
       <c r="N686" t="n">
         <v>1</v>
       </c>
       <c r="O686" t="n">
-        <v>0.8451646071692897</v>
+        <v>0.3507839739322662</v>
       </c>
       <c r="P686" t="n">
-        <v>0.07771171929663059</v>
+        <v>0.3240694105625153</v>
       </c>
       <c r="Q686" t="n">
-        <v>0.07712367353407977</v>
+        <v>0.3251466155052185</v>
       </c>
       <c r="R686" t="n">
         <v>1</v>
       </c>
       <c r="S686" t="n">
-        <v>0.1516833311637419</v>
+        <v>-0.3445188690838029</v>
       </c>
       <c r="T686" t="n">
         <v>1</v>
       </c>
       <c r="U686" t="n">
-        <v>0.1516833311637419</v>
+        <v>-0.3445188690838029</v>
       </c>
       <c r="V686" t="n">
-        <v>0.8451646071692897</v>
+        <v>0.3507839739322662</v>
       </c>
       <c r="W686" t="n">
         <v>1.36</v>
@@ -68859,7 +68859,7 @@
       </c>
       <c r="Y686" t="inlineStr"/>
       <c r="Z686" t="n">
-        <v>8.874228375277541</v>
+        <v>3.683231726288795</v>
       </c>
       <c r="AA686" t="inlineStr">
         <is>
@@ -68922,34 +68922,34 @@
         <v>0.05009387267451793</v>
       </c>
       <c r="N687" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O687" t="n">
-        <v>0.305886745942742</v>
+        <v>0.3466003835201263</v>
       </c>
       <c r="P687" t="n">
-        <v>0.1593788878408367</v>
+        <v>0.3370699882507324</v>
       </c>
       <c r="Q687" t="n">
-        <v>0.5347343662164213</v>
+        <v>0.3163296282291412</v>
       </c>
       <c r="R687" t="n">
         <v>1</v>
       </c>
       <c r="S687" t="n">
-        <v>0.1820322126203223</v>
+        <v>0.006494735409602215</v>
       </c>
       <c r="T687" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U687" t="n">
-        <v>0.1820322126203223</v>
+        <v>0.006494735409602215</v>
       </c>
       <c r="V687" t="n">
-        <v>0.5347343662164213</v>
+        <v>0.3466003835201263</v>
       </c>
       <c r="W687" t="n">
-        <v>2.7</v>
+        <v>2.8</v>
       </c>
       <c r="X687" t="inlineStr">
         <is>
@@ -68958,7 +68958,7 @@
       </c>
       <c r="Y687" t="inlineStr"/>
       <c r="Z687" t="n">
-        <v>5.614710845272424</v>
+        <v>3.639304026961327</v>
       </c>
       <c r="AA687" t="inlineStr">
         <is>
@@ -69000,55 +69000,55 @@
         <v>1481</v>
       </c>
       <c r="G688" t="n">
-        <v>1.75</v>
+        <v>1.8</v>
       </c>
       <c r="H688" t="n">
         <v>3.6</v>
       </c>
       <c r="I688" t="n">
-        <v>4.75</v>
+        <v>4.5</v>
       </c>
       <c r="J688" t="n">
-        <v>0.5392195506503745</v>
+        <v>0.5263157894736842</v>
       </c>
       <c r="K688" t="n">
-        <v>0.2621206148994876</v>
+        <v>0.2631578947368421</v>
       </c>
       <c r="L688" t="n">
-        <v>0.198659834450138</v>
+        <v>0.2105263157894737</v>
       </c>
       <c r="M688" t="n">
-        <v>0.05973266499582275</v>
+        <v>0.05555555555555558</v>
       </c>
       <c r="N688" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O688" t="n">
-        <v>0.3471487420816711</v>
+        <v>0.3296301364898682</v>
       </c>
       <c r="P688" t="n">
-        <v>0.3416191168279354</v>
+        <v>0.326541393995285</v>
       </c>
       <c r="Q688" t="n">
-        <v>0.3112321410903934</v>
+        <v>0.3438284695148468</v>
       </c>
       <c r="R688" t="n">
         <v>1</v>
       </c>
       <c r="S688" t="n">
-        <v>-0.1920708085687034</v>
+        <v>0.1333021537253731</v>
       </c>
       <c r="T688" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U688" t="n">
-        <v>-0.1920708085687034</v>
+        <v>0.1333021537253731</v>
       </c>
       <c r="V688" t="n">
-        <v>0.3471487420816711</v>
+        <v>0.3438284695148468</v>
       </c>
       <c r="W688" t="n">
-        <v>1.75</v>
+        <v>4.5</v>
       </c>
       <c r="X688" t="inlineStr">
         <is>
@@ -69057,7 +69057,7 @@
       </c>
       <c r="Y688" t="inlineStr"/>
       <c r="Z688" t="n">
-        <v>0</v>
+        <v>2.707649197429419</v>
       </c>
       <c r="AA688" t="inlineStr">
         <is>
@@ -69125,28 +69125,28 @@
         <v>1</v>
       </c>
       <c r="O689" t="n">
-        <v>0.5748051679220132</v>
+        <v>0.3555161952972412</v>
       </c>
       <c r="P689" t="n">
-        <v>0.142279117365902</v>
+        <v>0.3192315399646759</v>
       </c>
       <c r="Q689" t="n">
-        <v>0.2829157147120847</v>
+        <v>0.3252522349357605</v>
       </c>
       <c r="R689" t="n">
         <v>1</v>
       </c>
       <c r="S689" t="n">
-        <v>0.1238767859591484</v>
+        <v>-0.09541218666562357</v>
       </c>
       <c r="T689" t="n">
         <v>1</v>
       </c>
       <c r="U689" t="n">
-        <v>0.1238767859591484</v>
+        <v>-0.09541218666562357</v>
       </c>
       <c r="V689" t="n">
-        <v>0.5748051679220132</v>
+        <v>0.3555161952972412</v>
       </c>
       <c r="W689" t="n">
         <v>2.1</v>
@@ -69158,7 +69158,7 @@
       </c>
       <c r="Y689" t="inlineStr"/>
       <c r="Z689" t="n">
-        <v>4.526590697385855</v>
+        <v>2.799690037965775</v>
       </c>
       <c r="AA689" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
DATA. Actualizo predicciones x cambio de modelo en SPA
</commit_message>
<xml_diff>
--- a/data/historial_predicciones.xlsx
+++ b/data/historial_predicciones.xlsx
@@ -68230,40 +68230,40 @@
         <v>1</v>
       </c>
       <c r="O680" t="n">
-        <v>0.3431180417537689</v>
+        <v>0.6148039698600769</v>
       </c>
       <c r="P680" t="n">
-        <v>0.3292394876480103</v>
+        <v>0.2291441261768341</v>
       </c>
       <c r="Q680" t="n">
-        <v>0.3276424705982208</v>
+        <v>0.1560518741607666</v>
       </c>
       <c r="R680" t="n">
         <v>1</v>
       </c>
       <c r="S680" t="n">
-        <v>-0.130566168772547</v>
+        <v>0.141119759333761</v>
       </c>
       <c r="T680" t="n">
         <v>1</v>
       </c>
       <c r="U680" t="n">
-        <v>-0.130566168772547</v>
+        <v>0.141119759333761</v>
       </c>
       <c r="V680" t="n">
-        <v>0.3431180417537689</v>
+        <v>0.6148039698600769</v>
       </c>
       <c r="W680" t="n">
         <v>2</v>
       </c>
       <c r="X680" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.5</t>
+          <t>dif_prob_mod_bm &gt; -0.25</t>
         </is>
       </c>
       <c r="Y680" t="inlineStr"/>
       <c r="Z680" t="n">
-        <v>3.602739438414574</v>
+        <v>6.455441683530807</v>
       </c>
       <c r="AA680" t="inlineStr">
         <is>
@@ -68329,40 +68329,40 @@
         <v>1</v>
       </c>
       <c r="O681" t="n">
-        <v>0.3493945300579071</v>
+        <v>0.6315798163414001</v>
       </c>
       <c r="P681" t="n">
-        <v>0.3345171511173248</v>
+        <v>0.2134162187576294</v>
       </c>
       <c r="Q681" t="n">
-        <v>0.3160882890224457</v>
+        <v>0.1550039499998093</v>
       </c>
       <c r="R681" t="n">
         <v>1</v>
       </c>
       <c r="S681" t="n">
-        <v>-0.4651718331428596</v>
+        <v>-0.1829865468593666</v>
       </c>
       <c r="T681" t="n">
         <v>1</v>
       </c>
       <c r="U681" t="n">
-        <v>-0.4651718331428596</v>
+        <v>-0.1829865468593666</v>
       </c>
       <c r="V681" t="n">
-        <v>0.3493945300579071</v>
+        <v>0.6315798163414001</v>
       </c>
       <c r="W681" t="n">
         <v>1.17</v>
       </c>
       <c r="X681" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.5</t>
+          <t>dif_prob_mod_bm &gt; -0.25</t>
         </is>
       </c>
       <c r="Y681" t="inlineStr"/>
       <c r="Z681" t="n">
-        <v>3.668642565608025</v>
+        <v>6.631588071584702</v>
       </c>
       <c r="AA681" t="inlineStr">
         <is>
@@ -68428,40 +68428,40 @@
         <v>0</v>
       </c>
       <c r="O682" t="n">
-        <v>0.3312021791934967</v>
+        <v>0.2924555242061615</v>
       </c>
       <c r="P682" t="n">
-        <v>0.3346035182476044</v>
+        <v>0.3657283782958984</v>
       </c>
       <c r="Q682" t="n">
-        <v>0.3341943621635437</v>
+        <v>0.3418160378932953</v>
       </c>
       <c r="R682" t="n">
         <v>1</v>
       </c>
       <c r="S682" t="n">
-        <v>0.05440426544561183</v>
+        <v>0.0855291254939059</v>
       </c>
       <c r="T682" t="n">
         <v>0</v>
       </c>
       <c r="U682" t="n">
-        <v>0.05440426544561183</v>
+        <v>0.0855291254939059</v>
       </c>
       <c r="V682" t="n">
-        <v>0.3346035182476044</v>
+        <v>0.3657283782958984</v>
       </c>
       <c r="W682" t="n">
         <v>3.4</v>
       </c>
       <c r="X682" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.5</t>
+          <t>dif_prob_mod_bm &gt; -0.25</t>
         </is>
       </c>
       <c r="Y682" t="inlineStr"/>
       <c r="Z682" t="n">
-        <v>3.513336941599846</v>
+        <v>3.840147972106934</v>
       </c>
       <c r="AA682" t="inlineStr">
         <is>
@@ -68524,43 +68524,43 @@
         <v>0.05169340463458116</v>
       </c>
       <c r="N683" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O683" t="n">
-        <v>0.3099367618560791</v>
+        <v>0.110199049115181</v>
       </c>
       <c r="P683" t="n">
-        <v>0.3478402495384216</v>
+        <v>0.2768021821975708</v>
       </c>
       <c r="Q683" t="n">
-        <v>0.3422229588031769</v>
+        <v>0.6129987239837646</v>
       </c>
       <c r="R683" t="n">
         <v>1</v>
       </c>
       <c r="S683" t="n">
-        <v>0.06817923258926911</v>
+        <v>0.1807953341532562</v>
       </c>
       <c r="T683" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="U683" t="n">
-        <v>0.06817923258926911</v>
+        <v>0.1807953341532562</v>
       </c>
       <c r="V683" t="n">
-        <v>0.3478402495384216</v>
+        <v>0.6129987239837646</v>
       </c>
       <c r="W683" t="n">
-        <v>3.4</v>
+        <v>2.2</v>
       </c>
       <c r="X683" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.5</t>
+          <t>dif_prob_mod_bm &gt; -0.25</t>
         </is>
       </c>
       <c r="Y683" t="inlineStr"/>
       <c r="Z683" t="n">
-        <v>2.73924196511507</v>
+        <v>4.827364951372147</v>
       </c>
       <c r="AA683" t="inlineStr">
         <is>
@@ -68628,40 +68628,40 @@
         <v>2</v>
       </c>
       <c r="O684" t="n">
-        <v>0.3339175879955292</v>
+        <v>0.09451180696487427</v>
       </c>
       <c r="P684" t="n">
-        <v>0.3184289336204529</v>
+        <v>0.2090925276279449</v>
       </c>
       <c r="Q684" t="n">
-        <v>0.3476535081863403</v>
+        <v>0.6963956356048584</v>
       </c>
       <c r="R684" t="n">
         <v>1</v>
       </c>
       <c r="S684" t="n">
-        <v>-0.2699027335428171</v>
+        <v>0.07883939387570094</v>
       </c>
       <c r="T684" t="n">
         <v>2</v>
       </c>
       <c r="U684" t="n">
-        <v>-0.2699027335428171</v>
+        <v>0.07883939387570094</v>
       </c>
       <c r="V684" t="n">
-        <v>0.3476535081863403</v>
+        <v>0.6963956356048584</v>
       </c>
       <c r="W684" t="n">
         <v>1.53</v>
       </c>
       <c r="X684" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.5</t>
+          <t>dif_prob_mod_bm &gt; -0.25</t>
         </is>
       </c>
       <c r="Y684" t="inlineStr"/>
       <c r="Z684" t="n">
-        <v>3.650361835956573</v>
+        <v>7.312154173851013</v>
       </c>
       <c r="AA684" t="inlineStr">
         <is>
@@ -68724,43 +68724,43 @@
         <v>0.05481359579720224</v>
       </c>
       <c r="N685" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O685" t="n">
-        <v>0.3452942371368408</v>
+        <v>0.1948871463537216</v>
       </c>
       <c r="P685" t="n">
-        <v>0.342877984046936</v>
+        <v>0.1989489793777466</v>
       </c>
       <c r="Q685" t="n">
-        <v>0.3118277788162231</v>
+        <v>0.6061638593673706</v>
       </c>
       <c r="R685" t="n">
         <v>1</v>
       </c>
       <c r="S685" t="n">
-        <v>-0.1727575680436773</v>
+        <v>0.3804412871101449</v>
       </c>
       <c r="T685" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U685" t="n">
-        <v>-0.1727575680436773</v>
+        <v>0.3804412871101449</v>
       </c>
       <c r="V685" t="n">
-        <v>0.3452942371368408</v>
+        <v>0.6061638593673706</v>
       </c>
       <c r="W685" t="n">
-        <v>1.83</v>
+        <v>4.2</v>
       </c>
       <c r="X685" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.5</t>
+          <t>dif_prob_mod_bm &gt; -0.25</t>
         </is>
       </c>
       <c r="Y685" t="inlineStr"/>
       <c r="Z685" t="n">
-        <v>3.625589489936829</v>
+        <v>6.364720523357391</v>
       </c>
       <c r="AA685" t="inlineStr">
         <is>
@@ -68826,40 +68826,40 @@
         <v>1</v>
       </c>
       <c r="O686" t="n">
-        <v>0.3507839739322662</v>
+        <v>0.5046667456626892</v>
       </c>
       <c r="P686" t="n">
-        <v>0.3240694105625153</v>
+        <v>0.3227453529834747</v>
       </c>
       <c r="Q686" t="n">
-        <v>0.3251466155052185</v>
+        <v>0.1725879162549973</v>
       </c>
       <c r="R686" t="n">
         <v>1</v>
       </c>
       <c r="S686" t="n">
-        <v>-0.3445188690838029</v>
+        <v>-0.1906360973533799</v>
       </c>
       <c r="T686" t="n">
         <v>1</v>
       </c>
       <c r="U686" t="n">
-        <v>-0.3445188690838029</v>
+        <v>-0.1906360973533799</v>
       </c>
       <c r="V686" t="n">
-        <v>0.3507839739322662</v>
+        <v>0.5046667456626892</v>
       </c>
       <c r="W686" t="n">
         <v>1.36</v>
       </c>
       <c r="X686" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.5</t>
+          <t>dif_prob_mod_bm &gt; -0.25</t>
         </is>
       </c>
       <c r="Y686" t="inlineStr"/>
       <c r="Z686" t="n">
-        <v>3.683231726288795</v>
+        <v>5.299000829458237</v>
       </c>
       <c r="AA686" t="inlineStr">
         <is>
@@ -68922,43 +68922,43 @@
         <v>0.05009387267451793</v>
       </c>
       <c r="N687" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O687" t="n">
-        <v>0.3466003835201263</v>
+        <v>0.1954513341188431</v>
       </c>
       <c r="P687" t="n">
-        <v>0.3370699882507324</v>
+        <v>0.4579564332962036</v>
       </c>
       <c r="Q687" t="n">
-        <v>0.3163296282291412</v>
+        <v>0.3465921580791473</v>
       </c>
       <c r="R687" t="n">
         <v>1</v>
       </c>
       <c r="S687" t="n">
-        <v>0.006494735409602215</v>
+        <v>0.150764235002827</v>
       </c>
       <c r="T687" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U687" t="n">
-        <v>0.006494735409602215</v>
+        <v>0.150764235002827</v>
       </c>
       <c r="V687" t="n">
-        <v>0.3466003835201263</v>
+        <v>0.4579564332962036</v>
       </c>
       <c r="W687" t="n">
-        <v>2.8</v>
+        <v>3.1</v>
       </c>
       <c r="X687" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.5</t>
+          <t>dif_prob_mod_bm &gt; -0.25</t>
         </is>
       </c>
       <c r="Y687" t="inlineStr"/>
       <c r="Z687" t="n">
-        <v>3.639304026961327</v>
+        <v>4.808542549610138</v>
       </c>
       <c r="AA687" t="inlineStr">
         <is>
@@ -69021,43 +69021,43 @@
         <v>0.05555555555555558</v>
       </c>
       <c r="N688" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O688" t="n">
-        <v>0.3296301364898682</v>
+        <v>0.2176385521888733</v>
       </c>
       <c r="P688" t="n">
-        <v>0.326541393995285</v>
+        <v>0.4210319221019745</v>
       </c>
       <c r="Q688" t="n">
-        <v>0.3438284695148468</v>
+        <v>0.3613295257091522</v>
       </c>
       <c r="R688" t="n">
         <v>1</v>
       </c>
       <c r="S688" t="n">
-        <v>0.1333021537253731</v>
+        <v>0.1578740273651324</v>
       </c>
       <c r="T688" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="U688" t="n">
-        <v>0.1333021537253731</v>
+        <v>0.1578740273651324</v>
       </c>
       <c r="V688" t="n">
-        <v>0.3438284695148468</v>
+        <v>0.4210319221019745</v>
       </c>
       <c r="W688" t="n">
-        <v>4.5</v>
+        <v>3.6</v>
       </c>
       <c r="X688" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.5</t>
+          <t>dif_prob_mod_bm &gt; -0.25</t>
         </is>
       </c>
       <c r="Y688" t="inlineStr"/>
       <c r="Z688" t="n">
-        <v>2.707649197429419</v>
+        <v>3.315626386553049</v>
       </c>
       <c r="AA688" t="inlineStr">
         <is>
@@ -69125,40 +69125,40 @@
         <v>1</v>
       </c>
       <c r="O689" t="n">
-        <v>0.3555161952972412</v>
+        <v>0.4133053123950958</v>
       </c>
       <c r="P689" t="n">
-        <v>0.3192315399646759</v>
+        <v>0.2662601470947266</v>
       </c>
       <c r="Q689" t="n">
-        <v>0.3252522349357605</v>
+        <v>0.3204345703125</v>
       </c>
       <c r="R689" t="n">
         <v>1</v>
       </c>
       <c r="S689" t="n">
-        <v>-0.09541218666562357</v>
+        <v>-0.03762306956776895</v>
       </c>
       <c r="T689" t="n">
         <v>1</v>
       </c>
       <c r="U689" t="n">
-        <v>-0.09541218666562357</v>
+        <v>-0.03762306956776895</v>
       </c>
       <c r="V689" t="n">
-        <v>0.3555161952972412</v>
+        <v>0.4133053123950958</v>
       </c>
       <c r="W689" t="n">
         <v>2.1</v>
       </c>
       <c r="X689" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.5</t>
+          <t>dif_prob_mod_bm &gt; -0.25</t>
         </is>
       </c>
       <c r="Y689" t="inlineStr"/>
       <c r="Z689" t="n">
-        <v>2.799690037965775</v>
+        <v>3.25477933511138</v>
       </c>
       <c r="AA689" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
DATA. Actualizo predicciones por cambio de modelo tras darle mas peso a Expected roi en la seleccion.
</commit_message>
<xml_diff>
--- a/data/historial_predicciones.xlsx
+++ b/data/historial_predicciones.xlsx
@@ -79727,28 +79727,28 @@
         <v>1</v>
       </c>
       <c r="O785" t="n">
-        <v>0.5092289941108454</v>
+        <v>0.4163012859071499</v>
       </c>
       <c r="P785" t="n">
-        <v>0.3414846270280875</v>
+        <v>0.3850638745611724</v>
       </c>
       <c r="Q785" t="n">
-        <v>0.1492863788610669</v>
+        <v>0.1986348395316778</v>
       </c>
       <c r="R785" t="n">
         <v>1</v>
       </c>
       <c r="S785" t="n">
-        <v>-0.07379795538330236</v>
+        <v>-0.1667256635869979</v>
       </c>
       <c r="T785" t="n">
         <v>1</v>
       </c>
       <c r="U785" t="n">
-        <v>-0.07379795538330236</v>
+        <v>-0.1667256635869979</v>
       </c>
       <c r="V785" t="n">
-        <v>0.5092289941108454</v>
+        <v>0.4163012859071499</v>
       </c>
       <c r="W785" t="n">
         <v>1.62</v>
@@ -79760,7 +79760,7 @@
       </c>
       <c r="Y785" t="inlineStr"/>
       <c r="Z785" t="n">
-        <v>5.346904438163877</v>
+        <v>1.871817167401141</v>
       </c>
       <c r="AA785" t="inlineStr">
         <is>
@@ -79827,28 +79827,28 @@
         <v>1</v>
       </c>
       <c r="O786" t="n">
-        <v>0.7025689275723888</v>
+        <v>0.7780799390283771</v>
       </c>
       <c r="P786" t="n">
-        <v>0.2802401381886497</v>
+        <v>0.1513442600050631</v>
       </c>
       <c r="Q786" t="n">
-        <v>0.01719093423896149</v>
+        <v>0.07057580096655983</v>
       </c>
       <c r="R786" t="n">
         <v>1</v>
       </c>
       <c r="S786" t="n">
-        <v>-0.1289166600107597</v>
+        <v>-0.05340564855477137</v>
       </c>
       <c r="T786" t="n">
         <v>1</v>
       </c>
       <c r="U786" t="n">
-        <v>-0.1289166600107597</v>
+        <v>-0.05340564855477137</v>
       </c>
       <c r="V786" t="n">
-        <v>0.7025689275723888</v>
+        <v>0.7780799390283771</v>
       </c>
       <c r="W786" t="n">
         <v>1.14</v>
@@ -79860,7 +79860,7 @@
       </c>
       <c r="Y786" t="inlineStr"/>
       <c r="Z786" t="n">
-        <v>7.376973739510082</v>
+        <v>5.435057178552043</v>
       </c>
       <c r="AA786" t="inlineStr">
         <is>
@@ -79931,28 +79931,28 @@
         <v>2</v>
       </c>
       <c r="O787" t="n">
-        <v>0.04634760893189991</v>
+        <v>0.09547139052459465</v>
       </c>
       <c r="P787" t="n">
-        <v>0.2122972311087638</v>
+        <v>0.1754970829918797</v>
       </c>
       <c r="Q787" t="n">
-        <v>0.7413551599593363</v>
+        <v>0.7290315264835258</v>
       </c>
       <c r="R787" t="n">
         <v>1</v>
       </c>
       <c r="S787" t="n">
-        <v>0.04137212924492939</v>
+        <v>0.02904849576911883</v>
       </c>
       <c r="T787" t="n">
         <v>2</v>
       </c>
       <c r="U787" t="n">
-        <v>0.04137212924492939</v>
+        <v>0.02904849576911883</v>
       </c>
       <c r="V787" t="n">
-        <v>0.7413551599593363</v>
+        <v>0.7290315264835258</v>
       </c>
       <c r="W787" t="n">
         <v>1.36</v>
@@ -79964,7 +79964,7 @@
       </c>
       <c r="Y787" t="inlineStr"/>
       <c r="Z787" t="n">
-        <v>7.784229179573031</v>
+        <v>5.685600166894835</v>
       </c>
       <c r="AA787" t="inlineStr">
         <is>
@@ -80031,28 +80031,28 @@
         <v>1</v>
       </c>
       <c r="O788" t="n">
-        <v>0.5446225841843005</v>
+        <v>0.7096095262326643</v>
       </c>
       <c r="P788" t="n">
-        <v>0.4193477977611727</v>
+        <v>0.222129545517187</v>
       </c>
       <c r="Q788" t="n">
-        <v>0.03602961805452683</v>
+        <v>0.06826092825014872</v>
       </c>
       <c r="R788" t="n">
         <v>1</v>
       </c>
       <c r="S788" t="n">
-        <v>-0.04778793282851423</v>
+        <v>0.1171990092198495</v>
       </c>
       <c r="T788" t="n">
         <v>1</v>
       </c>
       <c r="U788" t="n">
-        <v>-0.04778793282851423</v>
+        <v>0.1171990092198495</v>
       </c>
       <c r="V788" t="n">
-        <v>0.5446225841843005</v>
+        <v>0.7096095262326643</v>
       </c>
       <c r="W788" t="n">
         <v>1.57</v>
@@ -80064,7 +80064,7 @@
       </c>
       <c r="Y788" t="inlineStr"/>
       <c r="Z788" t="n">
-        <v>5.718537133935156</v>
+        <v>6.201064015893853</v>
       </c>
       <c r="AA788" t="inlineStr">
         <is>
@@ -80128,34 +80128,34 @@
         <v>0.05425824175824179</v>
       </c>
       <c r="N789" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O789" t="n">
-        <v>0.5244677610413325</v>
+        <v>0.3147015210197008</v>
       </c>
       <c r="P789" t="n">
-        <v>0.1935739139150954</v>
+        <v>0.4014903592486138</v>
       </c>
       <c r="Q789" t="n">
-        <v>0.2819583250435722</v>
+        <v>0.2838081197316854</v>
       </c>
       <c r="R789" t="n">
         <v>1</v>
       </c>
       <c r="S789" t="n">
-        <v>0.1596469141357951</v>
+        <v>0.1050734211378646</v>
       </c>
       <c r="T789" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U789" t="n">
-        <v>0.1596469141357951</v>
+        <v>0.1050734211378646</v>
       </c>
       <c r="V789" t="n">
-        <v>0.5244677610413325</v>
+        <v>0.4014903592486138</v>
       </c>
       <c r="W789" t="n">
-        <v>2.6</v>
+        <v>3.2</v>
       </c>
       <c r="X789" t="inlineStr">
         <is>
@@ -80164,7 +80164,7 @@
       </c>
       <c r="Y789" t="inlineStr"/>
       <c r="Z789" t="n">
-        <v>5.506911490933992</v>
+        <v>3.799228352898588</v>
       </c>
       <c r="AA789" t="inlineStr">
         <is>
@@ -80231,28 +80231,28 @@
         <v>0</v>
       </c>
       <c r="O790" t="n">
-        <v>0.2842865130944872</v>
+        <v>0.2500598330532756</v>
       </c>
       <c r="P790" t="n">
-        <v>0.4501632853253706</v>
+        <v>0.3877105036058738</v>
       </c>
       <c r="Q790" t="n">
-        <v>0.2655502015801422</v>
+        <v>0.3622296633408508</v>
       </c>
       <c r="R790" t="n">
         <v>1</v>
       </c>
       <c r="S790" t="n">
-        <v>0.1880550232171085</v>
+        <v>0.1256022414976117</v>
       </c>
       <c r="T790" t="n">
         <v>0</v>
       </c>
       <c r="U790" t="n">
-        <v>0.1880550232171085</v>
+        <v>0.1256022414976117</v>
       </c>
       <c r="V790" t="n">
-        <v>0.4501632853253706</v>
+        <v>0.3877105036058738</v>
       </c>
       <c r="W790" t="n">
         <v>3.6</v>
@@ -80264,7 +80264,7 @@
       </c>
       <c r="Y790" t="inlineStr"/>
       <c r="Z790" t="n">
-        <v>4.726714495916391</v>
+        <v>3.849845588276141</v>
       </c>
       <c r="AA790" t="inlineStr">
         <is>
@@ -80331,28 +80331,28 @@
         <v>0</v>
       </c>
       <c r="O791" t="n">
-        <v>0.1308736546210394</v>
+        <v>0.2340053671405052</v>
       </c>
       <c r="P791" t="n">
-        <v>0.4790865081691381</v>
+        <v>0.614419936587252</v>
       </c>
       <c r="Q791" t="n">
-        <v>0.3900398372098225</v>
+        <v>0.1515746962722427</v>
       </c>
       <c r="R791" t="n">
         <v>1</v>
       </c>
       <c r="S791" t="n">
-        <v>0.2909566089530127</v>
+        <v>0.4262900373711266</v>
       </c>
       <c r="T791" t="n">
         <v>0</v>
       </c>
       <c r="U791" t="n">
-        <v>0.2909566089530127</v>
+        <v>0.4262900373711266</v>
       </c>
       <c r="V791" t="n">
-        <v>0.4790865081691381</v>
+        <v>0.614419936587252</v>
       </c>
       <c r="W791" t="n">
         <v>5</v>
@@ -80364,7 +80364,7 @@
       </c>
       <c r="Y791" t="inlineStr"/>
       <c r="Z791" t="n">
-        <v>5.030408335775951</v>
+        <v>7.805324804687839</v>
       </c>
       <c r="AA791" t="inlineStr">
         <is>
@@ -80431,28 +80431,28 @@
         <v>2</v>
       </c>
       <c r="O792" t="n">
-        <v>0.1044436757554368</v>
+        <v>0.1503662772130578</v>
       </c>
       <c r="P792" t="n">
-        <v>0.2410643244711771</v>
+        <v>0.3163356959020147</v>
       </c>
       <c r="Q792" t="n">
-        <v>0.6544919997733862</v>
+        <v>0.5332980268849274</v>
       </c>
       <c r="R792" t="n">
         <v>1</v>
       </c>
       <c r="S792" t="n">
-        <v>-0.02118367590228942</v>
+        <v>-0.1423776487907482</v>
       </c>
       <c r="T792" t="n">
         <v>2</v>
       </c>
       <c r="U792" t="n">
-        <v>-0.02118367590228942</v>
+        <v>-0.1423776487907482</v>
       </c>
       <c r="V792" t="n">
-        <v>0.6544919997733862</v>
+        <v>0.5332980268849274</v>
       </c>
       <c r="W792" t="n">
         <v>1.4</v>
@@ -80464,7 +80464,7 @@
       </c>
       <c r="Y792" t="inlineStr"/>
       <c r="Z792" t="n">
-        <v>6.872165997620556</v>
+        <v>2.931902835706344</v>
       </c>
       <c r="AA792" t="inlineStr">
         <is>
@@ -80528,34 +80528,34 @@
         <v>0.06725146198830423</v>
       </c>
       <c r="N793" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O793" t="n">
-        <v>0.42463767222677</v>
+        <v>0.668828536322369</v>
       </c>
       <c r="P793" t="n">
-        <v>0.4537419782296451</v>
+        <v>0.2421892560983642</v>
       </c>
       <c r="Q793" t="n">
-        <v>0.1216203495435848</v>
+        <v>0.08898220757926678</v>
       </c>
       <c r="R793" t="n">
         <v>1</v>
       </c>
       <c r="S793" t="n">
-        <v>0.2071666357638917</v>
+        <v>0.1756778513908623</v>
       </c>
       <c r="T793" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U793" t="n">
-        <v>0.2071666357638917</v>
+        <v>0.1756778513908623</v>
       </c>
       <c r="V793" t="n">
-        <v>0.4537419782296451</v>
+        <v>0.668828536322369</v>
       </c>
       <c r="W793" t="n">
-        <v>3.8</v>
+        <v>1.9</v>
       </c>
       <c r="X793" t="inlineStr">
         <is>
@@ -80564,7 +80564,7 @@
       </c>
       <c r="Y793" t="inlineStr"/>
       <c r="Z793" t="n">
-        <v>4.764290771411273</v>
+        <v>6.333797907849235</v>
       </c>
       <c r="AA793" t="inlineStr">
         <is>
@@ -80631,28 +80631,28 @@
         <v>2</v>
       </c>
       <c r="O794" t="n">
-        <v>0.08728969824916612</v>
+        <v>0.0783645521969986</v>
       </c>
       <c r="P794" t="n">
-        <v>0.2486876408615044</v>
+        <v>0.3616600723770544</v>
       </c>
       <c r="Q794" t="n">
-        <v>0.6640226608893294</v>
+        <v>0.559975375425947</v>
       </c>
       <c r="R794" t="n">
         <v>1</v>
       </c>
       <c r="S794" t="n">
-        <v>0.005004517879724224</v>
+        <v>-0.09904276758365815</v>
       </c>
       <c r="T794" t="n">
         <v>2</v>
       </c>
       <c r="U794" t="n">
-        <v>0.005004517879724224</v>
+        <v>-0.09904276758365815</v>
       </c>
       <c r="V794" t="n">
-        <v>0.6640226608893294</v>
+        <v>0.559975375425947</v>
       </c>
       <c r="W794" t="n">
         <v>1.42</v>
@@ -80664,7 +80664,7 @@
       </c>
       <c r="Y794" t="inlineStr"/>
       <c r="Z794" t="n">
-        <v>6.972237939337958</v>
+        <v>3.456994558817166</v>
       </c>
       <c r="AA794" t="inlineStr">
         <is>
@@ -80728,34 +80728,34 @@
         <v>0.04150751209574732</v>
       </c>
       <c r="N795" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O795" t="n">
-        <v>0.3738123863679146</v>
+        <v>0.4150379231667436</v>
       </c>
       <c r="P795" t="n">
-        <v>0.222207514482362</v>
+        <v>0.390098775667103</v>
       </c>
       <c r="Q795" t="n">
-        <v>0.4039800991497235</v>
+        <v>0.1948633011661534</v>
       </c>
       <c r="R795" t="n">
         <v>1</v>
       </c>
       <c r="S795" t="n">
-        <v>0.02745198179031022</v>
+        <v>0.06589366888801496</v>
       </c>
       <c r="T795" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U795" t="n">
-        <v>0.02745198179031022</v>
+        <v>0.06589366888801496</v>
       </c>
       <c r="V795" t="n">
-        <v>0.4039800991497235</v>
+        <v>0.4150379231667436</v>
       </c>
       <c r="W795" t="n">
-        <v>2.55</v>
+        <v>2.75</v>
       </c>
       <c r="X795" t="inlineStr">
         <is>
@@ -80764,7 +80764,7 @@
       </c>
       <c r="Y795" t="inlineStr"/>
       <c r="Z795" t="n">
-        <v>4.241791041072097</v>
+        <v>3.606986940410689</v>
       </c>
       <c r="AA795" t="inlineStr">
         <is>
@@ -80831,28 +80831,28 @@
         <v>2</v>
       </c>
       <c r="O796" t="n">
-        <v>0.1471395188753668</v>
+        <v>0.09689707861261347</v>
       </c>
       <c r="P796" t="n">
-        <v>0.3643517645014451</v>
+        <v>0.2722214807658915</v>
       </c>
       <c r="Q796" t="n">
-        <v>0.488508716623188</v>
+        <v>0.630881440621495</v>
       </c>
       <c r="R796" t="n">
         <v>1</v>
       </c>
       <c r="S796" t="n">
-        <v>-0.1387640106495393</v>
+        <v>0.003608713348767667</v>
       </c>
       <c r="T796" t="n">
         <v>2</v>
       </c>
       <c r="U796" t="n">
-        <v>-0.1387640106495393</v>
+        <v>0.003608713348767667</v>
       </c>
       <c r="V796" t="n">
-        <v>0.488508716623188</v>
+        <v>0.630881440621495</v>
       </c>
       <c r="W796" t="n">
         <v>1.5</v>
@@ -80864,7 +80864,7 @@
       </c>
       <c r="Y796" t="inlineStr"/>
       <c r="Z796" t="n">
-        <v>5.129341524543474</v>
+        <v>4.75867615477697</v>
       </c>
       <c r="AA796" t="inlineStr">
         <is>
@@ -80931,28 +80931,28 @@
         <v>0</v>
       </c>
       <c r="O797" t="n">
-        <v>0.1574923527742556</v>
+        <v>0.2088331223789345</v>
       </c>
       <c r="P797" t="n">
-        <v>0.4300901620948807</v>
+        <v>0.5348698369114847</v>
       </c>
       <c r="Q797" t="n">
-        <v>0.4124174851308637</v>
+        <v>0.2562970407095808</v>
       </c>
       <c r="R797" t="n">
         <v>1</v>
       </c>
       <c r="S797" t="n">
-        <v>0.1463203982238594</v>
+        <v>0.2511000730404634</v>
       </c>
       <c r="T797" t="n">
         <v>0</v>
       </c>
       <c r="U797" t="n">
-        <v>0.1463203982238594</v>
+        <v>0.2511000730404634</v>
       </c>
       <c r="V797" t="n">
-        <v>0.4300901620948807</v>
+        <v>0.5348698369114847</v>
       </c>
       <c r="W797" t="n">
         <v>3.3</v>
@@ -80964,7 +80964,7 @@
       </c>
       <c r="Y797" t="inlineStr"/>
       <c r="Z797" t="n">
-        <v>4.515946701996247</v>
+        <v>5.894774324639611</v>
       </c>
       <c r="AA797" t="inlineStr">
         <is>
@@ -81031,28 +81031,28 @@
         <v>1</v>
       </c>
       <c r="O798" t="n">
-        <v>0.6236860345475682</v>
+        <v>0.7042321714709319</v>
       </c>
       <c r="P798" t="n">
-        <v>0.205813716083146</v>
+        <v>0.232253277494293</v>
       </c>
       <c r="Q798" t="n">
-        <v>0.1705002493692858</v>
+        <v>0.06351455103477525</v>
       </c>
       <c r="R798" t="n">
         <v>1</v>
       </c>
       <c r="S798" t="n">
-        <v>-0.0911799280844382</v>
+        <v>-0.01063379116107455</v>
       </c>
       <c r="T798" t="n">
         <v>1</v>
       </c>
       <c r="U798" t="n">
-        <v>-0.0911799280844382</v>
+        <v>-0.01063379116107455</v>
       </c>
       <c r="V798" t="n">
-        <v>0.6236860345475682</v>
+        <v>0.7042321714709319</v>
       </c>
       <c r="W798" t="n">
         <v>1.3</v>
@@ -81064,7 +81064,7 @@
       </c>
       <c r="Y798" t="inlineStr"/>
       <c r="Z798" t="n">
-        <v>6.548703362749467</v>
+        <v>5.20198785232393</v>
       </c>
       <c r="AA798" t="inlineStr">
         <is>
@@ -81131,28 +81131,28 @@
         <v>0</v>
       </c>
       <c r="O799" t="n">
-        <v>0.3710455118577684</v>
+        <v>0.4033138879806065</v>
       </c>
       <c r="P799" t="n">
-        <v>0.438386025585098</v>
+        <v>0.4556884252719923</v>
       </c>
       <c r="Q799" t="n">
-        <v>0.1905684625571337</v>
+        <v>0.1409976867474011</v>
       </c>
       <c r="R799" t="n">
         <v>1</v>
       </c>
       <c r="S799" t="n">
-        <v>0.1930589227813597</v>
+        <v>0.210361322468254</v>
       </c>
       <c r="T799" t="n">
         <v>0</v>
       </c>
       <c r="U799" t="n">
-        <v>0.1930589227813597</v>
+        <v>0.210361322468254</v>
       </c>
       <c r="V799" t="n">
-        <v>0.438386025585098</v>
+        <v>0.4556884252719923</v>
       </c>
       <c r="W799" t="n">
         <v>3.8</v>
@@ -81164,7 +81164,7 @@
       </c>
       <c r="Y799" t="inlineStr"/>
       <c r="Z799" t="n">
-        <v>4.603053268643529</v>
+        <v>4.995373108051847</v>
       </c>
       <c r="AA799" t="inlineStr">
         <is>
@@ -81231,28 +81231,28 @@
         <v>0</v>
       </c>
       <c r="O800" t="n">
-        <v>0.1473263041500863</v>
+        <v>0.1256190672145784</v>
       </c>
       <c r="P800" t="n">
-        <v>0.482071837748568</v>
+        <v>0.5757215697334177</v>
       </c>
       <c r="Q800" t="n">
-        <v>0.3706018581013456</v>
+        <v>0.298659363052004</v>
       </c>
       <c r="R800" t="n">
         <v>1</v>
       </c>
       <c r="S800" t="n">
-        <v>0.2280395796840519</v>
+        <v>0.3216893116689016</v>
       </c>
       <c r="T800" t="n">
         <v>0</v>
       </c>
       <c r="U800" t="n">
-        <v>0.2280395796840519</v>
+        <v>0.3216893116689016</v>
       </c>
       <c r="V800" t="n">
-        <v>0.482071837748568</v>
+        <v>0.5757215697334177</v>
       </c>
       <c r="W800" t="n">
         <v>3.7</v>
@@ -81264,7 +81264,7 @@
       </c>
       <c r="Y800" t="inlineStr"/>
       <c r="Z800" t="n">
-        <v>5.061754296359965</v>
+        <v>6.730581610517395</v>
       </c>
       <c r="AA800" t="inlineStr">
         <is>
@@ -81328,34 +81328,34 @@
         <v>0.06572585309427414</v>
       </c>
       <c r="N801" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O801" t="n">
-        <v>0.4310469021852965</v>
+        <v>0.4821308049784111</v>
       </c>
       <c r="P801" t="n">
-        <v>0.5472413686026405</v>
+        <v>0.4534845644434831</v>
       </c>
       <c r="Q801" t="n">
-        <v>0.02171172921206298</v>
+        <v>0.06438463057810576</v>
       </c>
       <c r="R801" t="n">
         <v>1</v>
       </c>
       <c r="S801" t="n">
-        <v>0.3971089498990413</v>
+        <v>-0.2233786814106827</v>
       </c>
       <c r="T801" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U801" t="n">
-        <v>0.3971089498990413</v>
+        <v>-0.2233786814106827</v>
       </c>
       <c r="V801" t="n">
-        <v>0.5472413686026405</v>
+        <v>0.4821308049784111</v>
       </c>
       <c r="W801" t="n">
-        <v>6.25</v>
+        <v>1.33</v>
       </c>
       <c r="X801" t="inlineStr">
         <is>
@@ -81364,7 +81364,7 @@
       </c>
       <c r="Y801" t="inlineStr"/>
       <c r="Z801" t="n">
-        <v>5.746034370327726</v>
+        <v>1.940640926757963</v>
       </c>
       <c r="AA801" t="inlineStr">
         <is>
@@ -81428,34 +81428,34 @@
         <v>0.06555753614577142</v>
       </c>
       <c r="N802" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O802" t="n">
-        <v>0.5367145159637345</v>
+        <v>0.2507085206948234</v>
       </c>
       <c r="P802" t="n">
-        <v>0.3562084296252203</v>
+        <v>0.2133503050251686</v>
       </c>
       <c r="Q802" t="n">
-        <v>0.1070770544110452</v>
+        <v>0.535941174280008</v>
       </c>
       <c r="R802" t="n">
         <v>1</v>
       </c>
       <c r="S802" t="n">
-        <v>0.189130872841058</v>
+        <v>0.1679114345030562</v>
       </c>
       <c r="T802" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U802" t="n">
-        <v>0.189130872841058</v>
+        <v>0.1679114345030562</v>
       </c>
       <c r="V802" t="n">
-        <v>0.5367145159637345</v>
+        <v>0.535941174280008</v>
       </c>
       <c r="W802" t="n">
-        <v>2.7</v>
+        <v>2.55</v>
       </c>
       <c r="X802" t="inlineStr">
         <is>
@@ -81464,7 +81464,7 @@
       </c>
       <c r="Y802" t="inlineStr"/>
       <c r="Z802" t="n">
-        <v>5.635502417619213</v>
+        <v>5.278894565872982</v>
       </c>
       <c r="AA802" t="inlineStr">
         <is>
@@ -81532,34 +81532,34 @@
         <v>0.0642802155504234</v>
       </c>
       <c r="N803" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O803" t="n">
-        <v>0.1619026486591099</v>
+        <v>0.1486557701836623</v>
       </c>
       <c r="P803" t="n">
-        <v>0.4516790736563854</v>
+        <v>0.3067029727225868</v>
       </c>
       <c r="Q803" t="n">
-        <v>0.3864182776845047</v>
+        <v>0.544641257093751</v>
       </c>
       <c r="R803" t="n">
         <v>1</v>
       </c>
       <c r="S803" t="n">
-        <v>0.1906784708836307</v>
+        <v>0.02264005154824167</v>
       </c>
       <c r="T803" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="U803" t="n">
-        <v>0.1906784708836307</v>
+        <v>0.02264005154824167</v>
       </c>
       <c r="V803" t="n">
-        <v>0.4516790736563854</v>
+        <v>0.544641257093751</v>
       </c>
       <c r="W803" t="n">
-        <v>3.6</v>
+        <v>1.8</v>
       </c>
       <c r="X803" t="inlineStr">
         <is>
@@ -81568,7 +81568,7 @@
       </c>
       <c r="Y803" t="inlineStr"/>
       <c r="Z803" t="n">
-        <v>4.742630273392047</v>
+        <v>4.254609814814945</v>
       </c>
       <c r="AA803" t="inlineStr">
         <is>
@@ -81635,28 +81635,28 @@
         <v>1</v>
       </c>
       <c r="O804" t="n">
-        <v>0.5866634068617192</v>
+        <v>0.4508759008941493</v>
       </c>
       <c r="P804" t="n">
-        <v>0.3496478379670511</v>
+        <v>0.2285184540939349</v>
       </c>
       <c r="Q804" t="n">
-        <v>0.06368875517122981</v>
+        <v>0.3206056450119157</v>
       </c>
       <c r="R804" t="n">
         <v>1</v>
       </c>
       <c r="S804" t="n">
-        <v>-0.05203308456555444</v>
+        <v>-0.1878205905331244</v>
       </c>
       <c r="T804" t="n">
         <v>1</v>
       </c>
       <c r="U804" t="n">
-        <v>-0.05203308456555444</v>
+        <v>-0.1878205905331244</v>
       </c>
       <c r="V804" t="n">
-        <v>0.5866634068617192</v>
+        <v>0.4508759008941493</v>
       </c>
       <c r="W804" t="n">
         <v>1.48</v>
@@ -81668,7 +81668,7 @@
       </c>
       <c r="Y804" t="inlineStr"/>
       <c r="Z804" t="n">
-        <v>6.159965772048052</v>
+        <v>1.972914827707687</v>
       </c>
       <c r="AA804" t="inlineStr">
         <is>
@@ -81736,34 +81736,34 @@
         <v>0.07449392712550607</v>
       </c>
       <c r="N805" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O805" t="n">
-        <v>0.3995849870108082</v>
+        <v>0.5503598610958481</v>
       </c>
       <c r="P805" t="n">
-        <v>0.4202789944814728</v>
+        <v>0.3773769491585818</v>
       </c>
       <c r="Q805" t="n">
-        <v>0.1801360185077191</v>
+        <v>0.07226318974557</v>
       </c>
       <c r="R805" t="n">
         <v>1</v>
       </c>
       <c r="S805" t="n">
-        <v>0.2341448573300033</v>
+        <v>-0.1655406664098037</v>
       </c>
       <c r="T805" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U805" t="n">
-        <v>0.2341448573300033</v>
+        <v>-0.1655406664098037</v>
       </c>
       <c r="V805" t="n">
-        <v>0.4202789944814728</v>
+        <v>0.5503598610958481</v>
       </c>
       <c r="W805" t="n">
-        <v>5</v>
+        <v>1.3</v>
       </c>
       <c r="X805" t="inlineStr">
         <is>
@@ -81772,7 +81772,7 @@
       </c>
       <c r="Y805" t="inlineStr"/>
       <c r="Z805" t="n">
-        <v>4.412929442055464</v>
+        <v>2.886143960145333</v>
       </c>
       <c r="AA805" t="inlineStr">
         <is>
@@ -81839,28 +81839,28 @@
         <v>1</v>
       </c>
       <c r="O806" t="n">
-        <v>0.4840339158983135</v>
+        <v>0.5242036523409902</v>
       </c>
       <c r="P806" t="n">
-        <v>0.176257951507396</v>
+        <v>0.2349479415483951</v>
       </c>
       <c r="Q806" t="n">
-        <v>0.3397081325942906</v>
+        <v>0.2408484061106148</v>
       </c>
       <c r="R806" t="n">
         <v>1</v>
       </c>
       <c r="S806" t="n">
-        <v>0.1431248249892226</v>
+        <v>0.1832945614318994</v>
       </c>
       <c r="T806" t="n">
         <v>1</v>
       </c>
       <c r="U806" t="n">
-        <v>0.1431248249892226</v>
+        <v>0.1832945614318994</v>
       </c>
       <c r="V806" t="n">
-        <v>0.4840339158983135</v>
+        <v>0.5242036523409902</v>
       </c>
       <c r="W806" t="n">
         <v>2.75</v>
@@ -81872,7 +81872,7 @@
       </c>
       <c r="Y806" t="inlineStr"/>
       <c r="Z806" t="n">
-        <v>5.082356116932291</v>
+        <v>5.306236603296671</v>
       </c>
       <c r="AA806" t="inlineStr">
         <is>
@@ -81925,13 +81925,13 @@
         <v>2</v>
       </c>
       <c r="O807" t="n">
-        <v>0.09521870087495758</v>
+        <v>0.1404077831145912</v>
       </c>
       <c r="P807" t="n">
-        <v>0.2539205918363993</v>
+        <v>0.2410564208072057</v>
       </c>
       <c r="Q807" t="n">
-        <v>0.6508607072886432</v>
+        <v>0.6185357960782031</v>
       </c>
       <c r="R807" t="n">
         <v>1</v>
@@ -81942,7 +81942,7 @@
       </c>
       <c r="U807" t="inlineStr"/>
       <c r="V807" t="n">
-        <v>0.3491392927113568</v>
+        <v>0.3814642039217969</v>
       </c>
       <c r="W807" t="inlineStr"/>
       <c r="X807" t="inlineStr">
@@ -82003,13 +82003,13 @@
         <v>1</v>
       </c>
       <c r="O808" t="n">
-        <v>0.4590028515354094</v>
+        <v>0.4928896298320464</v>
       </c>
       <c r="P808" t="n">
-        <v>0.4002904591348134</v>
+        <v>0.372727452443282</v>
       </c>
       <c r="Q808" t="n">
-        <v>0.1407066893297772</v>
+        <v>0.1343829177246716</v>
       </c>
       <c r="R808" t="n">
         <v>1</v>
@@ -82020,7 +82020,7 @@
       </c>
       <c r="U808" t="inlineStr"/>
       <c r="V808" t="n">
-        <v>0.5409971484645906</v>
+        <v>0.5071103701679536</v>
       </c>
       <c r="W808" t="inlineStr"/>
       <c r="X808" t="inlineStr">
@@ -82081,13 +82081,13 @@
         <v>0</v>
       </c>
       <c r="O809" t="n">
-        <v>0.2765464094530681</v>
+        <v>0.3108903765353306</v>
       </c>
       <c r="P809" t="n">
-        <v>0.3745201324691835</v>
+        <v>0.4209719977319064</v>
       </c>
       <c r="Q809" t="n">
-        <v>0.3489334580777484</v>
+        <v>0.2681376257327631</v>
       </c>
       <c r="R809" t="n">
         <v>1</v>
@@ -82098,7 +82098,7 @@
       </c>
       <c r="U809" t="inlineStr"/>
       <c r="V809" t="n">
-        <v>0.6254798675308164</v>
+        <v>0.5790280022680936</v>
       </c>
       <c r="W809" t="inlineStr"/>
       <c r="X809" t="inlineStr">
@@ -82159,13 +82159,13 @@
         <v>2</v>
       </c>
       <c r="O810" t="n">
-        <v>0.1159651659974166</v>
+        <v>0.1947041493302815</v>
       </c>
       <c r="P810" t="n">
-        <v>0.3065263098875333</v>
+        <v>0.3743005269439676</v>
       </c>
       <c r="Q810" t="n">
-        <v>0.5775085241150499</v>
+        <v>0.4309953237257507</v>
       </c>
       <c r="R810" t="n">
         <v>1</v>
@@ -82176,7 +82176,7 @@
       </c>
       <c r="U810" t="inlineStr"/>
       <c r="V810" t="n">
-        <v>0.4224914758849501</v>
+        <v>0.5690046762742493</v>
       </c>
       <c r="W810" t="inlineStr"/>
       <c r="X810" t="inlineStr">
@@ -82237,13 +82237,13 @@
         <v>2</v>
       </c>
       <c r="O811" t="n">
-        <v>0.2526336269138234</v>
+        <v>0.2759336133792271</v>
       </c>
       <c r="P811" t="n">
-        <v>0.08904208527688624</v>
+        <v>0.311643971783173</v>
       </c>
       <c r="Q811" t="n">
-        <v>0.6583242878092903</v>
+        <v>0.4124224148375999</v>
       </c>
       <c r="R811" t="n">
         <v>1</v>
@@ -82254,7 +82254,7 @@
       </c>
       <c r="U811" t="inlineStr"/>
       <c r="V811" t="n">
-        <v>0.3416757121907097</v>
+        <v>0.5875775851624001</v>
       </c>
       <c r="W811" t="inlineStr"/>
       <c r="X811" t="inlineStr">
@@ -82312,27 +82312,27 @@
       <c r="L812" t="inlineStr"/>
       <c r="M812" t="inlineStr"/>
       <c r="N812" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O812" t="n">
-        <v>0.07540606598657494</v>
+        <v>0.1166836106676965</v>
       </c>
       <c r="P812" t="n">
-        <v>0.4053477941475529</v>
+        <v>0.4513090915549166</v>
       </c>
       <c r="Q812" t="n">
-        <v>0.5192461398658722</v>
+        <v>0.4320072977773868</v>
       </c>
       <c r="R812" t="n">
         <v>1</v>
       </c>
       <c r="S812" t="inlineStr"/>
       <c r="T812" t="n">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="U812" t="inlineStr"/>
       <c r="V812" t="n">
-        <v>0.4807538601341278</v>
+        <v>0.5486909084450834</v>
       </c>
       <c r="W812" t="inlineStr"/>
       <c r="X812" t="inlineStr">
@@ -82390,27 +82390,27 @@
       <c r="L813" t="inlineStr"/>
       <c r="M813" t="inlineStr"/>
       <c r="N813" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O813" t="n">
-        <v>0.3121003667242244</v>
+        <v>0.3945086144240301</v>
       </c>
       <c r="P813" t="n">
-        <v>0.1942617490478571</v>
+        <v>0.4816284954539337</v>
       </c>
       <c r="Q813" t="n">
-        <v>0.4936378842279185</v>
+        <v>0.1238628901220363</v>
       </c>
       <c r="R813" t="n">
         <v>1</v>
       </c>
       <c r="S813" t="inlineStr"/>
       <c r="T813" t="n">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="U813" t="inlineStr"/>
       <c r="V813" t="n">
-        <v>0.5063621157720815</v>
+        <v>0.5183715045460663</v>
       </c>
       <c r="W813" t="inlineStr"/>
       <c r="X813" t="inlineStr">
@@ -82471,13 +82471,13 @@
         <v>1</v>
       </c>
       <c r="O814" t="n">
-        <v>0.5181174037940751</v>
+        <v>0.4719291039989259</v>
       </c>
       <c r="P814" t="n">
-        <v>0.313856615941432</v>
+        <v>0.3833542880789495</v>
       </c>
       <c r="Q814" t="n">
-        <v>0.1680259802644929</v>
+        <v>0.1447166079221247</v>
       </c>
       <c r="R814" t="n">
         <v>1</v>
@@ -82488,7 +82488,7 @@
       </c>
       <c r="U814" t="inlineStr"/>
       <c r="V814" t="n">
-        <v>0.4818825962059249</v>
+        <v>0.528070896001074</v>
       </c>
       <c r="W814" t="inlineStr"/>
       <c r="X814" t="inlineStr">
@@ -82563,28 +82563,28 @@
         <v>0</v>
       </c>
       <c r="O815" t="n">
-        <v>0.4081229714264447</v>
+        <v>0.324077692928472</v>
       </c>
       <c r="P815" t="n">
-        <v>0.4336215137799843</v>
+        <v>0.4639103892601431</v>
       </c>
       <c r="Q815" t="n">
-        <v>0.1582555147935711</v>
+        <v>0.2120119178113849</v>
       </c>
       <c r="R815" t="n">
         <v>1</v>
       </c>
       <c r="S815" t="n">
-        <v>0.1507267769378791</v>
+        <v>0.1810156524180379</v>
       </c>
       <c r="T815" t="n">
         <v>0</v>
       </c>
       <c r="U815" t="n">
-        <v>0.1507267769378791</v>
+        <v>0.1810156524180379</v>
       </c>
       <c r="V815" t="n">
-        <v>0.4336215137799843</v>
+        <v>0.4639103892601431</v>
       </c>
       <c r="W815" t="n">
         <v>3.3</v>
@@ -82596,7 +82596,7 @@
       </c>
       <c r="Y815" t="inlineStr"/>
       <c r="Z815" t="n">
-        <v>0.7588376491149725</v>
+        <v>7.739112500138172</v>
       </c>
       <c r="AA815" t="inlineStr">
         <is>
@@ -82608,7 +82608,9 @@
           <t>ligue 1</t>
         </is>
       </c>
-      <c r="AC815" t="inlineStr"/>
+      <c r="AC815" t="n">
+        <v>1</v>
+      </c>
       <c r="AD815" t="inlineStr"/>
       <c r="AE815" t="inlineStr"/>
       <c r="AF815" t="n">
@@ -82665,28 +82667,28 @@
         <v>0</v>
       </c>
       <c r="O816" t="n">
-        <v>0.1540605978838488</v>
+        <v>0.1379803712266632</v>
       </c>
       <c r="P816" t="n">
-        <v>0.6916568036688272</v>
+        <v>0.5149237071361238</v>
       </c>
       <c r="Q816" t="n">
-        <v>0.1542825984473239</v>
+        <v>0.347095921637213</v>
       </c>
       <c r="R816" t="n">
         <v>1</v>
       </c>
       <c r="S816" t="n">
-        <v>0.4071039581403719</v>
+        <v>0.2303708616076685</v>
       </c>
       <c r="T816" t="n">
         <v>0</v>
       </c>
       <c r="U816" t="n">
-        <v>0.4071039581403719</v>
+        <v>0.2303708616076685</v>
       </c>
       <c r="V816" t="n">
-        <v>0.6916568036688272</v>
+        <v>0.5149237071361238</v>
       </c>
       <c r="W816" t="n">
         <v>3.3</v>
@@ -82698,7 +82700,7 @@
       </c>
       <c r="Y816" t="inlineStr"/>
       <c r="Z816" t="n">
-        <v>1.210399406420448</v>
+        <v>8.943534824925507</v>
       </c>
       <c r="AA816" t="inlineStr">
         <is>
@@ -82710,7 +82712,9 @@
           <t>ligue 1</t>
         </is>
       </c>
-      <c r="AC816" t="inlineStr"/>
+      <c r="AC816" t="n">
+        <v>1</v>
+      </c>
       <c r="AD816" t="inlineStr"/>
       <c r="AE816" t="inlineStr"/>
       <c r="AF816" t="n">
@@ -82767,28 +82771,28 @@
         <v>1</v>
       </c>
       <c r="O817" t="n">
-        <v>0.4612877305655307</v>
+        <v>0.4540643885737281</v>
       </c>
       <c r="P817" t="n">
-        <v>0.2960909986728214</v>
+        <v>0.4387363630093123</v>
       </c>
       <c r="Q817" t="n">
-        <v>0.242621270761648</v>
+        <v>0.1071992484169596</v>
       </c>
       <c r="R817" t="n">
         <v>1</v>
       </c>
       <c r="S817" t="n">
-        <v>-0.1405294356188704</v>
+        <v>-0.147752777610673</v>
       </c>
       <c r="T817" t="n">
         <v>1</v>
       </c>
       <c r="U817" t="n">
-        <v>-0.1405294356188704</v>
+        <v>-0.147752777610673</v>
       </c>
       <c r="V817" t="n">
-        <v>0.4612877305655307</v>
+        <v>0.4540643885737281</v>
       </c>
       <c r="W817" t="n">
         <v>1.57</v>
@@ -82800,7 +82804,7 @@
       </c>
       <c r="Y817" t="inlineStr"/>
       <c r="Z817" t="n">
-        <v>0.8072535284896787</v>
+        <v>3.675739331556662</v>
       </c>
       <c r="AA817" t="inlineStr">
         <is>
@@ -82812,7 +82816,9 @@
           <t>ligue 1</t>
         </is>
       </c>
-      <c r="AC817" t="inlineStr"/>
+      <c r="AC817" t="n">
+        <v>1</v>
+      </c>
       <c r="AD817" t="inlineStr"/>
       <c r="AE817" t="inlineStr"/>
       <c r="AF817" t="n">
@@ -82869,28 +82875,28 @@
         <v>1</v>
       </c>
       <c r="O818" t="n">
-        <v>0.4933269530486849</v>
+        <v>0.7806472412053725</v>
       </c>
       <c r="P818" t="n">
-        <v>0.2675547565480448</v>
+        <v>0.1657313185467316</v>
       </c>
       <c r="Q818" t="n">
-        <v>0.2391182904032703</v>
+        <v>0.05362144024789593</v>
       </c>
       <c r="R818" t="n">
         <v>1</v>
       </c>
       <c r="S818" t="n">
-        <v>-0.1947464414467279</v>
+        <v>0.09257384670995972</v>
       </c>
       <c r="T818" t="n">
         <v>1</v>
       </c>
       <c r="U818" t="n">
-        <v>-0.1947464414467279</v>
+        <v>0.09257384670995972</v>
       </c>
       <c r="V818" t="n">
-        <v>0.4933269530486849</v>
+        <v>0.7806472412053725</v>
       </c>
       <c r="W818" t="n">
         <v>1.36</v>
@@ -82902,7 +82908,7 @@
       </c>
       <c r="Y818" t="inlineStr"/>
       <c r="Z818" t="n">
-        <v>0.8633221678351986</v>
+        <v>10.47865305498399</v>
       </c>
       <c r="AA818" t="inlineStr">
         <is>
@@ -82914,7 +82920,9 @@
           <t>ligue 1</t>
         </is>
       </c>
-      <c r="AC818" t="inlineStr"/>
+      <c r="AC818" t="n">
+        <v>1</v>
+      </c>
       <c r="AD818" t="inlineStr"/>
       <c r="AE818" t="inlineStr"/>
       <c r="AF818" t="n">
@@ -82971,28 +82979,28 @@
         <v>0</v>
       </c>
       <c r="O819" t="n">
-        <v>0.1388525485245407</v>
+        <v>0.1053726601706592</v>
       </c>
       <c r="P819" t="n">
-        <v>0.4673355310121895</v>
+        <v>0.4974088918099869</v>
       </c>
       <c r="Q819" t="n">
-        <v>0.3938119204632699</v>
+        <v>0.3972184480193539</v>
       </c>
       <c r="R819" t="n">
         <v>1</v>
       </c>
       <c r="S819" t="n">
-        <v>0.1752421266697069</v>
+        <v>0.2053154874675043</v>
       </c>
       <c r="T819" t="n">
         <v>0</v>
       </c>
       <c r="U819" t="n">
-        <v>0.1752421266697069</v>
+        <v>0.2053154874675043</v>
       </c>
       <c r="V819" t="n">
-        <v>0.4673355310121895</v>
+        <v>0.4974088918099869</v>
       </c>
       <c r="W819" t="n">
         <v>3.2</v>
@@ -83004,7 +83012,7 @@
       </c>
       <c r="Y819" t="inlineStr"/>
       <c r="Z819" t="n">
-        <v>0.8178371792713316</v>
+        <v>8.432692551329893</v>
       </c>
       <c r="AA819" t="inlineStr">
         <is>
@@ -83016,7 +83024,9 @@
           <t>ligue 1</t>
         </is>
       </c>
-      <c r="AC819" t="inlineStr"/>
+      <c r="AC819" t="n">
+        <v>1</v>
+      </c>
       <c r="AD819" t="inlineStr"/>
       <c r="AE819" t="inlineStr"/>
       <c r="AF819" t="n">
@@ -83073,28 +83083,28 @@
         <v>1</v>
       </c>
       <c r="O820" t="n">
-        <v>0.5232983734289283</v>
+        <v>0.4204282090040678</v>
       </c>
       <c r="P820" t="n">
-        <v>0.2043189535242267</v>
+        <v>0.225270261780631</v>
       </c>
       <c r="Q820" t="n">
-        <v>0.272382673046845</v>
+        <v>0.3543015292153012</v>
       </c>
       <c r="R820" t="n">
         <v>1</v>
       </c>
       <c r="S820" t="n">
-        <v>0.02608388874926254</v>
+        <v>-0.07678627567559793</v>
       </c>
       <c r="T820" t="n">
         <v>1</v>
       </c>
       <c r="U820" t="n">
-        <v>0.02608388874926254</v>
+        <v>-0.07678627567559793</v>
       </c>
       <c r="V820" t="n">
-        <v>0.5232983734289283</v>
+        <v>0.4204282090040678</v>
       </c>
       <c r="W820" t="n">
         <v>1.9</v>
@@ -83106,7 +83116,7 @@
       </c>
       <c r="Y820" t="inlineStr"/>
       <c r="Z820" t="n">
-        <v>0.9157721535006245</v>
+        <v>4.123703199941638</v>
       </c>
       <c r="AA820" t="inlineStr">
         <is>
@@ -83118,7 +83128,9 @@
           <t>ligue 1</t>
         </is>
       </c>
-      <c r="AC820" t="inlineStr"/>
+      <c r="AC820" t="n">
+        <v>1</v>
+      </c>
       <c r="AD820" t="inlineStr"/>
       <c r="AE820" t="inlineStr"/>
       <c r="AF820" t="n">
@@ -83172,34 +83184,34 @@
         <v>0.06169269327164062</v>
       </c>
       <c r="N821" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O821" t="n">
-        <v>0.2974468989596019</v>
+        <v>0.3533676711964743</v>
       </c>
       <c r="P821" t="n">
-        <v>0.4043345963148964</v>
+        <v>0.3528524669748195</v>
       </c>
       <c r="Q821" t="n">
-        <v>0.2982185047255018</v>
+        <v>0.2937798618287061</v>
       </c>
       <c r="R821" t="n">
         <v>1</v>
       </c>
       <c r="S821" t="n">
-        <v>0.135222557092089</v>
+        <v>-0.1296539376649748</v>
       </c>
       <c r="T821" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U821" t="n">
-        <v>0.135222557092089</v>
+        <v>-0.1296539376649748</v>
       </c>
       <c r="V821" t="n">
-        <v>0.4043345963148964</v>
+        <v>0.3533676711964743</v>
       </c>
       <c r="W821" t="n">
-        <v>3.5</v>
+        <v>1.95</v>
       </c>
       <c r="X821" t="inlineStr">
         <is>
@@ -83208,7 +83220,7 @@
       </c>
       <c r="Y821" t="inlineStr"/>
       <c r="Z821" t="n">
-        <v>0.7075855435510686</v>
+        <v>2.684564802377994</v>
       </c>
       <c r="AA821" t="inlineStr">
         <is>
@@ -83220,7 +83232,9 @@
           <t>ligue 1</t>
         </is>
       </c>
-      <c r="AC821" t="inlineStr"/>
+      <c r="AC821" t="n">
+        <v>1</v>
+      </c>
       <c r="AD821" t="inlineStr"/>
       <c r="AE821" t="inlineStr"/>
       <c r="AF821" t="n">
@@ -83277,28 +83291,28 @@
         <v>1</v>
       </c>
       <c r="O822" t="n">
-        <v>0.4487653052663452</v>
+        <v>0.5279251711191212</v>
       </c>
       <c r="P822" t="n">
-        <v>0.3832956232498627</v>
+        <v>0.3224510307173515</v>
       </c>
       <c r="Q822" t="n">
-        <v>0.1679390714837922</v>
+        <v>0.1496237981635273</v>
       </c>
       <c r="R822" t="n">
         <v>1</v>
       </c>
       <c r="S822" t="n">
-        <v>-0.2614275766640881</v>
+        <v>-0.1822677108113121</v>
       </c>
       <c r="T822" t="n">
         <v>1</v>
       </c>
       <c r="U822" t="n">
-        <v>-0.2614275766640881</v>
+        <v>-0.1822677108113121</v>
       </c>
       <c r="V822" t="n">
-        <v>0.4487653052663452</v>
+        <v>0.5279251711191212</v>
       </c>
       <c r="W822" t="n">
         <v>1.33</v>
@@ -83310,7 +83324,7 @@
       </c>
       <c r="Y822" t="inlineStr"/>
       <c r="Z822" t="n">
-        <v>0.7853392842161041</v>
+        <v>4.147889523693709</v>
       </c>
       <c r="AA822" t="inlineStr">
         <is>
@@ -83322,7 +83336,9 @@
           <t>ligue 1</t>
         </is>
       </c>
-      <c r="AC822" t="inlineStr"/>
+      <c r="AC822" t="n">
+        <v>1</v>
+      </c>
       <c r="AD822" t="inlineStr"/>
       <c r="AE822" t="inlineStr"/>
       <c r="AF822" t="n">
@@ -83379,28 +83395,28 @@
         <v>2</v>
       </c>
       <c r="O823" t="n">
-        <v>0.2320831047002737</v>
+        <v>0.1306911853381278</v>
       </c>
       <c r="P823" t="n">
-        <v>0.1794979337780964</v>
+        <v>0.2895975621293707</v>
       </c>
       <c r="Q823" t="n">
-        <v>0.58841896152163</v>
+        <v>0.5797112525325016</v>
       </c>
       <c r="R823" t="n">
         <v>1</v>
       </c>
       <c r="S823" t="n">
-        <v>0.08546356119922283</v>
+        <v>0.0767558522100944</v>
       </c>
       <c r="T823" t="n">
         <v>2</v>
       </c>
       <c r="U823" t="n">
-        <v>0.08546356119922283</v>
+        <v>0.0767558522100944</v>
       </c>
       <c r="V823" t="n">
-        <v>0.58841896152163</v>
+        <v>0.5797112525325016</v>
       </c>
       <c r="W823" t="n">
         <v>1.85</v>
@@ -83412,7 +83428,7 @@
       </c>
       <c r="Y823" t="inlineStr"/>
       <c r="Z823" t="n">
-        <v>1.029733182662852</v>
+        <v>7.877605256911151</v>
       </c>
       <c r="AA823" t="inlineStr">
         <is>
@@ -83424,7 +83440,9 @@
           <t>ligue 1</t>
         </is>
       </c>
-      <c r="AC823" t="inlineStr"/>
+      <c r="AC823" t="n">
+        <v>1</v>
+      </c>
       <c r="AD823" t="inlineStr"/>
       <c r="AE823" t="inlineStr"/>
       <c r="AF823" t="n">
@@ -83478,34 +83496,34 @@
         <v>0.07160825747213195</v>
       </c>
       <c r="N824" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O824" t="n">
-        <v>0.09338662682896103</v>
+        <v>0.09878743911723988</v>
       </c>
       <c r="P824" t="n">
-        <v>0.6301845339145807</v>
+        <v>0.300170513860593</v>
       </c>
       <c r="Q824" t="n">
-        <v>0.2764288392564582</v>
+        <v>0.6010420470221672</v>
       </c>
       <c r="R824" t="n">
         <v>1</v>
       </c>
       <c r="S824" t="n">
-        <v>0.3779745790306722</v>
+        <v>0.1124677888700931</v>
       </c>
       <c r="T824" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="U824" t="n">
-        <v>0.3779745790306722</v>
+        <v>0.1124677888700931</v>
       </c>
       <c r="V824" t="n">
-        <v>0.6301845339145807</v>
+        <v>0.6010420470221672</v>
       </c>
       <c r="W824" t="n">
-        <v>3.7</v>
+        <v>1.91</v>
       </c>
       <c r="X824" t="inlineStr">
         <is>
@@ -83514,7 +83532,7 @@
       </c>
       <c r="Y824" t="inlineStr"/>
       <c r="Z824" t="n">
-        <v>1.102822934350516</v>
+        <v>8.562118030707122</v>
       </c>
       <c r="AA824" t="inlineStr">
         <is>
@@ -83526,7 +83544,9 @@
           <t>ligue 1</t>
         </is>
       </c>
-      <c r="AC824" t="inlineStr"/>
+      <c r="AC824" t="n">
+        <v>1</v>
+      </c>
       <c r="AD824" t="inlineStr"/>
       <c r="AE824" t="inlineStr"/>
       <c r="AF824" t="n">
@@ -83580,34 +83600,34 @@
         <v>0.06333056478405319</v>
       </c>
       <c r="N825" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O825" t="n">
-        <v>0.4333994997931968</v>
+        <v>0.2581118841958259</v>
       </c>
       <c r="P825" t="n">
-        <v>0.2713702604968151</v>
+        <v>0.1989939058272581</v>
       </c>
       <c r="Q825" t="n">
-        <v>0.2952302397099882</v>
+        <v>0.5428942099769158</v>
       </c>
       <c r="R825" t="n">
         <v>1</v>
       </c>
       <c r="S825" t="n">
-        <v>0.1395115872761102</v>
+        <v>0.1054796425096243</v>
       </c>
       <c r="T825" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U825" t="n">
-        <v>0.1395115872761102</v>
+        <v>0.1054796425096243</v>
       </c>
       <c r="V825" t="n">
-        <v>0.4333994997931968</v>
+        <v>0.5428942099769158</v>
       </c>
       <c r="W825" t="n">
-        <v>3.2</v>
+        <v>2.15</v>
       </c>
       <c r="X825" t="inlineStr">
         <is>
@@ -83616,7 +83636,7 @@
       </c>
       <c r="Y825" t="inlineStr"/>
       <c r="Z825" t="n">
-        <v>0.7584491246380943</v>
+        <v>7.780486229838481</v>
       </c>
       <c r="AA825" t="inlineStr">
         <is>
@@ -83628,7 +83648,9 @@
           <t>ligue 1</t>
         </is>
       </c>
-      <c r="AC825" t="inlineStr"/>
+      <c r="AC825" t="n">
+        <v>1</v>
+      </c>
       <c r="AD825" t="inlineStr"/>
       <c r="AE825" t="inlineStr"/>
       <c r="AF825" t="n">
@@ -83685,28 +83707,28 @@
         <v>0</v>
       </c>
       <c r="O826" t="n">
-        <v>0.1343757632289512</v>
+        <v>0.2172319316671834</v>
       </c>
       <c r="P826" t="n">
-        <v>0.6987021480065809</v>
+        <v>0.5756568182435053</v>
       </c>
       <c r="Q826" t="n">
-        <v>0.1669220887644678</v>
+        <v>0.2071112500893112</v>
       </c>
       <c r="R826" t="n">
         <v>1</v>
       </c>
       <c r="S826" t="n">
-        <v>0.4290392266582663</v>
+        <v>0.3059938968951907</v>
       </c>
       <c r="T826" t="n">
         <v>0</v>
       </c>
       <c r="U826" t="n">
-        <v>0.4290392266582663</v>
+        <v>0.3059938968951907</v>
       </c>
       <c r="V826" t="n">
-        <v>0.6987021480065809</v>
+        <v>0.5756568182435053</v>
       </c>
       <c r="W826" t="n">
         <v>3.5</v>
@@ -83718,7 +83740,7 @@
       </c>
       <c r="Y826" t="inlineStr"/>
       <c r="Z826" t="n">
-        <v>1.222728759011517</v>
+        <v>10.57980858166435</v>
       </c>
       <c r="AA826" t="inlineStr">
         <is>
@@ -83730,7 +83752,9 @@
           <t>ligue 1</t>
         </is>
       </c>
-      <c r="AC826" t="inlineStr"/>
+      <c r="AC826" t="n">
+        <v>1</v>
+      </c>
       <c r="AD826" t="inlineStr"/>
       <c r="AE826" t="inlineStr"/>
       <c r="AF826" t="n">
@@ -83784,34 +83808,34 @@
         <v>0.06644514567978321</v>
       </c>
       <c r="N827" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O827" t="n">
-        <v>0.3557892749159625</v>
+        <v>0.2127509025395223</v>
       </c>
       <c r="P827" t="n">
-        <v>0.3075828597526143</v>
+        <v>0.3128499105222691</v>
       </c>
       <c r="Q827" t="n">
-        <v>0.3366278653314231</v>
+        <v>0.4743991869382086</v>
       </c>
       <c r="R827" t="n">
         <v>1</v>
       </c>
       <c r="S827" t="n">
-        <v>0.01480937068978572</v>
+        <v>0.1178612642682518</v>
       </c>
       <c r="T827" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U827" t="n">
-        <v>0.01480937068978572</v>
+        <v>0.1178612642682518</v>
       </c>
       <c r="V827" t="n">
-        <v>0.3557892749159625</v>
+        <v>0.4743991869382086</v>
       </c>
       <c r="W827" t="n">
-        <v>2.75</v>
+        <v>2.63</v>
       </c>
       <c r="X827" t="inlineStr">
         <is>
@@ -83820,7 +83844,7 @@
       </c>
       <c r="Y827" t="inlineStr"/>
       <c r="Z827" t="n">
-        <v>0.6226312311029344</v>
+        <v>7.107125414477525</v>
       </c>
       <c r="AA827" t="inlineStr">
         <is>
@@ -83832,7 +83856,9 @@
           <t>ligue 1</t>
         </is>
       </c>
-      <c r="AC827" t="inlineStr"/>
+      <c r="AC827" t="n">
+        <v>1</v>
+      </c>
       <c r="AD827" t="inlineStr"/>
       <c r="AE827" t="inlineStr"/>
       <c r="AF827" t="n">
@@ -83886,34 +83912,34 @@
         <v>0.06392106392106389</v>
       </c>
       <c r="N828" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O828" t="n">
-        <v>0.0916476116353241</v>
+        <v>0.05460418857725669</v>
       </c>
       <c r="P828" t="n">
-        <v>0.6136761318261399</v>
+        <v>0.1805041553973031</v>
       </c>
       <c r="Q828" t="n">
-        <v>0.2946762565385361</v>
+        <v>0.7648916560254403</v>
       </c>
       <c r="R828" t="n">
         <v>1</v>
       </c>
       <c r="S828" t="n">
-        <v>0.3596438737616238</v>
+        <v>0.2277948818318919</v>
       </c>
       <c r="T828" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="U828" t="n">
-        <v>0.3596438737616238</v>
+        <v>0.2277948818318919</v>
       </c>
       <c r="V828" t="n">
-        <v>0.6136761318261399</v>
+        <v>0.7648916560254403</v>
       </c>
       <c r="W828" t="n">
-        <v>3.7</v>
+        <v>1.75</v>
       </c>
       <c r="X828" t="inlineStr">
         <is>
@@ -83922,7 +83948,7 @@
       </c>
       <c r="Y828" t="inlineStr"/>
       <c r="Z828" t="n">
-        <v>1.073933230695745</v>
+        <v>11.91223845428799</v>
       </c>
       <c r="AA828" t="inlineStr">
         <is>
@@ -83934,7 +83960,9 @@
           <t>ligue 1</t>
         </is>
       </c>
-      <c r="AC828" t="inlineStr"/>
+      <c r="AC828" t="n">
+        <v>1</v>
+      </c>
       <c r="AD828" t="inlineStr"/>
       <c r="AE828" t="inlineStr"/>
       <c r="AF828" t="n">
@@ -83988,34 +84016,34 @@
         <v>0.08080808080808088</v>
       </c>
       <c r="N829" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O829" t="n">
-        <v>0.3555932207147527</v>
+        <v>0.5252561394618671</v>
       </c>
       <c r="P829" t="n">
-        <v>0.4065874187987044</v>
+        <v>0.302188005534936</v>
       </c>
       <c r="Q829" t="n">
-        <v>0.2378193604865428</v>
+        <v>0.1725558550031968</v>
       </c>
       <c r="R829" t="n">
         <v>1</v>
       </c>
       <c r="S829" t="n">
-        <v>0.1495780730043119</v>
+        <v>0.06263931703196063</v>
       </c>
       <c r="T829" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U829" t="n">
-        <v>0.1495780730043119</v>
+        <v>0.06263931703196063</v>
       </c>
       <c r="V829" t="n">
-        <v>0.4065874187987044</v>
+        <v>0.5252561394618671</v>
       </c>
       <c r="W829" t="n">
-        <v>3.6</v>
+        <v>2</v>
       </c>
       <c r="X829" t="inlineStr">
         <is>
@@ -84024,7 +84052,7 @@
       </c>
       <c r="Y829" t="inlineStr"/>
       <c r="Z829" t="n">
-        <v>0.7115279828977328</v>
+        <v>7.054745477925932</v>
       </c>
       <c r="AA829" t="inlineStr">
         <is>
@@ -84036,7 +84064,9 @@
           <t>ligue 1</t>
         </is>
       </c>
-      <c r="AC829" t="inlineStr"/>
+      <c r="AC829" t="n">
+        <v>1</v>
+      </c>
       <c r="AD829" t="inlineStr"/>
       <c r="AE829" t="inlineStr"/>
       <c r="AF829" t="n">
@@ -84093,28 +84123,28 @@
         <v>1</v>
       </c>
       <c r="O830" t="n">
-        <v>0.636303740991945</v>
+        <v>0.5923005946901039</v>
       </c>
       <c r="P830" t="n">
-        <v>0.1959937461397251</v>
+        <v>0.2737003625815118</v>
       </c>
       <c r="Q830" t="n">
-        <v>0.16770251286833</v>
+        <v>0.1339990427283844</v>
       </c>
       <c r="R830" t="n">
         <v>1</v>
       </c>
       <c r="S830" t="n">
-        <v>0.09412340148377996</v>
+        <v>0.05012025518193886</v>
       </c>
       <c r="T830" t="n">
         <v>1</v>
       </c>
       <c r="U830" t="n">
-        <v>0.09412340148377996</v>
+        <v>0.05012025518193886</v>
       </c>
       <c r="V830" t="n">
-        <v>0.636303740991945</v>
+        <v>0.5923005946901039</v>
       </c>
       <c r="W830" t="n">
         <v>1.73</v>
@@ -84126,7 +84156,7 @@
       </c>
       <c r="Y830" t="inlineStr"/>
       <c r="Z830" t="n">
-        <v>1.113531546735904</v>
+        <v>7.709050198464513</v>
       </c>
       <c r="AA830" t="inlineStr">
         <is>
@@ -84138,7 +84168,9 @@
           <t>ligue 1</t>
         </is>
       </c>
-      <c r="AC830" t="inlineStr"/>
+      <c r="AC830" t="n">
+        <v>1</v>
+      </c>
       <c r="AD830" t="inlineStr"/>
       <c r="AE830" t="inlineStr"/>
       <c r="AF830" t="n">
@@ -84195,28 +84227,28 @@
         <v>1</v>
       </c>
       <c r="O831" t="n">
-        <v>0.7386308201627008</v>
+        <v>0.8406706848051954</v>
       </c>
       <c r="P831" t="n">
-        <v>0.1861917812018613</v>
+        <v>0.1467482517014496</v>
       </c>
       <c r="Q831" t="n">
-        <v>0.07517739863543794</v>
+        <v>0.01258106349335509</v>
       </c>
       <c r="R831" t="n">
         <v>1</v>
       </c>
       <c r="S831" t="n">
-        <v>-0.139774536267165</v>
+        <v>-0.03773467162467037</v>
       </c>
       <c r="T831" t="n">
         <v>1</v>
       </c>
       <c r="U831" t="n">
-        <v>-0.139774536267165</v>
+        <v>-0.03773467162467037</v>
       </c>
       <c r="V831" t="n">
-        <v>0.7386308201627008</v>
+        <v>0.8406706848051954</v>
       </c>
       <c r="W831" t="n">
         <v>1.07</v>
@@ -84228,7 +84260,7 @@
       </c>
       <c r="Y831" t="inlineStr"/>
       <c r="Z831" t="n">
-        <v>1.292603935284726</v>
+        <v>9.6352321581663</v>
       </c>
       <c r="AA831" t="inlineStr">
         <is>
@@ -84240,7 +84272,9 @@
           <t>ligue 1</t>
         </is>
       </c>
-      <c r="AC831" t="inlineStr"/>
+      <c r="AC831" t="n">
+        <v>1</v>
+      </c>
       <c r="AD831" t="inlineStr"/>
       <c r="AE831" t="inlineStr"/>
       <c r="AF831" t="n">
@@ -84325,12 +84359,12 @@
       </c>
       <c r="X832" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.5</t>
+          <t>dif_prob_mod_bm &gt; -1.0</t>
         </is>
       </c>
       <c r="Y832" t="inlineStr"/>
       <c r="Z832" t="n">
-        <v>1.861688895550771</v>
+        <v>1.906538670462715</v>
       </c>
       <c r="AA832" t="inlineStr">
         <is>
@@ -84425,12 +84459,12 @@
       </c>
       <c r="X833" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.5</t>
+          <t>dif_prob_mod_bm &gt; -1.0</t>
         </is>
       </c>
       <c r="Y833" t="inlineStr"/>
       <c r="Z833" t="n">
-        <v>2.626902217842867</v>
+        <v>3.358656917225145</v>
       </c>
       <c r="AA833" t="inlineStr">
         <is>
@@ -84525,12 +84559,12 @@
       </c>
       <c r="X834" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.5</t>
+          <t>dif_prob_mod_bm &gt; -1.0</t>
         </is>
       </c>
       <c r="Y834" t="inlineStr"/>
       <c r="Z834" t="n">
-        <v>1.793867657710195</v>
+        <v>1.769793186005687</v>
       </c>
       <c r="AA834" t="inlineStr">
         <is>
@@ -84625,12 +84659,12 @@
       </c>
       <c r="X835" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.5</t>
+          <t>dif_prob_mod_bm &gt; -1.0</t>
         </is>
       </c>
       <c r="Y835" t="inlineStr"/>
       <c r="Z835" t="n">
-        <v>1.657636717733401</v>
+        <v>1.833201813791061</v>
       </c>
       <c r="AA835" t="inlineStr">
         <is>
@@ -84725,12 +84759,12 @@
       </c>
       <c r="X836" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.5</t>
+          <t>dif_prob_mod_bm &gt; -1.0</t>
         </is>
       </c>
       <c r="Y836" t="inlineStr"/>
       <c r="Z836" t="n">
-        <v>0.4795529072617221</v>
+        <v>0</v>
       </c>
       <c r="AA836" t="inlineStr">
         <is>
@@ -84825,12 +84859,12 @@
       </c>
       <c r="X837" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.5</t>
+          <t>dif_prob_mod_bm &gt; -1.0</t>
         </is>
       </c>
       <c r="Y837" t="inlineStr"/>
       <c r="Z837" t="n">
-        <v>2.111343835509833</v>
+        <v>2.479620113446103</v>
       </c>
       <c r="AA837" t="inlineStr">
         <is>
@@ -84925,12 +84959,12 @@
       </c>
       <c r="X838" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.5</t>
+          <t>dif_prob_mod_bm &gt; -1.0</t>
         </is>
       </c>
       <c r="Y838" t="inlineStr"/>
       <c r="Z838" t="n">
-        <v>4.380723748400699</v>
+        <v>5.90039503029898</v>
       </c>
       <c r="AA838" t="inlineStr">
         <is>
@@ -85029,12 +85063,12 @@
       </c>
       <c r="X839" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.5</t>
+          <t>dif_prob_mod_bm &gt; -1.0</t>
         </is>
       </c>
       <c r="Y839" t="inlineStr"/>
       <c r="Z839" t="n">
-        <v>1.887674951707864</v>
+        <v>1.532394872442724</v>
       </c>
       <c r="AA839" t="inlineStr">
         <is>
@@ -85129,12 +85163,12 @@
       </c>
       <c r="X840" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.5</t>
+          <t>dif_prob_mod_bm &gt; -1.0</t>
         </is>
       </c>
       <c r="Y840" t="inlineStr"/>
       <c r="Z840" t="n">
-        <v>1.441869728526905</v>
+        <v>1.162746617849576</v>
       </c>
       <c r="AA840" t="inlineStr">
         <is>
@@ -85229,12 +85263,12 @@
       </c>
       <c r="X841" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.5</t>
+          <t>dif_prob_mod_bm &gt; -1.0</t>
         </is>
       </c>
       <c r="Y841" t="inlineStr"/>
       <c r="Z841" t="n">
-        <v>1.870938981982678</v>
+        <v>1.423943683181157</v>
       </c>
       <c r="AA841" t="inlineStr">
         <is>
@@ -85329,12 +85363,12 @@
       </c>
       <c r="X842" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.5</t>
+          <t>dif_prob_mod_bm &gt; -1.0</t>
         </is>
       </c>
       <c r="Y842" t="inlineStr"/>
       <c r="Z842" t="n">
-        <v>2.262709945272415</v>
+        <v>1.888634633415834</v>
       </c>
       <c r="AA842" t="inlineStr">
         <is>
@@ -85429,12 +85463,12 @@
       </c>
       <c r="X843" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.5</t>
+          <t>dif_prob_mod_bm &gt; -1.0</t>
         </is>
       </c>
       <c r="Y843" t="inlineStr"/>
       <c r="Z843" t="n">
-        <v>2.653870142527809</v>
+        <v>3.32225706707945</v>
       </c>
       <c r="AA843" t="inlineStr">
         <is>
@@ -85529,12 +85563,12 @@
       </c>
       <c r="X844" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.5</t>
+          <t>dif_prob_mod_bm &gt; -1.0</t>
         </is>
       </c>
       <c r="Y844" t="inlineStr"/>
       <c r="Z844" t="n">
-        <v>2.515564885949821</v>
+        <v>3.09793141895397</v>
       </c>
       <c r="AA844" t="inlineStr">
         <is>
@@ -85629,12 +85663,12 @@
       </c>
       <c r="X845" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.5</t>
+          <t>dif_prob_mod_bm &gt; -1.0</t>
         </is>
       </c>
       <c r="Y845" t="inlineStr"/>
       <c r="Z845" t="n">
-        <v>1.446013068924971</v>
+        <v>1.375163007420573</v>
       </c>
       <c r="AA845" t="inlineStr">
         <is>
@@ -85729,12 +85763,12 @@
       </c>
       <c r="X846" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.5</t>
+          <t>dif_prob_mod_bm &gt; -1.0</t>
         </is>
       </c>
       <c r="Y846" t="inlineStr"/>
       <c r="Z846" t="n">
-        <v>1.690983536983486</v>
+        <v>0.7408139198286251</v>
       </c>
       <c r="AA846" t="inlineStr">
         <is>
@@ -85829,12 +85863,12 @@
       </c>
       <c r="X847" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.5</t>
+          <t>dif_prob_mod_bm &gt; -1.0</t>
         </is>
       </c>
       <c r="Y847" t="inlineStr"/>
       <c r="Z847" t="n">
-        <v>3.038453247862559</v>
+        <v>3.845025114000188</v>
       </c>
       <c r="AA847" t="inlineStr">
         <is>
@@ -85929,12 +85963,12 @@
       </c>
       <c r="X848" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.5</t>
+          <t>dif_prob_mod_bm &gt; -1.0</t>
         </is>
       </c>
       <c r="Y848" t="inlineStr"/>
       <c r="Z848" t="n">
-        <v>2.434336652629688</v>
+        <v>2.925603804976195</v>
       </c>
       <c r="AA848" t="inlineStr">
         <is>
@@ -86029,12 +86063,12 @@
       </c>
       <c r="X849" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.5</t>
+          <t>dif_prob_mod_bm &gt; -1.0</t>
         </is>
       </c>
       <c r="Y849" t="inlineStr"/>
       <c r="Z849" t="n">
-        <v>1.69144074184685</v>
+        <v>1.190501101732166</v>
       </c>
       <c r="AA849" t="inlineStr">
         <is>
@@ -86105,40 +86139,40 @@
         <v>2</v>
       </c>
       <c r="O850" t="n">
-        <v>0.3440873148248372</v>
+        <v>0.3676469729873349</v>
       </c>
       <c r="P850" t="n">
-        <v>0.2687155428411054</v>
+        <v>0.2249110818940491</v>
       </c>
       <c r="Q850" t="n">
-        <v>0.3871971423340574</v>
+        <v>0.407441945118616</v>
       </c>
       <c r="R850" t="n">
         <v>1</v>
       </c>
       <c r="S850" t="n">
-        <v>0.08275086814714927</v>
+        <v>0.1029956709317078</v>
       </c>
       <c r="T850" t="n">
         <v>2</v>
       </c>
       <c r="U850" t="n">
-        <v>0.08275086814714927</v>
+        <v>0.1029956709317078</v>
       </c>
       <c r="V850" t="n">
-        <v>0.3871971423340574</v>
+        <v>0.407441945118616</v>
       </c>
       <c r="W850" t="n">
         <v>3.1</v>
       </c>
       <c r="X850" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.5</t>
+          <t>dif_prob_mod_bm &gt; -1.0</t>
         </is>
       </c>
       <c r="Y850" t="inlineStr"/>
       <c r="Z850" t="n">
-        <v>9.486329987184407</v>
+        <v>9.778606682846783</v>
       </c>
       <c r="AA850" t="inlineStr">
         <is>
@@ -86205,40 +86239,40 @@
         <v>0</v>
       </c>
       <c r="O851" t="n">
-        <v>0.3048371867065628</v>
+        <v>0.2458557704484058</v>
       </c>
       <c r="P851" t="n">
-        <v>0.4695941977326032</v>
+        <v>0.4568542455458197</v>
       </c>
       <c r="Q851" t="n">
-        <v>0.2255686155608338</v>
+        <v>0.2972899840057746</v>
       </c>
       <c r="R851" t="n">
         <v>1</v>
       </c>
       <c r="S851" t="n">
-        <v>0.1984743549035266</v>
+        <v>0.185734402716743</v>
       </c>
       <c r="T851" t="n">
         <v>0</v>
       </c>
       <c r="U851" t="n">
-        <v>0.1984743549035266</v>
+        <v>0.185734402716743</v>
       </c>
       <c r="V851" t="n">
-        <v>0.4695941977326032</v>
+        <v>0.4568542455458197</v>
       </c>
       <c r="W851" t="n">
         <v>3.5</v>
       </c>
       <c r="X851" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.5</t>
+          <t>dif_prob_mod_bm &gt; -1.0</t>
         </is>
       </c>
       <c r="Y851" t="inlineStr"/>
       <c r="Z851" t="n">
-        <v>11.50505784444878</v>
+        <v>10.96450189309967</v>
       </c>
       <c r="AA851" t="inlineStr">
         <is>
@@ -86305,40 +86339,40 @@
         <v>2</v>
       </c>
       <c r="O852" t="n">
-        <v>0.0851109473078217</v>
+        <v>0.07871046675703819</v>
       </c>
       <c r="P852" t="n">
-        <v>0.2265154790824266</v>
+        <v>0.1787167095466377</v>
       </c>
       <c r="Q852" t="n">
-        <v>0.6883735736097517</v>
+        <v>0.7425728236963242</v>
       </c>
       <c r="R852" t="n">
         <v>1</v>
       </c>
       <c r="S852" t="n">
-        <v>0.03250527833625194</v>
+        <v>0.08670452842282439</v>
       </c>
       <c r="T852" t="n">
         <v>2</v>
       </c>
       <c r="U852" t="n">
-        <v>0.03250527833625194</v>
+        <v>0.08670452842282439</v>
       </c>
       <c r="V852" t="n">
-        <v>0.6883735736097517</v>
+        <v>0.7425728236963242</v>
       </c>
       <c r="W852" t="n">
         <v>1.44</v>
       </c>
       <c r="X852" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.5</t>
+          <t>dif_prob_mod_bm &gt; -1.0</t>
         </is>
       </c>
       <c r="Y852" t="inlineStr"/>
       <c r="Z852" t="n">
-        <v>16.86515255343892</v>
+        <v>17.82174776871178</v>
       </c>
       <c r="AA852" t="inlineStr">
         <is>
@@ -86402,43 +86436,43 @@
         <v>0.05303030303030298</v>
       </c>
       <c r="N853" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O853" t="n">
-        <v>0.274270355239342</v>
+        <v>0.3531592641477292</v>
       </c>
       <c r="P853" t="n">
-        <v>0.398227382239566</v>
+        <v>0.3418092762478577</v>
       </c>
       <c r="Q853" t="n">
-        <v>0.327502262521092</v>
+        <v>0.3050314596044131</v>
       </c>
       <c r="R853" t="n">
         <v>1</v>
       </c>
       <c r="S853" t="n">
-        <v>0.1104575980669041</v>
+        <v>0.03661250155780121</v>
       </c>
       <c r="T853" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U853" t="n">
-        <v>0.1104575980669041</v>
+        <v>0.03661250155780121</v>
       </c>
       <c r="V853" t="n">
-        <v>0.398227382239566</v>
+        <v>0.3531592641477292</v>
       </c>
       <c r="W853" t="n">
-        <v>3.3</v>
+        <v>3</v>
       </c>
       <c r="X853" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.5</t>
+          <t>dif_prob_mod_bm &gt; -1.0</t>
         </is>
       </c>
       <c r="Y853" t="inlineStr"/>
       <c r="Z853" t="n">
-        <v>9.756570864869367</v>
+        <v>8.475822339545502</v>
       </c>
       <c r="AA853" t="inlineStr">
         <is>
@@ -86502,43 +86536,43 @@
         <v>0.05273937532002027</v>
       </c>
       <c r="N854" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O854" t="n">
-        <v>0.2299324461228716</v>
+        <v>0.2492848668078031</v>
       </c>
       <c r="P854" t="n">
-        <v>0.4415438193210025</v>
+        <v>0.3686379664055513</v>
       </c>
       <c r="Q854" t="n">
-        <v>0.328523734556126</v>
+        <v>0.3820771667866456</v>
       </c>
       <c r="R854" t="n">
         <v>1</v>
       </c>
       <c r="S854" t="n">
-        <v>0.1351235858579674</v>
+        <v>0.1106763885765288</v>
       </c>
       <c r="T854" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="U854" t="n">
-        <v>0.1351235858579674</v>
+        <v>0.1106763885765288</v>
       </c>
       <c r="V854" t="n">
-        <v>0.4415438193210025</v>
+        <v>0.3820771667866456</v>
       </c>
       <c r="W854" t="n">
-        <v>3.1</v>
+        <v>3.5</v>
       </c>
       <c r="X854" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.5</t>
+          <t>dif_prob_mod_bm &gt; -1.0</t>
         </is>
       </c>
       <c r="Y854" t="inlineStr"/>
       <c r="Z854" t="n">
-        <v>10.81782357336456</v>
+        <v>9.169852002879493</v>
       </c>
       <c r="AA854" t="inlineStr">
         <is>
@@ -86605,40 +86639,40 @@
         <v>1</v>
       </c>
       <c r="O855" t="n">
-        <v>0.7260686221236928</v>
+        <v>0.6478128035818833</v>
       </c>
       <c r="P855" t="n">
-        <v>0.1901469942527821</v>
+        <v>0.2675424415706188</v>
       </c>
       <c r="Q855" t="n">
-        <v>0.0837843836235251</v>
+        <v>0.08464475484749796</v>
       </c>
       <c r="R855" t="n">
         <v>1</v>
       </c>
       <c r="S855" t="n">
-        <v>-0.01667276882836655</v>
+        <v>-0.09492858737017607</v>
       </c>
       <c r="T855" t="n">
         <v>1</v>
       </c>
       <c r="U855" t="n">
-        <v>-0.01667276882836655</v>
+        <v>-0.09492858737017607</v>
       </c>
       <c r="V855" t="n">
-        <v>0.7260686221236928</v>
+        <v>0.6478128035818833</v>
       </c>
       <c r="W855" t="n">
         <v>1.27</v>
       </c>
       <c r="X855" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.5</t>
+          <t>dif_prob_mod_bm &gt; -1.0</t>
         </is>
       </c>
       <c r="Y855" t="inlineStr"/>
       <c r="Z855" t="n">
-        <v>17.78868124203047</v>
+        <v>10.99093509219675</v>
       </c>
       <c r="AA855" t="inlineStr">
         <is>
@@ -86702,43 +86736,43 @@
         <v>0.05394605394605412</v>
       </c>
       <c r="N856" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O856" t="n">
-        <v>0.32230391206242</v>
+        <v>0.4609246386828041</v>
       </c>
       <c r="P856" t="n">
-        <v>0.4348347032098798</v>
+        <v>0.3254621602832685</v>
       </c>
       <c r="Q856" t="n">
-        <v>0.2428613847277002</v>
+        <v>0.2136132010339273</v>
       </c>
       <c r="R856" t="n">
         <v>1</v>
       </c>
       <c r="S856" t="n">
-        <v>0.1473149559744928</v>
+        <v>-0.02564724125400475</v>
       </c>
       <c r="T856" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U856" t="n">
-        <v>0.1473149559744928</v>
+        <v>-0.02564724125400475</v>
       </c>
       <c r="V856" t="n">
-        <v>0.4348347032098798</v>
+        <v>0.4609246386828041</v>
       </c>
       <c r="W856" t="n">
-        <v>3.3</v>
+        <v>1.95</v>
       </c>
       <c r="X856" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.5</t>
+          <t>dif_prob_mod_bm &gt; -1.0</t>
         </is>
       </c>
       <c r="Y856" t="inlineStr"/>
       <c r="Z856" t="n">
-        <v>10.65345022864206</v>
+        <v>9.83112374819507</v>
       </c>
       <c r="AA856" t="inlineStr">
         <is>
@@ -86805,40 +86839,40 @@
         <v>1</v>
       </c>
       <c r="O857" t="n">
-        <v>0.4869844459100298</v>
+        <v>0.4448480976423265</v>
       </c>
       <c r="P857" t="n">
-        <v>0.3771867718088371</v>
+        <v>0.3923345053144631</v>
       </c>
       <c r="Q857" t="n">
-        <v>0.1358287822811332</v>
+        <v>0.1628173970432104</v>
       </c>
       <c r="R857" t="n">
         <v>1</v>
       </c>
       <c r="S857" t="n">
-        <v>0.06413174478294081</v>
+        <v>0.02199539651523758</v>
       </c>
       <c r="T857" t="n">
         <v>1</v>
       </c>
       <c r="U857" t="n">
-        <v>0.06413174478294081</v>
+        <v>0.02199539651523758</v>
       </c>
       <c r="V857" t="n">
-        <v>0.4869844459100298</v>
+        <v>0.4448480976423265</v>
       </c>
       <c r="W857" t="n">
         <v>2.25</v>
       </c>
       <c r="X857" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.5</t>
+          <t>dif_prob_mod_bm &gt; -1.0</t>
         </is>
       </c>
       <c r="Y857" t="inlineStr"/>
       <c r="Z857" t="n">
-        <v>11.93111892479573</v>
+        <v>10.67635434341584</v>
       </c>
       <c r="AA857" t="inlineStr">
         <is>
@@ -86905,40 +86939,40 @@
         <v>0</v>
       </c>
       <c r="O858" t="n">
-        <v>0.3091142152748929</v>
+        <v>0.3394023454810446</v>
       </c>
       <c r="P858" t="n">
-        <v>0.4610007247819783</v>
+        <v>0.4132490180980417</v>
       </c>
       <c r="Q858" t="n">
-        <v>0.2298850599431289</v>
+        <v>0.2473486364209138</v>
       </c>
       <c r="R858" t="n">
         <v>1</v>
       </c>
       <c r="S858" t="n">
-        <v>0.2056687932710141</v>
+        <v>0.1579170865870775</v>
       </c>
       <c r="T858" t="n">
         <v>0</v>
       </c>
       <c r="U858" t="n">
-        <v>0.2056687932710141</v>
+        <v>0.1579170865870775</v>
       </c>
       <c r="V858" t="n">
-        <v>0.4610007247819783</v>
+        <v>0.4132490180980417</v>
       </c>
       <c r="W858" t="n">
         <v>3.7</v>
       </c>
       <c r="X858" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.5</t>
+          <t>dif_prob_mod_bm &gt; -1.0</t>
         </is>
       </c>
       <c r="Y858" t="inlineStr"/>
       <c r="Z858" t="n">
-        <v>5.647258878579235</v>
+        <v>4.958988217176501</v>
       </c>
       <c r="AA858" t="inlineStr">
         <is>
@@ -87009,40 +87043,40 @@
         <v>1</v>
       </c>
       <c r="O859" t="n">
-        <v>0.4296073297505719</v>
+        <v>0.4495162961494563</v>
       </c>
       <c r="P859" t="n">
-        <v>0.4035337602264751</v>
+        <v>0.3626157658589798</v>
       </c>
       <c r="Q859" t="n">
-        <v>0.1668589100229531</v>
+        <v>0.1878679379915639</v>
       </c>
       <c r="R859" t="n">
         <v>1</v>
       </c>
       <c r="S859" t="n">
-        <v>-0.2032482380553818</v>
+        <v>-0.1833392716564974</v>
       </c>
       <c r="T859" t="n">
         <v>1</v>
       </c>
       <c r="U859" t="n">
-        <v>-0.2032482380553818</v>
+        <v>-0.1833392716564974</v>
       </c>
       <c r="V859" t="n">
-        <v>0.4296073297505719</v>
+        <v>0.4495162961494563</v>
       </c>
       <c r="W859" t="n">
         <v>1.5</v>
       </c>
       <c r="X859" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.5</t>
+          <t>dif_prob_mod_bm &gt; -1.0</t>
         </is>
       </c>
       <c r="Y859" t="inlineStr"/>
       <c r="Z859" t="n">
-        <v>10.52537957888901</v>
+        <v>1.988106068075076</v>
       </c>
       <c r="AA859" t="inlineStr">
         <is>
@@ -87109,40 +87143,40 @@
         <v>2</v>
       </c>
       <c r="O860" t="n">
-        <v>0.2721475794665427</v>
+        <v>0.2966831996760659</v>
       </c>
       <c r="P860" t="n">
-        <v>0.2667752538905723</v>
+        <v>0.2716022204369036</v>
       </c>
       <c r="Q860" t="n">
-        <v>0.4610771666428851</v>
+        <v>0.4317145798870305</v>
       </c>
       <c r="R860" t="n">
         <v>1</v>
       </c>
       <c r="S860" t="n">
-        <v>0.1476443308219896</v>
+        <v>0.118281744066135</v>
       </c>
       <c r="T860" t="n">
         <v>2</v>
       </c>
       <c r="U860" t="n">
-        <v>0.1476443308219896</v>
+        <v>0.118281744066135</v>
       </c>
       <c r="V860" t="n">
-        <v>0.4610771666428851</v>
+        <v>0.4317145798870305</v>
       </c>
       <c r="W860" t="n">
         <v>3</v>
       </c>
       <c r="X860" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.5</t>
+          <t>dif_prob_mod_bm &gt; -1.0</t>
         </is>
       </c>
       <c r="Y860" t="inlineStr"/>
       <c r="Z860" t="n">
-        <v>11.29639058275068</v>
+        <v>10.36114991728873</v>
       </c>
       <c r="AA860" t="inlineStr">
         <is>
@@ -87209,40 +87243,40 @@
         <v>2</v>
       </c>
       <c r="O861" t="n">
-        <v>0.1345738992701279</v>
+        <v>0.1627928510829592</v>
       </c>
       <c r="P861" t="n">
-        <v>0.1464733013085174</v>
+        <v>0.2370145136145586</v>
       </c>
       <c r="Q861" t="n">
-        <v>0.7189527994213547</v>
+        <v>0.6001926353024822</v>
       </c>
       <c r="R861" t="n">
         <v>1</v>
       </c>
       <c r="S861" t="n">
-        <v>0.3230137131269384</v>
+        <v>0.204253549008066</v>
       </c>
       <c r="T861" t="n">
         <v>2</v>
       </c>
       <c r="U861" t="n">
-        <v>0.3230137131269384</v>
+        <v>0.204253549008066</v>
       </c>
       <c r="V861" t="n">
-        <v>0.7189527994213547</v>
+        <v>0.6001926353024822</v>
       </c>
       <c r="W861" t="n">
         <v>2.38</v>
       </c>
       <c r="X861" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.5</t>
+          <t>dif_prob_mod_bm &gt; -1.0</t>
         </is>
       </c>
       <c r="Y861" t="inlineStr"/>
       <c r="Z861" t="n">
-        <v>17.61434358582319</v>
+        <v>14.40462324725957</v>
       </c>
       <c r="AA861" t="inlineStr">
         <is>
@@ -87309,40 +87343,40 @@
         <v>1</v>
       </c>
       <c r="O862" t="n">
-        <v>0.430063021484079</v>
+        <v>0.4655900543342097</v>
       </c>
       <c r="P862" t="n">
-        <v>0.3067831530109094</v>
+        <v>0.3139843299514171</v>
       </c>
       <c r="Q862" t="n">
-        <v>0.2631538255050116</v>
+        <v>0.2204256157143731</v>
       </c>
       <c r="R862" t="n">
         <v>1</v>
       </c>
       <c r="S862" t="n">
-        <v>0.08813419219062879</v>
+        <v>0.1236612250407595</v>
       </c>
       <c r="T862" t="n">
         <v>1</v>
       </c>
       <c r="U862" t="n">
-        <v>0.08813419219062879</v>
+        <v>0.1236612250407595</v>
       </c>
       <c r="V862" t="n">
-        <v>0.430063021484079</v>
+        <v>0.4655900543342097</v>
       </c>
       <c r="W862" t="n">
         <v>2.75</v>
       </c>
       <c r="X862" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.5</t>
+          <t>dif_prob_mod_bm &gt; -1.0</t>
         </is>
       </c>
       <c r="Y862" t="inlineStr"/>
       <c r="Z862" t="n">
-        <v>10.53654402635994</v>
+        <v>11.17416130402103</v>
       </c>
       <c r="AA862" t="inlineStr">
         <is>
@@ -87409,40 +87443,40 @@
         <v>0</v>
       </c>
       <c r="O863" t="n">
-        <v>0.1937504311976685</v>
+        <v>0.2879965528448061</v>
       </c>
       <c r="P863" t="n">
-        <v>0.4372403611960575</v>
+        <v>0.3855928237766273</v>
       </c>
       <c r="Q863" t="n">
-        <v>0.369009207606274</v>
+        <v>0.3264106233785666</v>
       </c>
       <c r="R863" t="n">
         <v>1</v>
       </c>
       <c r="S863" t="n">
-        <v>0.1535934726287637</v>
+        <v>0.1019459352093336</v>
       </c>
       <c r="T863" t="n">
         <v>0</v>
       </c>
       <c r="U863" t="n">
-        <v>0.1535934726287637</v>
+        <v>0.1019459352093336</v>
       </c>
       <c r="V863" t="n">
-        <v>0.4372403611960575</v>
+        <v>0.3855928237766273</v>
       </c>
       <c r="W863" t="n">
         <v>3.3</v>
       </c>
       <c r="X863" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.5</t>
+          <t>dif_prob_mod_bm &gt; -1.0</t>
         </is>
       </c>
       <c r="Y863" t="inlineStr"/>
       <c r="Z863" t="n">
-        <v>10.71238884930341</v>
+        <v>9.254227770639057</v>
       </c>
       <c r="AA863" t="inlineStr">
         <is>
@@ -87509,40 +87543,40 @@
         <v>2</v>
       </c>
       <c r="O864" t="n">
-        <v>0.3361838870050958</v>
+        <v>0.336086963244507</v>
       </c>
       <c r="P864" t="n">
-        <v>0.2433854322236544</v>
+        <v>0.2619519997150369</v>
       </c>
       <c r="Q864" t="n">
-        <v>0.4204306807712498</v>
+        <v>0.401961037040456</v>
       </c>
       <c r="R864" t="n">
         <v>1</v>
       </c>
       <c r="S864" t="n">
-        <v>0.09825759169986642</v>
+        <v>0.07978794796907263</v>
       </c>
       <c r="T864" t="n">
         <v>2</v>
       </c>
       <c r="U864" t="n">
-        <v>0.09825759169986642</v>
+        <v>0.07978794796907263</v>
       </c>
       <c r="V864" t="n">
-        <v>0.4204306807712498</v>
+        <v>0.401961037040456</v>
       </c>
       <c r="W864" t="n">
         <v>2.9</v>
       </c>
       <c r="X864" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.5</t>
+          <t>dif_prob_mod_bm &gt; -1.0</t>
         </is>
       </c>
       <c r="Y864" t="inlineStr"/>
       <c r="Z864" t="n">
-        <v>10.30055167889562</v>
+        <v>9.647064888970945</v>
       </c>
       <c r="AA864" t="inlineStr">
         <is>
@@ -87609,40 +87643,40 @@
         <v>0</v>
       </c>
       <c r="O865" t="n">
-        <v>0.1924504782199172</v>
+        <v>0.218999075991924</v>
       </c>
       <c r="P865" t="n">
-        <v>0.439738160486175</v>
+        <v>0.4096057548849228</v>
       </c>
       <c r="Q865" t="n">
-        <v>0.3678113612939078</v>
+        <v>0.3713951691231532</v>
       </c>
       <c r="R865" t="n">
         <v>1</v>
       </c>
       <c r="S865" t="n">
-        <v>0.1561646734544748</v>
+        <v>0.1260322678532226</v>
       </c>
       <c r="T865" t="n">
         <v>0</v>
       </c>
       <c r="U865" t="n">
-        <v>0.1561646734544748</v>
+        <v>0.1260322678532226</v>
       </c>
       <c r="V865" t="n">
-        <v>0.439738160486175</v>
+        <v>0.4096057548849228</v>
       </c>
       <c r="W865" t="n">
         <v>3.3</v>
       </c>
       <c r="X865" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.5</t>
+          <t>dif_prob_mod_bm &gt; -1.0</t>
         </is>
       </c>
       <c r="Y865" t="inlineStr"/>
       <c r="Z865" t="n">
-        <v>10.77358493191129</v>
+        <v>9.830538117238149</v>
       </c>
       <c r="AA865" t="inlineStr">
         <is>
@@ -87709,40 +87743,40 @@
         <v>2</v>
       </c>
       <c r="O866" t="n">
-        <v>0.2824774203563148</v>
+        <v>0.3655134793720591</v>
       </c>
       <c r="P866" t="n">
-        <v>0.2236739731754825</v>
+        <v>0.2330284447336559</v>
       </c>
       <c r="Q866" t="n">
-        <v>0.4938486064682027</v>
+        <v>0.401458075894285</v>
       </c>
       <c r="R866" t="n">
         <v>1</v>
       </c>
       <c r="S866" t="n">
-        <v>0.1574924646710057</v>
+        <v>0.06510193409708798</v>
       </c>
       <c r="T866" t="n">
         <v>2</v>
       </c>
       <c r="U866" t="n">
-        <v>0.1574924646710057</v>
+        <v>0.06510193409708798</v>
       </c>
       <c r="V866" t="n">
-        <v>0.4938486064682027</v>
+        <v>0.401458075894285</v>
       </c>
       <c r="W866" t="n">
         <v>2.8</v>
       </c>
       <c r="X866" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &gt; -0.5</t>
+          <t>dif_prob_mod_bm &gt; -1.0</t>
         </is>
       </c>
       <c r="Y866" t="inlineStr"/>
       <c r="Z866" t="n">
-        <v>12.09929085847097</v>
+        <v>9.634993821462841</v>
       </c>
       <c r="AA866" t="inlineStr">
         <is>
@@ -87795,13 +87829,13 @@
         <v>0</v>
       </c>
       <c r="O867" t="n">
-        <v>0.3391783540016225</v>
+        <v>0.4109397757775142</v>
       </c>
       <c r="P867" t="n">
-        <v>0.4945874731952484</v>
+        <v>0.418740116585585</v>
       </c>
       <c r="Q867" t="n">
-        <v>0.1662341728031292</v>
+        <v>0.1703201076369009</v>
       </c>
       <c r="R867" t="n">
         <v>1</v>
@@ -87812,12 +87846,12 @@
       </c>
       <c r="U867" t="inlineStr"/>
       <c r="V867" t="n">
-        <v>0.5054125268047516</v>
+        <v>0.5812598834144149</v>
       </c>
       <c r="W867" t="inlineStr"/>
       <c r="X867" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &lt; -0.5</t>
+          <t>dif_prob_mod_bm &lt; -1.0</t>
         </is>
       </c>
       <c r="Y867" t="inlineStr"/>
@@ -87877,13 +87911,13 @@
         <v>2</v>
       </c>
       <c r="O868" t="n">
-        <v>0.2137960003870185</v>
+        <v>0.3098099887795165</v>
       </c>
       <c r="P868" t="n">
-        <v>0.388320665497163</v>
+        <v>0.3249086187794775</v>
       </c>
       <c r="Q868" t="n">
-        <v>0.3978833341158185</v>
+        <v>0.3652813924410062</v>
       </c>
       <c r="R868" t="n">
         <v>1</v>
@@ -87894,12 +87928,12 @@
       </c>
       <c r="U868" t="inlineStr"/>
       <c r="V868" t="n">
-        <v>0.6021166658841814</v>
+        <v>0.6347186075589939</v>
       </c>
       <c r="W868" t="inlineStr"/>
       <c r="X868" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &lt; -0.5</t>
+          <t>dif_prob_mod_bm &lt; -1.0</t>
         </is>
       </c>
       <c r="Y868" t="inlineStr"/>
@@ -87955,13 +87989,13 @@
         <v>2</v>
       </c>
       <c r="O869" t="n">
-        <v>0.1180938319134574</v>
+        <v>0.1380744936353678</v>
       </c>
       <c r="P869" t="n">
-        <v>0.3336586052369478</v>
+        <v>0.3248414581756698</v>
       </c>
       <c r="Q869" t="n">
-        <v>0.5482475628495947</v>
+        <v>0.5370840481889624</v>
       </c>
       <c r="R869" t="n">
         <v>1</v>
@@ -87972,12 +88006,12 @@
       </c>
       <c r="U869" t="inlineStr"/>
       <c r="V869" t="n">
-        <v>0.4517524371504053</v>
+        <v>0.4629159518110376</v>
       </c>
       <c r="W869" t="inlineStr"/>
       <c r="X869" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &lt; -0.5</t>
+          <t>dif_prob_mod_bm &lt; -1.0</t>
         </is>
       </c>
       <c r="Y869" t="inlineStr"/>
@@ -88033,13 +88067,13 @@
         <v>2</v>
       </c>
       <c r="O870" t="n">
-        <v>0.1112147264717963</v>
+        <v>0.1276617308838463</v>
       </c>
       <c r="P870" t="n">
-        <v>0.3161193156961487</v>
+        <v>0.3320262717579585</v>
       </c>
       <c r="Q870" t="n">
-        <v>0.572665957832055</v>
+        <v>0.5403119973581952</v>
       </c>
       <c r="R870" t="n">
         <v>1</v>
@@ -88050,12 +88084,12 @@
       </c>
       <c r="U870" t="inlineStr"/>
       <c r="V870" t="n">
-        <v>0.427334042167945</v>
+        <v>0.4596880026418048</v>
       </c>
       <c r="W870" t="inlineStr"/>
       <c r="X870" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &lt; -0.5</t>
+          <t>dif_prob_mod_bm &lt; -1.0</t>
         </is>
       </c>
       <c r="Y870" t="inlineStr"/>
@@ -88111,13 +88145,13 @@
         <v>1</v>
       </c>
       <c r="O871" t="n">
-        <v>0.5691994738121433</v>
+        <v>0.6270696053784655</v>
       </c>
       <c r="P871" t="n">
-        <v>0.3295675708489639</v>
+        <v>0.2860697369253029</v>
       </c>
       <c r="Q871" t="n">
-        <v>0.1012329553388928</v>
+        <v>0.08686065769623169</v>
       </c>
       <c r="R871" t="n">
         <v>1</v>
@@ -88128,12 +88162,12 @@
       </c>
       <c r="U871" t="inlineStr"/>
       <c r="V871" t="n">
-        <v>0.4308005261878567</v>
+        <v>0.3729303946215345</v>
       </c>
       <c r="W871" t="inlineStr"/>
       <c r="X871" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &lt; -0.5</t>
+          <t>dif_prob_mod_bm &lt; -1.0</t>
         </is>
       </c>
       <c r="Y871" t="inlineStr"/>
@@ -88189,13 +88223,13 @@
         <v>2</v>
       </c>
       <c r="O872" t="n">
-        <v>0.1208030197510242</v>
+        <v>0.1596599583679663</v>
       </c>
       <c r="P872" t="n">
-        <v>0.3528388441179133</v>
+        <v>0.3488294693298283</v>
       </c>
       <c r="Q872" t="n">
-        <v>0.5263581361310625</v>
+        <v>0.4915105723022052</v>
       </c>
       <c r="R872" t="n">
         <v>1</v>
@@ -88206,12 +88240,12 @@
       </c>
       <c r="U872" t="inlineStr"/>
       <c r="V872" t="n">
-        <v>0.4736418638689375</v>
+        <v>0.5084894276977947</v>
       </c>
       <c r="W872" t="inlineStr"/>
       <c r="X872" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &lt; -0.5</t>
+          <t>dif_prob_mod_bm &lt; -1.0</t>
         </is>
       </c>
       <c r="Y872" t="inlineStr"/>
@@ -88267,13 +88301,13 @@
         <v>2</v>
       </c>
       <c r="O873" t="n">
-        <v>0.03874120732801711</v>
+        <v>0.04453653348987016</v>
       </c>
       <c r="P873" t="n">
-        <v>0.1747535027917853</v>
+        <v>0.1902896090967515</v>
       </c>
       <c r="Q873" t="n">
-        <v>0.7865052898801975</v>
+        <v>0.7651738574133784</v>
       </c>
       <c r="R873" t="n">
         <v>1</v>
@@ -88284,12 +88318,12 @@
       </c>
       <c r="U873" t="inlineStr"/>
       <c r="V873" t="n">
-        <v>0.2134947101198025</v>
+        <v>0.2348261425866216</v>
       </c>
       <c r="W873" t="inlineStr"/>
       <c r="X873" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &lt; -0.5</t>
+          <t>dif_prob_mod_bm &lt; -1.0</t>
         </is>
       </c>
       <c r="Y873" t="inlineStr"/>
@@ -88345,13 +88379,13 @@
         <v>0</v>
       </c>
       <c r="O874" t="n">
-        <v>0.2155786560732419</v>
+        <v>0.1838963941735427</v>
       </c>
       <c r="P874" t="n">
-        <v>0.5815166255119247</v>
+        <v>0.5290742664934772</v>
       </c>
       <c r="Q874" t="n">
-        <v>0.2029047184148335</v>
+        <v>0.2870293393329801</v>
       </c>
       <c r="R874" t="n">
         <v>1</v>
@@ -88362,12 +88396,12 @@
       </c>
       <c r="U874" t="inlineStr"/>
       <c r="V874" t="n">
-        <v>0.4184833744880753</v>
+        <v>0.4709257335065228</v>
       </c>
       <c r="W874" t="inlineStr"/>
       <c r="X874" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &lt; -0.5</t>
+          <t>dif_prob_mod_bm &lt; -1.0</t>
         </is>
       </c>
       <c r="Y874" t="inlineStr"/>
@@ -88423,13 +88457,13 @@
         <v>1</v>
       </c>
       <c r="O875" t="n">
-        <v>0.6568537610122002</v>
+        <v>0.6273946584020182</v>
       </c>
       <c r="P875" t="n">
-        <v>0.2210519216483076</v>
+        <v>0.2663504598488211</v>
       </c>
       <c r="Q875" t="n">
-        <v>0.1220943173394922</v>
+        <v>0.1062548817491607</v>
       </c>
       <c r="R875" t="n">
         <v>1</v>
@@ -88440,12 +88474,12 @@
       </c>
       <c r="U875" t="inlineStr"/>
       <c r="V875" t="n">
-        <v>0.3431462389877998</v>
+        <v>0.3726053415979818</v>
       </c>
       <c r="W875" t="inlineStr"/>
       <c r="X875" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &lt; -0.5</t>
+          <t>dif_prob_mod_bm &lt; -1.0</t>
         </is>
       </c>
       <c r="Y875" t="inlineStr"/>
@@ -88501,13 +88535,13 @@
         <v>2</v>
       </c>
       <c r="O876" t="n">
-        <v>0.1393678962107191</v>
+        <v>0.208709238623122</v>
       </c>
       <c r="P876" t="n">
-        <v>0.4033691373400079</v>
+        <v>0.3643242918407215</v>
       </c>
       <c r="Q876" t="n">
-        <v>0.4572629664492731</v>
+        <v>0.4269664695361565</v>
       </c>
       <c r="R876" t="n">
         <v>1</v>
@@ -88518,12 +88552,12 @@
       </c>
       <c r="U876" t="inlineStr"/>
       <c r="V876" t="n">
-        <v>0.5427370335507269</v>
+        <v>0.5730335304638435</v>
       </c>
       <c r="W876" t="inlineStr"/>
       <c r="X876" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &lt; -0.5</t>
+          <t>dif_prob_mod_bm &lt; -1.0</t>
         </is>
       </c>
       <c r="Y876" t="inlineStr"/>
@@ -88579,13 +88613,13 @@
         <v>0</v>
       </c>
       <c r="O877" t="n">
-        <v>0.3368799197219474</v>
+        <v>0.276100083134881</v>
       </c>
       <c r="P877" t="n">
-        <v>0.4143000112375599</v>
+        <v>0.4374145077284339</v>
       </c>
       <c r="Q877" t="n">
-        <v>0.2488200690404928</v>
+        <v>0.286485409136685</v>
       </c>
       <c r="R877" t="n">
         <v>1</v>
@@ -88596,12 +88630,12 @@
       </c>
       <c r="U877" t="inlineStr"/>
       <c r="V877" t="n">
-        <v>0.5856999887624401</v>
+        <v>0.5625854922715661</v>
       </c>
       <c r="W877" t="inlineStr"/>
       <c r="X877" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &lt; -0.5</t>
+          <t>dif_prob_mod_bm &lt; -1.0</t>
         </is>
       </c>
       <c r="Y877" t="inlineStr"/>
@@ -88661,13 +88695,13 @@
         <v>2</v>
       </c>
       <c r="O878" t="n">
-        <v>0.2458980743264169</v>
+        <v>0.2360517103918542</v>
       </c>
       <c r="P878" t="n">
-        <v>0.3743154144067939</v>
+        <v>0.3776250296704443</v>
       </c>
       <c r="Q878" t="n">
-        <v>0.379786511266789</v>
+        <v>0.3863232599377014</v>
       </c>
       <c r="R878" t="n">
         <v>1</v>
@@ -88678,12 +88712,12 @@
       </c>
       <c r="U878" t="inlineStr"/>
       <c r="V878" t="n">
-        <v>0.6202134887332109</v>
+        <v>0.6136767400622986</v>
       </c>
       <c r="W878" t="inlineStr"/>
       <c r="X878" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &lt; -0.5</t>
+          <t>dif_prob_mod_bm &lt; -1.0</t>
         </is>
       </c>
       <c r="Y878" t="inlineStr"/>
@@ -88739,13 +88773,13 @@
         <v>1</v>
       </c>
       <c r="O879" t="n">
-        <v>0.6193001145614184</v>
+        <v>0.6102912445334016</v>
       </c>
       <c r="P879" t="n">
-        <v>0.2777642252060036</v>
+        <v>0.2760987472780031</v>
       </c>
       <c r="Q879" t="n">
-        <v>0.1029356602325779</v>
+        <v>0.1136100081885953</v>
       </c>
       <c r="R879" t="n">
         <v>1</v>
@@ -88756,12 +88790,12 @@
       </c>
       <c r="U879" t="inlineStr"/>
       <c r="V879" t="n">
-        <v>0.3806998854385816</v>
+        <v>0.3897087554665984</v>
       </c>
       <c r="W879" t="inlineStr"/>
       <c r="X879" t="inlineStr">
         <is>
-          <t>dif_prob_mod_bm &lt; -0.5</t>
+          <t>dif_prob_mod_bm &lt; -1.0</t>
         </is>
       </c>
       <c r="Y879" t="inlineStr"/>
@@ -88831,28 +88865,28 @@
         <v>2</v>
       </c>
       <c r="O880" t="n">
-        <v>0.03811898036937345</v>
+        <v>0.0707914076409339</v>
       </c>
       <c r="P880" t="n">
-        <v>0.1788715898358706</v>
+        <v>0.1783465591759244</v>
       </c>
       <c r="Q880" t="n">
-        <v>0.783009429794756</v>
+        <v>0.7508620331831417</v>
       </c>
       <c r="R880" t="n">
         <v>1</v>
       </c>
       <c r="S880" t="n">
-        <v>0.1239912867851508</v>
+        <v>0.09184389017353656</v>
       </c>
       <c r="T880" t="n">
         <v>2</v>
       </c>
       <c r="U880" t="n">
-        <v>0.1239912867851508</v>
+        <v>0.09184389017353656</v>
       </c>
       <c r="V880" t="n">
-        <v>0.783009429794756</v>
+        <v>0.7508620331831417</v>
       </c>
       <c r="W880" t="n">
         <v>1.42</v>
@@ -88864,7 +88898,7 @@
       </c>
       <c r="Y880" t="inlineStr"/>
       <c r="Z880" t="n">
-        <v>8.221599012844937</v>
+        <v>6.709425563263728</v>
       </c>
       <c r="AA880" t="inlineStr">
         <is>
@@ -88935,28 +88969,28 @@
         <v>1</v>
       </c>
       <c r="O881" t="n">
-        <v>0.4161961383603509</v>
+        <v>0.3960788972176367</v>
       </c>
       <c r="P881" t="n">
-        <v>0.2693827774091418</v>
+        <v>0.2880414706184566</v>
       </c>
       <c r="Q881" t="n">
-        <v>0.3144210842305072</v>
+        <v>0.3158796321639066</v>
       </c>
       <c r="R881" t="n">
         <v>1</v>
       </c>
       <c r="S881" t="n">
-        <v>0.07953778424563773</v>
+        <v>0.05942054310292355</v>
       </c>
       <c r="T881" t="n">
         <v>1</v>
       </c>
       <c r="U881" t="n">
-        <v>0.07953778424563773</v>
+        <v>0.05942054310292355</v>
       </c>
       <c r="V881" t="n">
-        <v>0.4161961383603509</v>
+        <v>0.3960788972176367</v>
       </c>
       <c r="W881" t="n">
         <v>2.8</v>
@@ -88968,7 +89002,7 @@
       </c>
       <c r="Y881" t="inlineStr"/>
       <c r="Z881" t="n">
-        <v>4.370059452783685</v>
+        <v>3.802566417775986</v>
       </c>
       <c r="AA881" t="inlineStr">
         <is>
@@ -89039,28 +89073,28 @@
         <v>0</v>
       </c>
       <c r="O882" t="n">
-        <v>0.2619084320149278</v>
+        <v>0.2674026617077316</v>
       </c>
       <c r="P882" t="n">
-        <v>0.428527354889611</v>
+        <v>0.3688893929576748</v>
       </c>
       <c r="Q882" t="n">
-        <v>0.3095642130954612</v>
+        <v>0.3637079453345937</v>
       </c>
       <c r="R882" t="n">
         <v>1</v>
       </c>
       <c r="S882" t="n">
-        <v>0.1232230785738215</v>
+        <v>0.06358511664188532</v>
       </c>
       <c r="T882" t="n">
         <v>0</v>
       </c>
       <c r="U882" t="n">
-        <v>0.1232230785738215</v>
+        <v>0.06358511664188532</v>
       </c>
       <c r="V882" t="n">
-        <v>0.428527354889611</v>
+        <v>0.3688893929576748</v>
       </c>
       <c r="W882" t="n">
         <v>3.1</v>
@@ -89072,7 +89106,7 @@
       </c>
       <c r="Y882" t="inlineStr"/>
       <c r="Z882" t="n">
-        <v>4.499537226340915</v>
+        <v>3.739379157151296</v>
       </c>
       <c r="AA882" t="inlineStr">
         <is>
@@ -89143,28 +89177,28 @@
         <v>2</v>
       </c>
       <c r="O883" t="n">
-        <v>0.2102772783881113</v>
+        <v>0.171113592847635</v>
       </c>
       <c r="P883" t="n">
-        <v>0.2462328506220107</v>
+        <v>0.3508545619476816</v>
       </c>
       <c r="Q883" t="n">
-        <v>0.543489870989878</v>
+        <v>0.4780318452046833</v>
       </c>
       <c r="R883" t="n">
         <v>1</v>
       </c>
       <c r="S883" t="n">
-        <v>0.02909917901192327</v>
+        <v>-0.03635884677327139</v>
       </c>
       <c r="T883" t="n">
         <v>2</v>
       </c>
       <c r="U883" t="n">
-        <v>0.02909917901192327</v>
+        <v>-0.03635884677327139</v>
       </c>
       <c r="V883" t="n">
-        <v>0.543489870989878</v>
+        <v>0.4780318452046833</v>
       </c>
       <c r="W883" t="n">
         <v>1.83</v>
@@ -89176,7 +89210,7 @@
       </c>
       <c r="Y883" t="inlineStr"/>
       <c r="Z883" t="n">
-        <v>5.706643645393719</v>
+        <v>1.995578748669587</v>
       </c>
       <c r="AA883" t="inlineStr">
         <is>
@@ -89244,34 +89278,34 @@
         <v>0.06038552321007096</v>
       </c>
       <c r="N884" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O884" t="n">
-        <v>0.3516254837645627</v>
+        <v>0.3307142913162338</v>
       </c>
       <c r="P884" t="n">
-        <v>0.3072981303242432</v>
+        <v>0.3726888091343787</v>
       </c>
       <c r="Q884" t="n">
-        <v>0.341076385911194</v>
+        <v>0.2965968995493874</v>
       </c>
       <c r="R884" t="n">
         <v>1</v>
       </c>
       <c r="S884" t="n">
-        <v>-0.1084004854433765</v>
+        <v>0.06847808756138679</v>
       </c>
       <c r="T884" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U884" t="n">
-        <v>-0.1084004854433765</v>
+        <v>0.06847808756138679</v>
       </c>
       <c r="V884" t="n">
-        <v>0.3516254837645627</v>
+        <v>0.3726888091343787</v>
       </c>
       <c r="W884" t="n">
-        <v>2.05</v>
+        <v>3.1</v>
       </c>
       <c r="X884" t="inlineStr">
         <is>
@@ -89280,7 +89314,7 @@
       </c>
       <c r="Y884" t="inlineStr"/>
       <c r="Z884" t="n">
-        <v>3.692067579527908</v>
+        <v>3.879606956279555</v>
       </c>
       <c r="AA884" t="inlineStr">
         <is>
@@ -89348,34 +89382,34 @@
         <v>0.0625</v>
       </c>
       <c r="N885" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O885" t="n">
-        <v>0.3676622950568733</v>
+        <v>0.3778980908054501</v>
       </c>
       <c r="P885" t="n">
-        <v>0.3973135188685425</v>
+        <v>0.3543407228534319</v>
       </c>
       <c r="Q885" t="n">
-        <v>0.2350241860745842</v>
+        <v>0.267761186341118</v>
       </c>
       <c r="R885" t="n">
         <v>1</v>
       </c>
       <c r="S885" t="n">
-        <v>0.103195871809719</v>
+        <v>-0.09269014448866753</v>
       </c>
       <c r="T885" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U885" t="n">
-        <v>0.103195871809719</v>
+        <v>-0.09269014448866753</v>
       </c>
       <c r="V885" t="n">
-        <v>0.3973135188685425</v>
+        <v>0.3778980908054501</v>
       </c>
       <c r="W885" t="n">
-        <v>3.2</v>
+        <v>2</v>
       </c>
       <c r="X885" t="inlineStr">
         <is>
@@ -89384,7 +89418,7 @@
       </c>
       <c r="Y885" t="inlineStr"/>
       <c r="Z885" t="n">
-        <v>4.171791948119696</v>
+        <v>0.04282507710468009</v>
       </c>
       <c r="AA885" t="inlineStr">
         <is>
@@ -89455,28 +89489,28 @@
         <v>1</v>
       </c>
       <c r="O886" t="n">
-        <v>0.3945970795434188</v>
+        <v>0.4013209601574705</v>
       </c>
       <c r="P886" t="n">
-        <v>0.3172220959455754</v>
+        <v>0.2598774083564577</v>
       </c>
       <c r="Q886" t="n">
-        <v>0.2881808245110059</v>
+        <v>0.3388016314860719</v>
       </c>
       <c r="R886" t="n">
         <v>1</v>
       </c>
       <c r="S886" t="n">
-        <v>-0.001342006750997493</v>
+        <v>0.005381873863054276</v>
       </c>
       <c r="T886" t="n">
         <v>1</v>
       </c>
       <c r="U886" t="n">
-        <v>-0.001342006750997493</v>
+        <v>0.005381873863054276</v>
       </c>
       <c r="V886" t="n">
-        <v>0.3945970795434188</v>
+        <v>0.4013209601574705</v>
       </c>
       <c r="W886" t="n">
         <v>2.38</v>
@@ -89488,7 +89522,7 @@
       </c>
       <c r="Y886" t="inlineStr"/>
       <c r="Z886" t="n">
-        <v>4.143269335205897</v>
+        <v>2.537090733658126</v>
       </c>
       <c r="AA886" t="inlineStr">
         <is>
@@ -89559,28 +89593,28 @@
         <v>1</v>
       </c>
       <c r="O887" t="n">
-        <v>0.5842246515351605</v>
+        <v>0.5455460042845643</v>
       </c>
       <c r="P887" t="n">
-        <v>0.3203849175883086</v>
+        <v>0.3746080706648516</v>
       </c>
       <c r="Q887" t="n">
-        <v>0.09539043087653085</v>
+        <v>0.07984592505058404</v>
       </c>
       <c r="R887" t="n">
         <v>1</v>
       </c>
       <c r="S887" t="n">
-        <v>-0.1187775815307563</v>
+        <v>-0.1574562287813525</v>
       </c>
       <c r="T887" t="n">
         <v>1</v>
       </c>
       <c r="U887" t="n">
-        <v>-0.1187775815307563</v>
+        <v>-0.1574562287813525</v>
       </c>
       <c r="V887" t="n">
-        <v>0.5842246515351605</v>
+        <v>0.5455460042845643</v>
       </c>
       <c r="W887" t="n">
         <v>1.33</v>
@@ -89592,7 +89626,7 @@
       </c>
       <c r="Y887" t="inlineStr"/>
       <c r="Z887" t="n">
-        <v>6.134358841119185</v>
+        <v>0</v>
       </c>
       <c r="AA887" t="inlineStr">
         <is>
@@ -89663,28 +89697,28 @@
         <v>2</v>
       </c>
       <c r="O888" t="n">
-        <v>0.2969859406689073</v>
+        <v>0.3555858522195074</v>
       </c>
       <c r="P888" t="n">
-        <v>0.3055737538779895</v>
+        <v>0.23299534899876</v>
       </c>
       <c r="Q888" t="n">
-        <v>0.3974403054531032</v>
+        <v>0.4114187987817326</v>
       </c>
       <c r="R888" t="n">
         <v>1</v>
       </c>
       <c r="S888" t="n">
-        <v>0.1900328980456958</v>
+        <v>0.2040113913743252</v>
       </c>
       <c r="T888" t="n">
         <v>2</v>
       </c>
       <c r="U888" t="n">
-        <v>0.1900328980456958</v>
+        <v>0.2040113913743252</v>
       </c>
       <c r="V888" t="n">
-        <v>0.3974403054531032</v>
+        <v>0.4114187987817326</v>
       </c>
       <c r="W888" t="n">
         <v>4.5</v>
@@ -89696,7 +89730,7 @@
       </c>
       <c r="Y888" t="inlineStr"/>
       <c r="Z888" t="n">
-        <v>4.173123207257583</v>
+        <v>7.364786185674201</v>
       </c>
       <c r="AA888" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Data. Actualizo predicciones de FRA tras cambio de modelo
</commit_message>
<xml_diff>
--- a/data/historial_predicciones.xlsx
+++ b/data/historial_predicciones.xlsx
@@ -90078,78 +90078,78 @@
     <row r="888">
       <c r="A888" s="1" t="inlineStr">
         <is>
-          <t>tbGlN85K</t>
+          <t>W8pavTQ9</t>
         </is>
       </c>
       <c r="B888" s="2" t="n">
-        <v>45662.45833333334</v>
+        <v>45662.58333333334</v>
       </c>
       <c r="C888" t="inlineStr">
         <is>
-          <t>lens</t>
+          <t>torino</t>
         </is>
       </c>
       <c r="D888" t="inlineStr">
         <is>
-          <t>toulouse</t>
+          <t>parma</t>
         </is>
       </c>
       <c r="E888" t="n">
-        <v>55</v>
+        <v>77</v>
       </c>
       <c r="F888" t="n">
-        <v>551</v>
+        <v>771</v>
       </c>
       <c r="G888" t="n">
-        <v>2</v>
+        <v>1.85</v>
       </c>
       <c r="H888" t="n">
         <v>3.4</v>
       </c>
       <c r="I888" t="n">
-        <v>3.9</v>
+        <v>4.5</v>
       </c>
       <c r="J888" t="n">
-        <v>0.4759511844938981</v>
+        <v>0.5114491057997661</v>
       </c>
       <c r="K888" t="n">
-        <v>0.2799712849964106</v>
+        <v>0.2782884840381081</v>
       </c>
       <c r="L888" t="n">
-        <v>0.2440775305096913</v>
+        <v>0.2102624101621261</v>
       </c>
       <c r="M888" t="n">
-        <v>0.05052790346907998</v>
+        <v>0.05688040982158604</v>
       </c>
       <c r="N888" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O888" t="n">
-        <v>0.4769298279658987</v>
+        <v>0.304252303632831</v>
       </c>
       <c r="P888" t="n">
-        <v>0.2324925683993477</v>
+        <v>0.3971532082454944</v>
       </c>
       <c r="Q888" t="n">
-        <v>0.2905776036347535</v>
+        <v>0.2985944881216747</v>
       </c>
       <c r="R888" t="n">
         <v>1</v>
       </c>
       <c r="S888" t="n">
-        <v>0.000978643472000662</v>
+        <v>0.1188647242073863</v>
       </c>
       <c r="T888" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U888" t="n">
-        <v>0.000978643472000662</v>
+        <v>0.1188647242073863</v>
       </c>
       <c r="V888" t="n">
-        <v>0.4769298279658987</v>
+        <v>0.3971532082454944</v>
       </c>
       <c r="W888" t="n">
-        <v>2</v>
+        <v>3.4</v>
       </c>
       <c r="X888" t="inlineStr">
         <is>
@@ -90158,21 +90158,19 @@
       </c>
       <c r="Y888" t="inlineStr"/>
       <c r="Z888" t="n">
-        <v>2.861578967795392</v>
+        <v>7.853508945675356</v>
       </c>
       <c r="AA888" t="inlineStr">
         <is>
-          <t>france</t>
+          <t>italy</t>
         </is>
       </c>
       <c r="AB888" t="inlineStr">
         <is>
-          <t>ligue 1</t>
-        </is>
-      </c>
-      <c r="AC888" t="n">
-        <v>1</v>
-      </c>
+          <t>serie a</t>
+        </is>
+      </c>
+      <c r="AC888" t="inlineStr"/>
       <c r="AD888" t="inlineStr"/>
       <c r="AE888" t="inlineStr"/>
       <c r="AF888" t="n">
@@ -90182,78 +90180,78 @@
     <row r="889">
       <c r="A889" s="1" t="inlineStr">
         <is>
-          <t>08npCrcJ</t>
+          <t>8za4Io4j</t>
         </is>
       </c>
       <c r="B889" s="2" t="n">
-        <v>45662.69791666666</v>
+        <v>45662.35416666666</v>
       </c>
       <c r="C889" t="inlineStr">
         <is>
-          <t>marseille</t>
+          <t>monza</t>
         </is>
       </c>
       <c r="D889" t="inlineStr">
         <is>
-          <t>le havre</t>
+          <t>cagliari</t>
         </is>
       </c>
       <c r="E889" t="n">
-        <v>55</v>
+        <v>77</v>
       </c>
       <c r="F889" t="n">
-        <v>551</v>
+        <v>771</v>
       </c>
       <c r="G889" t="n">
-        <v>1.29</v>
+        <v>2.45</v>
       </c>
       <c r="H889" t="n">
-        <v>5.5</v>
+        <v>3.2</v>
       </c>
       <c r="I889" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="J889" t="n">
-        <v>0.7333822254816987</v>
+        <v>0.3872529245663574</v>
       </c>
       <c r="K889" t="n">
-        <v>0.1720114674311621</v>
+        <v>0.2964905203711174</v>
       </c>
       <c r="L889" t="n">
-        <v>0.09460630708713914</v>
+        <v>0.3162565550625252</v>
       </c>
       <c r="M889" t="n">
-        <v>0.05701198026779419</v>
+        <v>0.05399659863945572</v>
       </c>
       <c r="N889" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O889" t="n">
-        <v>0.6629813954358335</v>
+        <v>0.3063200939873246</v>
       </c>
       <c r="P889" t="n">
-        <v>0.2204529161196031</v>
+        <v>0.2505557436547355</v>
       </c>
       <c r="Q889" t="n">
-        <v>0.1165656884445635</v>
+        <v>0.4431241623579399</v>
       </c>
       <c r="R889" t="n">
         <v>1</v>
       </c>
       <c r="S889" t="n">
-        <v>-0.07040083004586528</v>
+        <v>0.1268676072954147</v>
       </c>
       <c r="T889" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U889" t="n">
-        <v>-0.07040083004586528</v>
+        <v>0.1268676072954147</v>
       </c>
       <c r="V889" t="n">
-        <v>0.6629813954358335</v>
+        <v>0.4431241623579399</v>
       </c>
       <c r="W889" t="n">
-        <v>1.29</v>
+        <v>3</v>
       </c>
       <c r="X889" t="inlineStr">
         <is>
@@ -90262,21 +90260,19 @@
       </c>
       <c r="Y889" t="inlineStr"/>
       <c r="Z889" t="n">
-        <v>3.133078412064617</v>
+        <v>11.96435238366438</v>
       </c>
       <c r="AA889" t="inlineStr">
         <is>
-          <t>france</t>
+          <t>italy</t>
         </is>
       </c>
       <c r="AB889" t="inlineStr">
         <is>
-          <t>ligue 1</t>
-        </is>
-      </c>
-      <c r="AC889" t="n">
-        <v>1</v>
-      </c>
+          <t>serie a</t>
+        </is>
+      </c>
+      <c r="AC889" t="inlineStr"/>
       <c r="AD889" t="inlineStr"/>
       <c r="AE889" t="inlineStr"/>
       <c r="AF889" t="n">
@@ -90286,7 +90282,7 @@
     <row r="890">
       <c r="A890" s="1" t="inlineStr">
         <is>
-          <t>YeeTFQcf</t>
+          <t>O2NXN7tT</t>
         </is>
       </c>
       <c r="B890" s="2" t="n">
@@ -90294,70 +90290,70 @@
       </c>
       <c r="C890" t="inlineStr">
         <is>
-          <t>angers</t>
+          <t>lecce</t>
         </is>
       </c>
       <c r="D890" t="inlineStr">
         <is>
-          <t>brest</t>
+          <t>genoa</t>
         </is>
       </c>
       <c r="E890" t="n">
-        <v>55</v>
+        <v>77</v>
       </c>
       <c r="F890" t="n">
-        <v>551</v>
+        <v>771</v>
       </c>
       <c r="G890" t="n">
-        <v>3.2</v>
+        <v>2.7</v>
       </c>
       <c r="H890" t="n">
-        <v>3.3</v>
+        <v>3</v>
       </c>
       <c r="I890" t="n">
-        <v>2.3</v>
+        <v>2.8</v>
       </c>
       <c r="J890" t="n">
-        <v>0.297530380243042</v>
+        <v>0.3491271820448877</v>
       </c>
       <c r="K890" t="n">
-        <v>0.2885143081144649</v>
+        <v>0.314214463840399</v>
       </c>
       <c r="L890" t="n">
-        <v>0.4139553116424932</v>
+        <v>0.3366583541147132</v>
       </c>
       <c r="M890" t="n">
-        <v>0.05031291172595509</v>
+        <v>0.06084656084656093</v>
       </c>
       <c r="N890" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O890" t="n">
-        <v>0.1200878862899446</v>
+        <v>0.4131168831170533</v>
       </c>
       <c r="P890" t="n">
-        <v>0.4955092062473773</v>
+        <v>0.1724169448332383</v>
       </c>
       <c r="Q890" t="n">
-        <v>0.384402907462678</v>
+        <v>0.4144661720497084</v>
       </c>
       <c r="R890" t="n">
         <v>1</v>
       </c>
       <c r="S890" t="n">
-        <v>0.2069948981329123</v>
+        <v>0.07780781793499525</v>
       </c>
       <c r="T890" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="U890" t="n">
-        <v>0.2069948981329123</v>
+        <v>0.07780781793499525</v>
       </c>
       <c r="V890" t="n">
-        <v>0.4955092062473773</v>
+        <v>0.4144661720497084</v>
       </c>
       <c r="W890" t="n">
-        <v>3.3</v>
+        <v>2.8</v>
       </c>
       <c r="X890" t="inlineStr">
         <is>
@@ -90366,21 +90362,19 @@
       </c>
       <c r="Y890" t="inlineStr"/>
       <c r="Z890" t="n">
-        <v>0.9910184124947544</v>
+        <v>11.19058664534213</v>
       </c>
       <c r="AA890" t="inlineStr">
         <is>
-          <t>france</t>
+          <t>italy</t>
         </is>
       </c>
       <c r="AB890" t="inlineStr">
         <is>
-          <t>ligue 1</t>
-        </is>
-      </c>
-      <c r="AC890" t="n">
-        <v>1</v>
-      </c>
+          <t>serie a</t>
+        </is>
+      </c>
+      <c r="AC890" t="inlineStr"/>
       <c r="AD890" t="inlineStr"/>
       <c r="AE890" t="inlineStr"/>
       <c r="AF890" t="n">
@@ -90390,78 +90384,78 @@
     <row r="891">
       <c r="A891" s="1" t="inlineStr">
         <is>
-          <t>SEvWZokQ</t>
+          <t>zsijtkdc</t>
         </is>
       </c>
       <c r="B891" s="2" t="n">
-        <v>45662.45833333334</v>
+        <v>45662.69791666666</v>
       </c>
       <c r="C891" t="inlineStr">
         <is>
-          <t>strasbourg</t>
+          <t>as roma</t>
         </is>
       </c>
       <c r="D891" t="inlineStr">
         <is>
-          <t>auxerre</t>
+          <t>lazio</t>
         </is>
       </c>
       <c r="E891" t="n">
-        <v>55</v>
+        <v>77</v>
       </c>
       <c r="F891" t="n">
-        <v>551</v>
+        <v>771</v>
       </c>
       <c r="G891" t="n">
-        <v>1.8</v>
+        <v>2.55</v>
       </c>
       <c r="H891" t="n">
-        <v>3.7</v>
+        <v>3.2</v>
       </c>
       <c r="I891" t="n">
-        <v>4.33</v>
+        <v>2.9</v>
       </c>
       <c r="J891" t="n">
-        <v>0.5257095980311731</v>
+        <v>0.373666196899537</v>
       </c>
       <c r="K891" t="n">
-        <v>0.2557506152584085</v>
+        <v>0.2977652506543185</v>
       </c>
       <c r="L891" t="n">
-        <v>0.2185397867104184</v>
+        <v>0.3285685524461445</v>
       </c>
       <c r="M891" t="n">
-        <v>0.0567727080429159</v>
+        <v>0.04948444895199478</v>
       </c>
       <c r="N891" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O891" t="n">
-        <v>0.275785697041999</v>
+        <v>0.1545191849059467</v>
       </c>
       <c r="P891" t="n">
-        <v>0.6439883917662587</v>
+        <v>0.1732454630248158</v>
       </c>
       <c r="Q891" t="n">
-        <v>0.08022591119174238</v>
+        <v>0.6722353520692376</v>
       </c>
       <c r="R891" t="n">
         <v>1</v>
       </c>
       <c r="S891" t="n">
-        <v>0.3882377765078502</v>
+        <v>0.343666799623093</v>
       </c>
       <c r="T891" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="U891" t="n">
-        <v>0.3882377765078502</v>
+        <v>0.343666799623093</v>
       </c>
       <c r="V891" t="n">
-        <v>0.6439883917662587</v>
+        <v>0.6722353520692376</v>
       </c>
       <c r="W891" t="n">
-        <v>3.7</v>
+        <v>2.9</v>
       </c>
       <c r="X891" t="inlineStr">
         <is>
@@ -90470,21 +90464,19 @@
       </c>
       <c r="Y891" t="inlineStr"/>
       <c r="Z891" t="n">
-        <v>1.287976783532517</v>
+        <v>18.15035450586942</v>
       </c>
       <c r="AA891" t="inlineStr">
         <is>
-          <t>france</t>
+          <t>italy</t>
         </is>
       </c>
       <c r="AB891" t="inlineStr">
         <is>
-          <t>ligue 1</t>
-        </is>
-      </c>
-      <c r="AC891" t="n">
-        <v>1</v>
-      </c>
+          <t>serie a</t>
+        </is>
+      </c>
+      <c r="AC891" t="inlineStr"/>
       <c r="AD891" t="inlineStr"/>
       <c r="AE891" t="inlineStr"/>
       <c r="AF891" t="n">
@@ -90494,78 +90486,78 @@
     <row r="892">
       <c r="A892" s="1" t="inlineStr">
         <is>
-          <t>W8pavTQ9</t>
+          <t>tbGlN85K</t>
         </is>
       </c>
       <c r="B892" s="2" t="n">
-        <v>45662.58333333334</v>
+        <v>45662.45833333334</v>
       </c>
       <c r="C892" t="inlineStr">
         <is>
-          <t>torino</t>
+          <t>lens</t>
         </is>
       </c>
       <c r="D892" t="inlineStr">
         <is>
-          <t>parma</t>
+          <t>toulouse</t>
         </is>
       </c>
       <c r="E892" t="n">
-        <v>77</v>
+        <v>55</v>
       </c>
       <c r="F892" t="n">
-        <v>771</v>
+        <v>551</v>
       </c>
       <c r="G892" t="n">
-        <v>1.85</v>
+        <v>2</v>
       </c>
       <c r="H892" t="n">
         <v>3.4</v>
       </c>
       <c r="I892" t="n">
-        <v>4.5</v>
+        <v>3.8</v>
       </c>
       <c r="J892" t="n">
-        <v>0.5114491057997661</v>
+        <v>0.472913616398243</v>
       </c>
       <c r="K892" t="n">
-        <v>0.2782884840381081</v>
+        <v>0.2781844802342606</v>
       </c>
       <c r="L892" t="n">
-        <v>0.2102624101621261</v>
+        <v>0.2489019033674963</v>
       </c>
       <c r="M892" t="n">
-        <v>0.05688040982158604</v>
+        <v>0.05727554179566563</v>
       </c>
       <c r="N892" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O892" t="n">
-        <v>0.304252303632831</v>
+        <v>0.4586936255080014</v>
       </c>
       <c r="P892" t="n">
-        <v>0.3971532082454944</v>
+        <v>0.2838609311100302</v>
       </c>
       <c r="Q892" t="n">
-        <v>0.2985944881216747</v>
+        <v>0.2574454433819685</v>
       </c>
       <c r="R892" t="n">
         <v>1</v>
       </c>
       <c r="S892" t="n">
-        <v>0.1188647242073863</v>
+        <v>-0.01421999089024162</v>
       </c>
       <c r="T892" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U892" t="n">
-        <v>0.1188647242073863</v>
+        <v>-0.01421999089024162</v>
       </c>
       <c r="V892" t="n">
-        <v>0.3971532082454944</v>
+        <v>0.4586936255080014</v>
       </c>
       <c r="W892" t="n">
-        <v>3.4</v>
+        <v>2</v>
       </c>
       <c r="X892" t="inlineStr">
         <is>
@@ -90574,19 +90566,21 @@
       </c>
       <c r="Y892" t="inlineStr"/>
       <c r="Z892" t="n">
-        <v>7.853508945675356</v>
+        <v>2.752161753048008</v>
       </c>
       <c r="AA892" t="inlineStr">
         <is>
-          <t>italy</t>
+          <t>france</t>
         </is>
       </c>
       <c r="AB892" t="inlineStr">
         <is>
-          <t>serie a</t>
-        </is>
-      </c>
-      <c r="AC892" t="inlineStr"/>
+          <t>ligue 1</t>
+        </is>
+      </c>
+      <c r="AC892" t="n">
+        <v>0</v>
+      </c>
       <c r="AD892" t="inlineStr"/>
       <c r="AE892" t="inlineStr"/>
       <c r="AF892" t="n">
@@ -90596,78 +90590,78 @@
     <row r="893">
       <c r="A893" s="1" t="inlineStr">
         <is>
-          <t>8za4Io4j</t>
+          <t>SEvWZokQ</t>
         </is>
       </c>
       <c r="B893" s="2" t="n">
-        <v>45662.35416666666</v>
+        <v>45662.45833333334</v>
       </c>
       <c r="C893" t="inlineStr">
         <is>
-          <t>monza</t>
+          <t>strasbourg</t>
         </is>
       </c>
       <c r="D893" t="inlineStr">
         <is>
-          <t>cagliari</t>
+          <t>auxerre</t>
         </is>
       </c>
       <c r="E893" t="n">
-        <v>77</v>
+        <v>55</v>
       </c>
       <c r="F893" t="n">
-        <v>771</v>
+        <v>551</v>
       </c>
       <c r="G893" t="n">
-        <v>2.45</v>
+        <v>1.85</v>
       </c>
       <c r="H893" t="n">
-        <v>3.2</v>
+        <v>3.75</v>
       </c>
       <c r="I893" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J893" t="n">
-        <v>0.3872529245663574</v>
+        <v>0.5112910097997443</v>
       </c>
       <c r="K893" t="n">
-        <v>0.2964905203711174</v>
+        <v>0.2522368981678739</v>
       </c>
       <c r="L893" t="n">
-        <v>0.3162565550625252</v>
+        <v>0.2364720920323818</v>
       </c>
       <c r="M893" t="n">
-        <v>0.05399659863945572</v>
+        <v>0.05720720720720718</v>
       </c>
       <c r="N893" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O893" t="n">
-        <v>0.3063200939873246</v>
+        <v>0.1293008246636046</v>
       </c>
       <c r="P893" t="n">
-        <v>0.2505557436547355</v>
+        <v>0.7711925875036827</v>
       </c>
       <c r="Q893" t="n">
-        <v>0.4431241623579399</v>
+        <v>0.09950658783271266</v>
       </c>
       <c r="R893" t="n">
         <v>1</v>
       </c>
       <c r="S893" t="n">
-        <v>0.1268676072954147</v>
+        <v>0.5189556893358088</v>
       </c>
       <c r="T893" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="U893" t="n">
-        <v>0.1268676072954147</v>
+        <v>0.5189556893358088</v>
       </c>
       <c r="V893" t="n">
-        <v>0.4431241623579399</v>
+        <v>0.7711925875036827</v>
       </c>
       <c r="W893" t="n">
-        <v>3</v>
+        <v>3.75</v>
       </c>
       <c r="X893" t="inlineStr">
         <is>
@@ -90676,19 +90670,21 @@
       </c>
       <c r="Y893" t="inlineStr"/>
       <c r="Z893" t="n">
-        <v>11.96435238366438</v>
+        <v>1.927981468759207</v>
       </c>
       <c r="AA893" t="inlineStr">
         <is>
-          <t>italy</t>
+          <t>france</t>
         </is>
       </c>
       <c r="AB893" t="inlineStr">
         <is>
-          <t>serie a</t>
-        </is>
-      </c>
-      <c r="AC893" t="inlineStr"/>
+          <t>ligue 1</t>
+        </is>
+      </c>
+      <c r="AC893" t="n">
+        <v>0</v>
+      </c>
       <c r="AD893" t="inlineStr"/>
       <c r="AE893" t="inlineStr"/>
       <c r="AF893" t="n">
@@ -90698,7 +90694,7 @@
     <row r="894">
       <c r="A894" s="1" t="inlineStr">
         <is>
-          <t>O2NXN7tT</t>
+          <t>YeeTFQcf</t>
         </is>
       </c>
       <c r="B894" s="2" t="n">
@@ -90706,70 +90702,70 @@
       </c>
       <c r="C894" t="inlineStr">
         <is>
-          <t>lecce</t>
+          <t>angers</t>
         </is>
       </c>
       <c r="D894" t="inlineStr">
         <is>
-          <t>genoa</t>
+          <t>brest</t>
         </is>
       </c>
       <c r="E894" t="n">
-        <v>77</v>
+        <v>55</v>
       </c>
       <c r="F894" t="n">
-        <v>771</v>
+        <v>551</v>
       </c>
       <c r="G894" t="n">
-        <v>2.7</v>
+        <v>3.25</v>
       </c>
       <c r="H894" t="n">
-        <v>3</v>
+        <v>3.3</v>
       </c>
       <c r="I894" t="n">
-        <v>2.8</v>
+        <v>2.25</v>
       </c>
       <c r="J894" t="n">
-        <v>0.3491271820448877</v>
+        <v>0.2916053019145803</v>
       </c>
       <c r="K894" t="n">
-        <v>0.314214463840399</v>
+        <v>0.2871870397643594</v>
       </c>
       <c r="L894" t="n">
-        <v>0.3366583541147132</v>
+        <v>0.4212076583210604</v>
       </c>
       <c r="M894" t="n">
-        <v>0.06084656084656093</v>
+        <v>0.05516705516705511</v>
       </c>
       <c r="N894" t="n">
         <v>2</v>
       </c>
       <c r="O894" t="n">
-        <v>0.4131168831170533</v>
+        <v>0.04271635861533991</v>
       </c>
       <c r="P894" t="n">
-        <v>0.1724169448332383</v>
+        <v>0.2441563316132538</v>
       </c>
       <c r="Q894" t="n">
-        <v>0.4144661720497084</v>
+        <v>0.7131273097714064</v>
       </c>
       <c r="R894" t="n">
         <v>1</v>
       </c>
       <c r="S894" t="n">
-        <v>0.07780781793499525</v>
+        <v>0.291919651450346</v>
       </c>
       <c r="T894" t="n">
         <v>2</v>
       </c>
       <c r="U894" t="n">
-        <v>0.07780781793499525</v>
+        <v>0.291919651450346</v>
       </c>
       <c r="V894" t="n">
-        <v>0.4144661720497084</v>
+        <v>0.7131273097714064</v>
       </c>
       <c r="W894" t="n">
-        <v>2.8</v>
+        <v>2.25</v>
       </c>
       <c r="X894" t="inlineStr">
         <is>
@@ -90778,19 +90774,21 @@
       </c>
       <c r="Y894" t="inlineStr"/>
       <c r="Z894" t="n">
-        <v>11.19058664534213</v>
+        <v>0.7131273097714063</v>
       </c>
       <c r="AA894" t="inlineStr">
         <is>
-          <t>italy</t>
+          <t>france</t>
         </is>
       </c>
       <c r="AB894" t="inlineStr">
         <is>
-          <t>serie a</t>
-        </is>
-      </c>
-      <c r="AC894" t="inlineStr"/>
+          <t>ligue 1</t>
+        </is>
+      </c>
+      <c r="AC894" t="n">
+        <v>0</v>
+      </c>
       <c r="AD894" t="inlineStr"/>
       <c r="AE894" t="inlineStr"/>
       <c r="AF894" t="n">
@@ -90800,7 +90798,7 @@
     <row r="895">
       <c r="A895" s="1" t="inlineStr">
         <is>
-          <t>zsijtkdc</t>
+          <t>08npCrcJ</t>
         </is>
       </c>
       <c r="B895" s="2" t="n">
@@ -90808,70 +90806,70 @@
       </c>
       <c r="C895" t="inlineStr">
         <is>
-          <t>as roma</t>
+          <t>marseille</t>
         </is>
       </c>
       <c r="D895" t="inlineStr">
         <is>
-          <t>lazio</t>
+          <t>le havre</t>
         </is>
       </c>
       <c r="E895" t="n">
-        <v>77</v>
+        <v>55</v>
       </c>
       <c r="F895" t="n">
-        <v>771</v>
+        <v>551</v>
       </c>
       <c r="G895" t="n">
-        <v>2.55</v>
+        <v>1.3</v>
       </c>
       <c r="H895" t="n">
-        <v>3.2</v>
+        <v>5.5</v>
       </c>
       <c r="I895" t="n">
-        <v>2.9</v>
+        <v>9</v>
       </c>
       <c r="J895" t="n">
-        <v>0.373666196899537</v>
+        <v>0.7242136064374541</v>
       </c>
       <c r="K895" t="n">
-        <v>0.2977652506543185</v>
+        <v>0.1711777615215801</v>
       </c>
       <c r="L895" t="n">
-        <v>0.3285685524461445</v>
+        <v>0.1046086320409656</v>
       </c>
       <c r="M895" t="n">
-        <v>0.04948444895199478</v>
+        <v>0.0621600621600622</v>
       </c>
       <c r="N895" t="n">
         <v>2</v>
       </c>
       <c r="O895" t="n">
-        <v>0.1545191849059467</v>
+        <v>0.3439379241087773</v>
       </c>
       <c r="P895" t="n">
-        <v>0.1732454630248158</v>
+        <v>0.3009208031158272</v>
       </c>
       <c r="Q895" t="n">
-        <v>0.6722353520692376</v>
+        <v>0.3551412727753955</v>
       </c>
       <c r="R895" t="n">
         <v>1</v>
       </c>
       <c r="S895" t="n">
-        <v>0.343666799623093</v>
+        <v>0.2505326407344299</v>
       </c>
       <c r="T895" t="n">
         <v>2</v>
       </c>
       <c r="U895" t="n">
-        <v>0.343666799623093</v>
+        <v>0.2505326407344299</v>
       </c>
       <c r="V895" t="n">
-        <v>0.6722353520692376</v>
+        <v>0.3551412727753955</v>
       </c>
       <c r="W895" t="n">
-        <v>2.9</v>
+        <v>9</v>
       </c>
       <c r="X895" t="inlineStr">
         <is>
@@ -90880,19 +90878,21 @@
       </c>
       <c r="Y895" t="inlineStr"/>
       <c r="Z895" t="n">
-        <v>18.15035450586942</v>
+        <v>0.3551412727753955</v>
       </c>
       <c r="AA895" t="inlineStr">
         <is>
-          <t>italy</t>
+          <t>france</t>
         </is>
       </c>
       <c r="AB895" t="inlineStr">
         <is>
-          <t>serie a</t>
-        </is>
-      </c>
-      <c r="AC895" t="inlineStr"/>
+          <t>ligue 1</t>
+        </is>
+      </c>
+      <c r="AC895" t="n">
+        <v>0</v>
+      </c>
       <c r="AD895" t="inlineStr"/>
       <c r="AE895" t="inlineStr"/>
       <c r="AF895" t="n">

</xml_diff>

<commit_message>
Data. Actualizo predicciones de FRA tras cambiar modelo
</commit_message>
<xml_diff>
--- a/data/historial_predicciones.xlsx
+++ b/data/historial_predicciones.xlsx
@@ -90509,55 +90509,55 @@
         <v>551</v>
       </c>
       <c r="G892" t="n">
-        <v>2</v>
+        <v>1.95</v>
       </c>
       <c r="H892" t="n">
-        <v>3.4</v>
+        <v>3.5</v>
       </c>
       <c r="I892" t="n">
-        <v>3.8</v>
+        <v>3.9</v>
       </c>
       <c r="J892" t="n">
-        <v>0.472913616398243</v>
+        <v>0.4861111111111112</v>
       </c>
       <c r="K892" t="n">
-        <v>0.2781844802342606</v>
+        <v>0.2708333333333333</v>
       </c>
       <c r="L892" t="n">
-        <v>0.2489019033674963</v>
+        <v>0.2430555555555556</v>
       </c>
       <c r="M892" t="n">
-        <v>0.05727554179566563</v>
+        <v>0.05494505494505497</v>
       </c>
       <c r="N892" t="n">
         <v>1</v>
       </c>
       <c r="O892" t="n">
-        <v>0.4586936255080014</v>
+        <v>0.424971329995716</v>
       </c>
       <c r="P892" t="n">
-        <v>0.2838609311100302</v>
+        <v>0.3306280715026779</v>
       </c>
       <c r="Q892" t="n">
-        <v>0.2574454433819685</v>
+        <v>0.2444005985016061</v>
       </c>
       <c r="R892" t="n">
         <v>1</v>
       </c>
       <c r="S892" t="n">
-        <v>-0.01421999089024162</v>
+        <v>-0.0611397811153952</v>
       </c>
       <c r="T892" t="n">
         <v>1</v>
       </c>
       <c r="U892" t="n">
-        <v>-0.01421999089024162</v>
+        <v>-0.0611397811153952</v>
       </c>
       <c r="V892" t="n">
-        <v>0.4586936255080014</v>
+        <v>0.424971329995716</v>
       </c>
       <c r="W892" t="n">
-        <v>2</v>
+        <v>1.95</v>
       </c>
       <c r="X892" t="inlineStr">
         <is>
@@ -90566,7 +90566,7 @@
       </c>
       <c r="Y892" t="inlineStr"/>
       <c r="Z892" t="n">
-        <v>2.752161753048008</v>
+        <v>2.118842374354479</v>
       </c>
       <c r="AA892" t="inlineStr">
         <is>
@@ -90590,20 +90590,20 @@
     <row r="893">
       <c r="A893" s="1" t="inlineStr">
         <is>
-          <t>SEvWZokQ</t>
+          <t>08npCrcJ</t>
         </is>
       </c>
       <c r="B893" s="2" t="n">
-        <v>45662.45833333334</v>
+        <v>45662.69791666666</v>
       </c>
       <c r="C893" t="inlineStr">
         <is>
-          <t>strasbourg</t>
+          <t>marseille</t>
         </is>
       </c>
       <c r="D893" t="inlineStr">
         <is>
-          <t>auxerre</t>
+          <t>le havre</t>
         </is>
       </c>
       <c r="E893" t="n">
@@ -90613,55 +90613,55 @@
         <v>551</v>
       </c>
       <c r="G893" t="n">
-        <v>1.85</v>
+        <v>1.3</v>
       </c>
       <c r="H893" t="n">
-        <v>3.75</v>
+        <v>5.25</v>
       </c>
       <c r="I893" t="n">
-        <v>4</v>
+        <v>9.5</v>
       </c>
       <c r="J893" t="n">
-        <v>0.5112910097997443</v>
+        <v>0.7223026792179579</v>
       </c>
       <c r="K893" t="n">
-        <v>0.2522368981678739</v>
+        <v>0.1788559015206372</v>
       </c>
       <c r="L893" t="n">
-        <v>0.2364720920323818</v>
+        <v>0.09884141926140477</v>
       </c>
       <c r="M893" t="n">
-        <v>0.05720720720720718</v>
+        <v>0.06497011760169658</v>
       </c>
       <c r="N893" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O893" t="n">
-        <v>0.1293008246636046</v>
+        <v>0.4846098670520239</v>
       </c>
       <c r="P893" t="n">
-        <v>0.7711925875036827</v>
+        <v>0.3375420524097365</v>
       </c>
       <c r="Q893" t="n">
-        <v>0.09950658783271266</v>
+        <v>0.1778480805382394</v>
       </c>
       <c r="R893" t="n">
         <v>1</v>
       </c>
       <c r="S893" t="n">
-        <v>0.5189556893358088</v>
+        <v>-0.237692812165934</v>
       </c>
       <c r="T893" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U893" t="n">
-        <v>0.5189556893358088</v>
+        <v>-0.237692812165934</v>
       </c>
       <c r="V893" t="n">
-        <v>0.7711925875036827</v>
+        <v>0.4846098670520239</v>
       </c>
       <c r="W893" t="n">
-        <v>3.75</v>
+        <v>1.3</v>
       </c>
       <c r="X893" t="inlineStr">
         <is>
@@ -90670,7 +90670,7 @@
       </c>
       <c r="Y893" t="inlineStr"/>
       <c r="Z893" t="n">
-        <v>1.927981468759207</v>
+        <v>0.06456969904109189</v>
       </c>
       <c r="AA893" t="inlineStr">
         <is>
@@ -90694,7 +90694,7 @@
     <row r="894">
       <c r="A894" s="1" t="inlineStr">
         <is>
-          <t>YeeTFQcf</t>
+          <t>SEvWZokQ</t>
         </is>
       </c>
       <c r="B894" s="2" t="n">
@@ -90702,12 +90702,12 @@
       </c>
       <c r="C894" t="inlineStr">
         <is>
-          <t>angers</t>
+          <t>strasbourg</t>
         </is>
       </c>
       <c r="D894" t="inlineStr">
         <is>
-          <t>brest</t>
+          <t>auxerre</t>
         </is>
       </c>
       <c r="E894" t="n">
@@ -90717,55 +90717,53 @@
         <v>551</v>
       </c>
       <c r="G894" t="n">
-        <v>3.25</v>
+        <v>1.75</v>
       </c>
       <c r="H894" t="n">
-        <v>3.3</v>
+        <v>4</v>
       </c>
       <c r="I894" t="n">
-        <v>2.25</v>
+        <v>4.2</v>
       </c>
       <c r="J894" t="n">
-        <v>0.2916053019145803</v>
+        <v>0.5393258426966292</v>
       </c>
       <c r="K894" t="n">
-        <v>0.2871870397643594</v>
+        <v>0.2359550561797753</v>
       </c>
       <c r="L894" t="n">
-        <v>0.4212076583210604</v>
+        <v>0.2247191011235955</v>
       </c>
       <c r="M894" t="n">
-        <v>0.05516705516705511</v>
+        <v>0.05952380952380953</v>
       </c>
       <c r="N894" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O894" t="n">
-        <v>0.04271635861533991</v>
+        <v>0.2838230840588489</v>
       </c>
       <c r="P894" t="n">
-        <v>0.2441563316132538</v>
+        <v>0.3986106052400763</v>
       </c>
       <c r="Q894" t="n">
-        <v>0.7131273097714064</v>
-      </c>
-      <c r="R894" t="n">
-        <v>1</v>
-      </c>
+        <v>0.3175663107010748</v>
+      </c>
+      <c r="R894" t="inlineStr"/>
       <c r="S894" t="n">
-        <v>0.291919651450346</v>
+        <v>0.162655549060301</v>
       </c>
       <c r="T894" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="U894" t="n">
-        <v>0.291919651450346</v>
+        <v>0.162655549060301</v>
       </c>
       <c r="V894" t="n">
-        <v>0.7131273097714064</v>
+        <v>0.3986106052400763</v>
       </c>
       <c r="W894" t="n">
-        <v>2.25</v>
+        <v>4</v>
       </c>
       <c r="X894" t="inlineStr">
         <is>
@@ -90774,7 +90772,7 @@
       </c>
       <c r="Y894" t="inlineStr"/>
       <c r="Z894" t="n">
-        <v>0.7131273097714063</v>
+        <v>0.7972212104801526</v>
       </c>
       <c r="AA894" t="inlineStr">
         <is>
@@ -90798,20 +90796,20 @@
     <row r="895">
       <c r="A895" s="1" t="inlineStr">
         <is>
-          <t>08npCrcJ</t>
+          <t>YeeTFQcf</t>
         </is>
       </c>
       <c r="B895" s="2" t="n">
-        <v>45662.69791666666</v>
+        <v>45662.45833333334</v>
       </c>
       <c r="C895" t="inlineStr">
         <is>
-          <t>marseille</t>
+          <t>angers</t>
         </is>
       </c>
       <c r="D895" t="inlineStr">
         <is>
-          <t>le havre</t>
+          <t>brest</t>
         </is>
       </c>
       <c r="E895" t="n">
@@ -90821,55 +90819,53 @@
         <v>551</v>
       </c>
       <c r="G895" t="n">
-        <v>1.3</v>
+        <v>3.2</v>
       </c>
       <c r="H895" t="n">
-        <v>5.5</v>
+        <v>3.25</v>
       </c>
       <c r="I895" t="n">
-        <v>9</v>
+        <v>2.3</v>
       </c>
       <c r="J895" t="n">
-        <v>0.7242136064374541</v>
+        <v>0.296215573608084</v>
       </c>
       <c r="K895" t="n">
-        <v>0.1711777615215801</v>
+        <v>0.2916584109371904</v>
       </c>
       <c r="L895" t="n">
-        <v>0.1046086320409656</v>
+        <v>0.4121260154547257</v>
       </c>
       <c r="M895" t="n">
-        <v>0.0621600621600622</v>
+        <v>0.05497491638795982</v>
       </c>
       <c r="N895" t="n">
         <v>2</v>
       </c>
       <c r="O895" t="n">
-        <v>0.3439379241087773</v>
+        <v>0.2252560070728517</v>
       </c>
       <c r="P895" t="n">
-        <v>0.3009208031158272</v>
+        <v>0.2779351464144777</v>
       </c>
       <c r="Q895" t="n">
-        <v>0.3551412727753955</v>
-      </c>
-      <c r="R895" t="n">
-        <v>1</v>
-      </c>
+        <v>0.4968088465126706</v>
+      </c>
+      <c r="R895" t="inlineStr"/>
       <c r="S895" t="n">
-        <v>0.2505326407344299</v>
+        <v>0.08468283105794494</v>
       </c>
       <c r="T895" t="n">
         <v>2</v>
       </c>
       <c r="U895" t="n">
-        <v>0.2505326407344299</v>
+        <v>0.08468283105794494</v>
       </c>
       <c r="V895" t="n">
-        <v>0.3551412727753955</v>
+        <v>0.4968088465126706</v>
       </c>
       <c r="W895" t="n">
-        <v>9</v>
+        <v>2.3</v>
       </c>
       <c r="X895" t="inlineStr">
         <is>
@@ -90878,7 +90874,7 @@
       </c>
       <c r="Y895" t="inlineStr"/>
       <c r="Z895" t="n">
-        <v>0.3551412727753955</v>
+        <v>2.088850426861125</v>
       </c>
       <c r="AA895" t="inlineStr">
         <is>

</xml_diff>